<commit_message>
UnitTest UT03 found bug in method booking don't check time to book
</commit_message>
<xml_diff>
--- a/test/FIWDEE_UnitTest_Report.xlsx
+++ b/test/FIWDEE_UnitTest_Report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\ProjectPOS\FIWDEE-CP353002-69_1PrinciplesOfSoftwareDesign\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A77A409-D322-4564-9DD4-5D56775C6F14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CD43C00-C407-427A-B4F1-8D5E71DF4907}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9B0ECA1C-B255-4EEE-B7A8-035645CFC3D9}"/>
   </bookViews>
@@ -16,10 +16,11 @@
     <sheet name="Test Summary" sheetId="1" r:id="rId1"/>
     <sheet name="UT01_CreateBooking_EC" sheetId="2" r:id="rId2"/>
     <sheet name="UT02_CreateBooking_DT" sheetId="3" r:id="rId3"/>
-    <sheet name="Defect Summary" sheetId="4" r:id="rId4"/>
+    <sheet name="UT03_CreateBooking_Time_BVA" sheetId="5" r:id="rId4"/>
+    <sheet name="Defect Summary" sheetId="4" r:id="rId5"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId5"/>
+    <externalReference r:id="rId6"/>
   </externalReferences>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -67,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="454" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="601" uniqueCount="298">
   <si>
     <t>FIWDEE – Unit Test Design</t>
   </si>
@@ -733,6 +734,234 @@
   </si>
   <si>
     <t>Decision Table (Limited Entry)</t>
+  </si>
+  <si>
+    <t>lead (นาทีล่วงหน้า)</t>
+  </si>
+  <si>
+    <t>เวลาเริ่ม (บริการ 60 นาที)</t>
+  </si>
+  <si>
+    <t>min-</t>
+  </si>
+  <si>
+    <t>29</t>
+  </si>
+  <si>
+    <t>09:59</t>
+  </si>
+  <si>
+    <t>BookingServiceImpl.createBooking – ช่วงเวลาที่จองได้</t>
+  </si>
+  <si>
+    <t>min</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>10:00</t>
+  </si>
+  <si>
+    <t>Functional testing - Robustness Testing</t>
+  </si>
+  <si>
+    <t>min+</t>
+  </si>
+  <si>
+    <t>10:01</t>
+  </si>
+  <si>
+    <t>nom</t>
+  </si>
+  <si>
+    <t>10110</t>
+  </si>
+  <si>
+    <t>15:30</t>
+  </si>
+  <si>
+    <t>createBooking(...) – เงื่อนไขของ startDateTime</t>
+  </si>
+  <si>
+    <t>max-</t>
+  </si>
+  <si>
+    <t>20159</t>
+  </si>
+  <si>
+    <t>20:59</t>
+  </si>
+  <si>
+    <t>20160</t>
+  </si>
+  <si>
+    <t>21:00</t>
+  </si>
+  <si>
+    <t>BR-BKG-02 Operating Hours • BR-BKG-03 (ล่วงหน้า ≥ 30 นาที) • SRS 3.3 Step 2 (สูงสุด 14 วัน) • ดู Q2</t>
+  </si>
+  <si>
+    <t>max+</t>
+  </si>
+  <si>
+    <t>20161</t>
+  </si>
+  <si>
+    <t>21:01</t>
+  </si>
+  <si>
+    <t>lead (นาที)</t>
+  </si>
+  <si>
+    <t>เวลาเริ่ม</t>
+  </si>
+  <si>
+    <t>UT03-TC001</t>
+  </si>
+  <si>
+    <t>2026-11-09 15:30</t>
+  </si>
+  <si>
+    <t>สร้างสำเร็จ status = PENDING</t>
+  </si>
+  <si>
+    <t>UT03-TC002</t>
+  </si>
+  <si>
+    <t>2026-11-02 15:29</t>
+  </si>
+  <si>
+    <t>15:29</t>
+  </si>
+  <si>
+    <t>ValidationException ต้องจองล่วงหน้าอย่างน้อย 30 นาที</t>
+  </si>
+  <si>
+    <t>UT03-TC003</t>
+  </si>
+  <si>
+    <t>2026-11-02 15:30</t>
+  </si>
+  <si>
+    <t>สร้างสำเร็จ</t>
+  </si>
+  <si>
+    <t>UT03-TC004</t>
+  </si>
+  <si>
+    <t>2026-11-02 15:31</t>
+  </si>
+  <si>
+    <t>15:31</t>
+  </si>
+  <si>
+    <t>UT03-TC005</t>
+  </si>
+  <si>
+    <t>2026-11-16 14:59</t>
+  </si>
+  <si>
+    <t>14:59</t>
+  </si>
+  <si>
+    <t>UT03-TC006</t>
+  </si>
+  <si>
+    <t>2026-11-16 15:00</t>
+  </si>
+  <si>
+    <t>15:00</t>
+  </si>
+  <si>
+    <t>UT03-TC007</t>
+  </si>
+  <si>
+    <t>2026-11-16 15:01</t>
+  </si>
+  <si>
+    <t>15:01</t>
+  </si>
+  <si>
+    <t>ValidationException จองล่วงหน้าได้ไม่เกิน 14 วัน</t>
+  </si>
+  <si>
+    <t>UT03-TC008</t>
+  </si>
+  <si>
+    <t>2026-11-09 09:59</t>
+  </si>
+  <si>
+    <t>9779</t>
+  </si>
+  <si>
+    <t>ValidationException เริ่มก่อนร้านเปิด</t>
+  </si>
+  <si>
+    <t>UT03-TC009</t>
+  </si>
+  <si>
+    <t>2026-11-09 10:00</t>
+  </si>
+  <si>
+    <t>9780</t>
+  </si>
+  <si>
+    <t>UT03-TC010</t>
+  </si>
+  <si>
+    <t>2026-11-09 10:01</t>
+  </si>
+  <si>
+    <t>9781</t>
+  </si>
+  <si>
+    <t>UT03-TC011</t>
+  </si>
+  <si>
+    <t>2026-11-09 20:59</t>
+  </si>
+  <si>
+    <t>10439</t>
+  </si>
+  <si>
+    <t>UT03-TC012</t>
+  </si>
+  <si>
+    <t>2026-11-09 21:00</t>
+  </si>
+  <si>
+    <t>10440</t>
+  </si>
+  <si>
+    <t>สร้างสำเร็จ (จบ 22:00 พอดี)</t>
+  </si>
+  <si>
+    <t>UT03-TC013</t>
+  </si>
+  <si>
+    <t>2026-11-09 21:01</t>
+  </si>
+  <si>
+    <t>10441</t>
+  </si>
+  <si>
+    <t>ValidationException จบ 22:01 เกินเวลาปิดร้าน</t>
+  </si>
+  <si>
+    <t>UT03 – BookingServiceImpl.createBooking – ช่วงเวลาที่จองได้</t>
+  </si>
+  <si>
+    <t>Robustness Testing</t>
+  </si>
+  <si>
+    <t>DEF-002</t>
+  </si>
+  <si>
+    <t>createBooking ไม่ตรวจเวลา: จองย้อนหลัง, จองกระชั้นกว่า 30 นาที, เกิน 14 วัน, นอกเวลาทำการได้</t>
+  </si>
+  <si>
+    <t>service/impl/BookingServiceImpl.java startDateTime ≠ null • ผิด BR-BKG-02, BR-BKG-03 • UT03-TC002, TC007, TC008, TC013</t>
   </si>
 </sst>
 </file>
@@ -992,25 +1221,17 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1022,19 +1243,30 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1044,14 +1276,53 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="12">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1570,7 +1841,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{659A469D-55E7-4F16-B797-78C1D60B492C}">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="1" width="5.25" customWidth="1"/>
@@ -1582,14 +1853,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
@@ -1624,17 +1895,17 @@
       </c>
     </row>
     <row r="3" spans="1:9" ht="21">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="27"/>
-      <c r="C3" s="27"/>
-      <c r="D3" s="27"/>
-      <c r="E3" s="27"/>
-      <c r="F3" s="27"/>
-      <c r="G3" s="27"/>
-      <c r="H3" s="27"/>
-      <c r="I3" s="27"/>
+      <c r="B3" s="25"/>
+      <c r="C3" s="25"/>
+      <c r="D3" s="25"/>
+      <c r="E3" s="25"/>
+      <c r="F3" s="25"/>
+      <c r="G3" s="25"/>
+      <c r="H3" s="25"/>
+      <c r="I3" s="25"/>
     </row>
     <row r="4" spans="1:9" ht="42">
       <c r="A4" s="3">
@@ -1702,37 +1973,71 @@
         <v>215</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="21">
-      <c r="A6" s="25" t="s">
+    <row r="6" spans="1:9" ht="64.5" customHeight="1">
+      <c r="A6" s="3">
+        <v>3</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>293</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D6" s="3">
+        <f>COUNTA(UT03_CreateBooking_Time_BVA!$A$11:$A$23)</f>
         <v>13</v>
       </c>
-      <c r="B6" s="25"/>
-      <c r="C6" s="25"/>
-      <c r="D6" s="5" cm="1">
-        <f t="array" ref="D6">SUMPRODUCT(ISNUMBER(D4:D5)*D4:D5)</f>
+      <c r="E6" s="3">
+        <f>COUNTIF(UT03_CreateBooking_Time_BVA!$G$11:$G$23,"Pass")</f>
+        <v>9</v>
+      </c>
+      <c r="F6" s="3">
+        <f>COUNTIF(UT03_CreateBooking_Time_BVA!$G$11:$G$23,"Fail")</f>
+        <v>4</v>
+      </c>
+      <c r="G6" s="3">
+        <f>COUNTIF(UT03_CreateBooking_Time_BVA!$G$11:$G$23,"No run")</f>
+        <v>0</v>
+      </c>
+      <c r="H6" s="3">
+        <f>COUNTIF(UT03_CreateBooking_Time_BVA!$G$11:$G$23,"Block")</f>
+        <v>0</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="21">
+      <c r="A7" s="23" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="23"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="5" cm="1">
+        <f t="array" ref="D7">SUMPRODUCT(ISNUMBER(D4:D5)*D4:D5)</f>
         <v>25</v>
       </c>
-      <c r="E6" s="6" cm="1">
-        <f t="array" ref="E6">SUMPRODUCT(ISNUMBER(E4:E5)*E4:E5)</f>
-        <v>24</v>
-      </c>
-      <c r="F6" s="7" cm="1">
-        <f t="array" ref="F6">SUMPRODUCT(ISNUMBER(F4:F5)*F4:F5)</f>
-        <v>1</v>
-      </c>
-      <c r="G6" s="5" cm="1">
-        <f t="array" ref="G6">SUMPRODUCT(ISNUMBER(G4:G5)*G4:G5)</f>
+      <c r="E7" s="6" cm="1">
+        <f t="array" ref="E7">SUMPRODUCT(ISNUMBER(E4:E6)*E4:E6)</f>
+        <v>33</v>
+      </c>
+      <c r="F7" s="7" cm="1">
+        <f t="array" ref="F7">SUMPRODUCT(ISNUMBER(F4:F6)*F4:F6)</f>
+        <v>5</v>
+      </c>
+      <c r="G7" s="5" cm="1">
+        <f t="array" ref="G7">SUMPRODUCT(ISNUMBER(G4:G5)*G4:G5)</f>
         <v>0</v>
       </c>
-      <c r="H6" s="5" cm="1">
-        <f t="array" ref="H6">SUMPRODUCT(ISNUMBER(H4:H5)*H4:H5)</f>
+      <c r="H7" s="5" cm="1">
+        <f t="array" ref="H7">SUMPRODUCT(ISNUMBER(H4:H5)*H4:H5)</f>
         <v>0</v>
       </c>
-      <c r="I6" s="4"/>
+      <c r="I7" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A7:C7"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A3:I3"/>
   </mergeCells>
@@ -1754,265 +2059,265 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="24" thickBot="1">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
-      <c r="I1" s="22"/>
-      <c r="J1" s="22"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
     </row>
     <row r="2" spans="1:10" ht="24" thickBot="1">
       <c r="A2" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="23" t="s">
+      <c r="F2" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="23"/>
+      <c r="G2" s="27"/>
     </row>
     <row r="3" spans="1:10" ht="24" thickBot="1">
       <c r="A3" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="24" t="s">
+      <c r="B3" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
       <c r="F3" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="24" t="s">
+      <c r="G3" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="24"/>
-      <c r="I3" s="24"/>
-      <c r="J3" s="24"/>
+      <c r="H3" s="28"/>
+      <c r="I3" s="28"/>
+      <c r="J3" s="28"/>
     </row>
     <row r="4" spans="1:10" ht="24" thickBot="1">
       <c r="A4" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="20" t="s">
+      <c r="B4" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
       <c r="F4" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="G4" s="20" t="s">
+      <c r="G4" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="H4" s="20"/>
-      <c r="I4" s="20"/>
-      <c r="J4" s="20"/>
+      <c r="H4" s="29"/>
+      <c r="I4" s="29"/>
+      <c r="J4" s="29"/>
     </row>
     <row r="5" spans="1:10" ht="24" thickBot="1">
       <c r="A5" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="C5" s="20"/>
-      <c r="D5" s="20"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="29"/>
       <c r="F5" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="G5" s="20" t="s">
+      <c r="G5" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="H5" s="20"/>
-      <c r="I5" s="20"/>
-      <c r="J5" s="20"/>
+      <c r="H5" s="29"/>
+      <c r="I5" s="29"/>
+      <c r="J5" s="29"/>
     </row>
     <row r="6" spans="1:10" ht="24" thickBot="1">
       <c r="A6" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="20" t="s">
+      <c r="B6" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="20"/>
-      <c r="D6" s="20"/>
+      <c r="C6" s="29"/>
+      <c r="D6" s="29"/>
       <c r="F6" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="G6" s="20" t="s">
+      <c r="G6" s="29" t="s">
         <v>30</v>
       </c>
-      <c r="H6" s="20"/>
-      <c r="I6" s="20"/>
-      <c r="J6" s="20"/>
+      <c r="H6" s="29"/>
+      <c r="I6" s="29"/>
+      <c r="J6" s="29"/>
     </row>
     <row r="7" spans="1:10" ht="24" thickBot="1">
       <c r="A7" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="20" t="s">
+      <c r="B7" s="29" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="20"/>
-      <c r="D7" s="20"/>
+      <c r="C7" s="29"/>
+      <c r="D7" s="29"/>
       <c r="F7" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="G7" s="20" t="s">
+      <c r="G7" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="H7" s="20"/>
-      <c r="I7" s="20"/>
-      <c r="J7" s="20"/>
+      <c r="H7" s="29"/>
+      <c r="I7" s="29"/>
+      <c r="J7" s="29"/>
     </row>
     <row r="8" spans="1:10" ht="24" thickBot="1">
       <c r="A8" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="29" t="s">
         <v>36</v>
       </c>
-      <c r="C8" s="20"/>
-      <c r="D8" s="20"/>
+      <c r="C8" s="29"/>
+      <c r="D8" s="29"/>
       <c r="F8" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="G8" s="20" t="s">
+      <c r="G8" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="H8" s="20"/>
-      <c r="I8" s="20"/>
-      <c r="J8" s="20"/>
+      <c r="H8" s="29"/>
+      <c r="I8" s="29"/>
+      <c r="J8" s="29"/>
     </row>
     <row r="9" spans="1:10" ht="24" thickBot="1">
       <c r="A9" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="B9" s="20" t="s">
+      <c r="B9" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="C9" s="20"/>
-      <c r="D9" s="20"/>
+      <c r="C9" s="29"/>
+      <c r="D9" s="29"/>
       <c r="F9" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="G9" s="20" t="s">
+      <c r="G9" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="H9" s="20"/>
-      <c r="I9" s="20"/>
-      <c r="J9" s="20"/>
+      <c r="H9" s="29"/>
+      <c r="I9" s="29"/>
+      <c r="J9" s="29"/>
     </row>
     <row r="10" spans="1:10" ht="24" thickBot="1">
       <c r="F10" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="G10" s="20" t="s">
+      <c r="G10" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="H10" s="20"/>
-      <c r="I10" s="20"/>
-      <c r="J10" s="20"/>
+      <c r="H10" s="29"/>
+      <c r="I10" s="29"/>
+      <c r="J10" s="29"/>
     </row>
     <row r="11" spans="1:10" ht="24" thickBot="1">
       <c r="F11" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="G11" s="20" t="s">
+      <c r="G11" s="29" t="s">
         <v>46</v>
       </c>
-      <c r="H11" s="20"/>
-      <c r="I11" s="20"/>
-      <c r="J11" s="20"/>
+      <c r="H11" s="29"/>
+      <c r="I11" s="29"/>
+      <c r="J11" s="29"/>
     </row>
     <row r="12" spans="1:10" ht="24" thickBot="1">
       <c r="F12" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="G12" s="20" t="s">
+      <c r="G12" s="29" t="s">
         <v>48</v>
       </c>
-      <c r="H12" s="20"/>
-      <c r="I12" s="20"/>
-      <c r="J12" s="20"/>
+      <c r="H12" s="29"/>
+      <c r="I12" s="29"/>
+      <c r="J12" s="29"/>
     </row>
     <row r="13" spans="1:10" ht="24" thickBot="1">
       <c r="F13" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="G13" s="20" t="s">
+      <c r="G13" s="29" t="s">
         <v>50</v>
       </c>
-      <c r="H13" s="20"/>
-      <c r="I13" s="20"/>
-      <c r="J13" s="20"/>
+      <c r="H13" s="29"/>
+      <c r="I13" s="29"/>
+      <c r="J13" s="29"/>
     </row>
     <row r="14" spans="1:10" ht="24" thickBot="1">
       <c r="F14" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="G14" s="20" t="s">
+      <c r="G14" s="29" t="s">
         <v>52</v>
       </c>
-      <c r="H14" s="20"/>
-      <c r="I14" s="20"/>
-      <c r="J14" s="20"/>
+      <c r="H14" s="29"/>
+      <c r="I14" s="29"/>
+      <c r="J14" s="29"/>
     </row>
     <row r="15" spans="1:10" ht="24" thickBot="1">
       <c r="F15" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="G15" s="20" t="s">
+      <c r="G15" s="29" t="s">
         <v>54</v>
       </c>
-      <c r="H15" s="20"/>
-      <c r="I15" s="20"/>
-      <c r="J15" s="20"/>
+      <c r="H15" s="29"/>
+      <c r="I15" s="29"/>
+      <c r="J15" s="29"/>
     </row>
     <row r="16" spans="1:10" ht="24" thickBot="1">
       <c r="F16" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="G16" s="20" t="s">
+      <c r="G16" s="29" t="s">
         <v>56</v>
       </c>
-      <c r="H16" s="20"/>
-      <c r="I16" s="20"/>
-      <c r="J16" s="20"/>
+      <c r="H16" s="29"/>
+      <c r="I16" s="29"/>
+      <c r="J16" s="29"/>
     </row>
     <row r="18" spans="1:10">
-      <c r="A18" s="21" t="s">
+      <c r="A18" s="30" t="s">
         <v>57</v>
       </c>
-      <c r="B18" s="21"/>
-      <c r="C18" s="21"/>
-      <c r="D18" s="21"/>
-      <c r="E18" s="21"/>
-      <c r="F18" s="21"/>
-      <c r="G18" s="21"/>
-      <c r="H18" s="21"/>
-      <c r="I18" s="21"/>
-      <c r="J18" s="21"/>
+      <c r="B18" s="30"/>
+      <c r="C18" s="30"/>
+      <c r="D18" s="30"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="30"/>
+      <c r="G18" s="30"/>
+      <c r="H18" s="30"/>
+      <c r="I18" s="30"/>
+      <c r="J18" s="30"/>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="B20" s="18" t="s">
+      <c r="B20" s="32" t="s">
         <v>59</v>
       </c>
-      <c r="C20" s="18"/>
-      <c r="D20" s="18"/>
-      <c r="E20" s="18"/>
-      <c r="F20" s="18"/>
-      <c r="G20" s="18"/>
-      <c r="H20" s="18"/>
+      <c r="C20" s="32"/>
+      <c r="D20" s="32"/>
+      <c r="E20" s="32"/>
+      <c r="F20" s="32"/>
+      <c r="G20" s="32"/>
+      <c r="H20" s="32"/>
       <c r="I20" s="12" t="s">
         <v>60</v>
       </c>
@@ -2024,15 +2329,15 @@
       <c r="A21" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="B21" s="18" t="s">
+      <c r="B21" s="32" t="s">
         <v>62</v>
       </c>
-      <c r="C21" s="18"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="18"/>
-      <c r="F21" s="18"/>
-      <c r="G21" s="18"/>
-      <c r="H21" s="18"/>
+      <c r="C21" s="32"/>
+      <c r="D21" s="32"/>
+      <c r="E21" s="32"/>
+      <c r="F21" s="32"/>
+      <c r="G21" s="32"/>
+      <c r="H21" s="32"/>
       <c r="I21" s="12" t="s">
         <v>63</v>
       </c>
@@ -2044,15 +2349,15 @@
       <c r="A22" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="B22" s="18" t="s">
+      <c r="B22" s="32" t="s">
         <v>65</v>
       </c>
-      <c r="C22" s="18"/>
-      <c r="D22" s="18"/>
-      <c r="E22" s="18"/>
-      <c r="F22" s="18"/>
-      <c r="G22" s="18"/>
-      <c r="H22" s="18"/>
+      <c r="C22" s="32"/>
+      <c r="D22" s="32"/>
+      <c r="E22" s="32"/>
+      <c r="F22" s="32"/>
+      <c r="G22" s="32"/>
+      <c r="H22" s="32"/>
       <c r="I22" s="12" t="s">
         <v>66</v>
       </c>
@@ -2064,58 +2369,58 @@
       <c r="A23" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="B23" s="18" t="s">
+      <c r="B23" s="32" t="s">
         <v>69</v>
       </c>
-      <c r="C23" s="18"/>
-      <c r="D23" s="18"/>
-      <c r="E23" s="18"/>
-      <c r="F23" s="18"/>
-      <c r="G23" s="18"/>
-      <c r="H23" s="18"/>
-      <c r="I23" s="18"/>
-      <c r="J23" s="18"/>
+      <c r="C23" s="32"/>
+      <c r="D23" s="32"/>
+      <c r="E23" s="32"/>
+      <c r="F23" s="32"/>
+      <c r="G23" s="32"/>
+      <c r="H23" s="32"/>
+      <c r="I23" s="32"/>
+      <c r="J23" s="32"/>
     </row>
     <row r="24" spans="1:10" ht="46.5">
       <c r="A24" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="B24" s="18" t="s">
+      <c r="B24" s="32" t="s">
         <v>71</v>
       </c>
-      <c r="C24" s="18"/>
-      <c r="D24" s="18"/>
-      <c r="E24" s="18"/>
-      <c r="F24" s="18"/>
-      <c r="G24" s="18"/>
-      <c r="H24" s="18"/>
-      <c r="I24" s="18"/>
-      <c r="J24" s="18"/>
+      <c r="C24" s="32"/>
+      <c r="D24" s="32"/>
+      <c r="E24" s="32"/>
+      <c r="F24" s="32"/>
+      <c r="G24" s="32"/>
+      <c r="H24" s="32"/>
+      <c r="I24" s="32"/>
+      <c r="J24" s="32"/>
     </row>
     <row r="26" spans="1:10">
-      <c r="A26" s="19" t="s">
+      <c r="A26" s="31" t="s">
         <v>72</v>
       </c>
-      <c r="B26" s="19" t="s">
+      <c r="B26" s="31" t="s">
         <v>73</v>
       </c>
-      <c r="C26" s="19"/>
-      <c r="D26" s="19"/>
-      <c r="E26" s="19"/>
-      <c r="F26" s="19"/>
-      <c r="G26" s="19"/>
-      <c r="H26" s="19" t="s">
+      <c r="C26" s="31"/>
+      <c r="D26" s="31"/>
+      <c r="E26" s="31"/>
+      <c r="F26" s="31"/>
+      <c r="G26" s="31"/>
+      <c r="H26" s="31" t="s">
         <v>74</v>
       </c>
-      <c r="I26" s="19" t="s">
+      <c r="I26" s="31" t="s">
         <v>75</v>
       </c>
-      <c r="J26" s="19" t="s">
+      <c r="J26" s="31" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="46.5">
-      <c r="A27" s="19"/>
+      <c r="A27" s="31"/>
       <c r="B27" s="15" t="s">
         <v>77</v>
       </c>
@@ -2134,9 +2439,9 @@
       <c r="G27" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="H27" s="19"/>
-      <c r="I27" s="19"/>
-      <c r="J27" s="19"/>
+      <c r="H27" s="31"/>
+      <c r="I27" s="31"/>
+      <c r="J27" s="31"/>
     </row>
     <row r="28" spans="1:10" ht="162.75">
       <c r="A28" s="16" t="s">
@@ -2620,18 +2925,16 @@
     </row>
   </sheetData>
   <mergeCells count="34">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="G3:J3"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="G4:J4"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="G5:J5"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="G6:J6"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="G7:J7"/>
+    <mergeCell ref="B20:H20"/>
+    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="B22:H22"/>
+    <mergeCell ref="B23:J23"/>
+    <mergeCell ref="B24:J24"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="B26:G26"/>
+    <mergeCell ref="H26:H27"/>
+    <mergeCell ref="I26:I27"/>
+    <mergeCell ref="J26:J27"/>
     <mergeCell ref="A18:J18"/>
     <mergeCell ref="B8:D8"/>
     <mergeCell ref="G8:J8"/>
@@ -2644,25 +2947,27 @@
     <mergeCell ref="G14:J14"/>
     <mergeCell ref="G15:J15"/>
     <mergeCell ref="G16:J16"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="B26:G26"/>
-    <mergeCell ref="H26:H27"/>
-    <mergeCell ref="I26:I27"/>
-    <mergeCell ref="J26:J27"/>
-    <mergeCell ref="B20:H20"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="B22:H22"/>
-    <mergeCell ref="B23:J23"/>
-    <mergeCell ref="B24:J24"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="G5:J5"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="G6:J6"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="G7:J7"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="G3:J3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="G4:J4"/>
   </mergeCells>
   <conditionalFormatting sqref="J28:J42">
-    <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2691,31 +2996,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="29" t="s">
+      <c r="B1" s="19" t="s">
         <v>126</v>
       </c>
-      <c r="C1" s="29" t="s">
+      <c r="C1" s="19" t="s">
         <v>127</v>
       </c>
-      <c r="D1" s="29" t="s">
+      <c r="D1" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="E1" s="29" t="s">
+      <c r="E1" s="19" t="s">
         <v>129</v>
       </c>
-      <c r="F1" s="29" t="s">
+      <c r="F1" s="19" t="s">
         <v>130</v>
       </c>
-      <c r="G1" s="29" t="s">
+      <c r="G1" s="19" t="s">
         <v>131</v>
       </c>
-      <c r="H1" s="29" t="s">
+      <c r="H1" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="I1" s="29" t="s">
+      <c r="I1" s="19" t="s">
         <v>133</v>
       </c>
     </row>
@@ -2923,17 +3228,17 @@
       </c>
     </row>
     <row r="9" spans="1:9">
-      <c r="A9" s="28" t="s">
+      <c r="A9" s="18" t="s">
         <v>143</v>
       </c>
-      <c r="B9" s="30"/>
-      <c r="C9" s="30"/>
-      <c r="D9" s="30"/>
-      <c r="E9" s="30"/>
-      <c r="F9" s="30"/>
-      <c r="G9" s="30"/>
-      <c r="H9" s="30"/>
-      <c r="I9" s="30"/>
+      <c r="B9" s="20"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="20"/>
+      <c r="H9" s="20"/>
+      <c r="I9" s="20"/>
     </row>
     <row r="10" spans="1:9" ht="46.5">
       <c r="A10" s="13" t="s">
@@ -3043,43 +3348,43 @@
       <c r="I16" s="17"/>
     </row>
     <row r="17" spans="1:9">
-      <c r="A17" s="31" t="s">
+      <c r="A17" s="33" t="s">
         <v>152</v>
       </c>
-      <c r="B17" s="31"/>
-      <c r="C17" s="31"/>
-      <c r="D17" s="31"/>
-      <c r="E17" s="31"/>
-      <c r="F17" s="31"/>
-      <c r="G17" s="31"/>
-      <c r="H17" s="31"/>
-      <c r="I17" s="31"/>
+      <c r="B17" s="33"/>
+      <c r="C17" s="33"/>
+      <c r="D17" s="33"/>
+      <c r="E17" s="33"/>
+      <c r="F17" s="33"/>
+      <c r="G17" s="33"/>
+      <c r="H17" s="33"/>
+      <c r="I17" s="33"/>
     </row>
     <row r="19" spans="1:9">
-      <c r="A19" s="21" t="s">
+      <c r="A19" s="30" t="s">
         <v>57</v>
       </c>
-      <c r="B19" s="21"/>
-      <c r="C19" s="21"/>
-      <c r="D19" s="21"/>
-      <c r="E19" s="21"/>
-      <c r="F19" s="21"/>
-      <c r="G19" s="21"/>
-      <c r="H19" s="21"/>
-      <c r="I19" s="21"/>
+      <c r="B19" s="30"/>
+      <c r="C19" s="30"/>
+      <c r="D19" s="30"/>
+      <c r="E19" s="30"/>
+      <c r="F19" s="30"/>
+      <c r="G19" s="30"/>
+      <c r="H19" s="30"/>
+      <c r="I19" s="30"/>
     </row>
     <row r="21" spans="1:9" ht="46.5">
       <c r="A21" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="B21" s="18" t="s">
+      <c r="B21" s="32" t="s">
         <v>153</v>
       </c>
-      <c r="C21" s="18"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="18"/>
-      <c r="F21" s="18"/>
-      <c r="G21" s="32"/>
+      <c r="C21" s="32"/>
+      <c r="D21" s="32"/>
+      <c r="E21" s="32"/>
+      <c r="F21" s="32"/>
+      <c r="G21" s="21"/>
       <c r="H21" s="12" t="s">
         <v>60</v>
       </c>
@@ -3091,14 +3396,14 @@
       <c r="A22" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="B22" s="18" t="s">
+      <c r="B22" s="32" t="s">
         <v>155</v>
       </c>
-      <c r="C22" s="18"/>
-      <c r="D22" s="18"/>
-      <c r="E22" s="18"/>
-      <c r="F22" s="18"/>
-      <c r="G22" s="32"/>
+      <c r="C22" s="32"/>
+      <c r="D22" s="32"/>
+      <c r="E22" s="32"/>
+      <c r="F22" s="32"/>
+      <c r="G22" s="21"/>
       <c r="H22" s="12" t="s">
         <v>63</v>
       </c>
@@ -3106,18 +3411,18 @@
         <v>156</v>
       </c>
     </row>
-    <row r="23" spans="1:9">
+    <row r="23" spans="1:9" ht="49.5" customHeight="1">
       <c r="A23" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="B23" s="33" t="s">
+      <c r="B23" s="34" t="s">
         <v>65</v>
       </c>
-      <c r="C23" s="34"/>
-      <c r="D23" s="34"/>
-      <c r="E23" s="34"/>
-      <c r="F23" s="35"/>
-      <c r="G23" s="32"/>
+      <c r="C23" s="35"/>
+      <c r="D23" s="35"/>
+      <c r="E23" s="35"/>
+      <c r="F23" s="36"/>
+      <c r="G23" s="21"/>
       <c r="H23" s="12" t="s">
         <v>66</v>
       </c>
@@ -3129,57 +3434,57 @@
       <c r="A24" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="B24" s="18" t="s">
+      <c r="B24" s="32" t="s">
         <v>157</v>
       </c>
-      <c r="C24" s="18"/>
-      <c r="D24" s="18"/>
-      <c r="E24" s="18"/>
-      <c r="F24" s="18"/>
-      <c r="G24" s="18"/>
-      <c r="H24" s="18"/>
-      <c r="I24" s="18"/>
+      <c r="C24" s="32"/>
+      <c r="D24" s="32"/>
+      <c r="E24" s="32"/>
+      <c r="F24" s="32"/>
+      <c r="G24" s="32"/>
+      <c r="H24" s="32"/>
+      <c r="I24" s="32"/>
     </row>
     <row r="25" spans="1:9">
       <c r="A25" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="B25" s="18" t="s">
+      <c r="B25" s="32" t="s">
         <v>158</v>
       </c>
-      <c r="C25" s="18"/>
-      <c r="D25" s="18"/>
-      <c r="E25" s="18"/>
-      <c r="F25" s="18"/>
-      <c r="G25" s="18"/>
-      <c r="H25" s="18"/>
-      <c r="I25" s="18"/>
+      <c r="C25" s="32"/>
+      <c r="D25" s="32"/>
+      <c r="E25" s="32"/>
+      <c r="F25" s="32"/>
+      <c r="G25" s="32"/>
+      <c r="H25" s="32"/>
+      <c r="I25" s="32"/>
     </row>
     <row r="27" spans="1:9">
-      <c r="A27" s="19" t="s">
+      <c r="A27" s="31" t="s">
         <v>159</v>
       </c>
-      <c r="B27" s="19" t="s">
+      <c r="B27" s="31" t="s">
         <v>72</v>
       </c>
-      <c r="C27" s="19" t="s">
+      <c r="C27" s="31" t="s">
         <v>73</v>
       </c>
-      <c r="D27" s="19"/>
-      <c r="E27" s="19"/>
-      <c r="F27" s="19" t="s">
+      <c r="D27" s="31"/>
+      <c r="E27" s="31"/>
+      <c r="F27" s="31" t="s">
         <v>74</v>
       </c>
-      <c r="G27" s="19" t="s">
+      <c r="G27" s="31" t="s">
         <v>75</v>
       </c>
-      <c r="H27" s="19" t="s">
+      <c r="H27" s="31" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="28" spans="1:9" ht="46.5">
-      <c r="A28" s="19"/>
-      <c r="B28" s="19"/>
+      <c r="A28" s="31"/>
+      <c r="B28" s="31"/>
       <c r="C28" s="15" t="s">
         <v>81</v>
       </c>
@@ -3189,9 +3494,9 @@
       <c r="E28" s="15" t="s">
         <v>161</v>
       </c>
-      <c r="F28" s="19"/>
-      <c r="G28" s="19"/>
-      <c r="H28" s="19"/>
+      <c r="F28" s="31"/>
+      <c r="G28" s="31"/>
+      <c r="H28" s="31"/>
     </row>
     <row r="29" spans="1:9" ht="69.75">
       <c r="A29" s="17" t="s">
@@ -3455,6 +3760,12 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="B24:I24"/>
+    <mergeCell ref="A17:I17"/>
+    <mergeCell ref="A19:I19"/>
+    <mergeCell ref="B21:F21"/>
+    <mergeCell ref="B22:F22"/>
+    <mergeCell ref="B23:F23"/>
     <mergeCell ref="B25:I25"/>
     <mergeCell ref="A27:A28"/>
     <mergeCell ref="B27:B28"/>
@@ -3462,21 +3773,15 @@
     <mergeCell ref="F27:F28"/>
     <mergeCell ref="G27:G28"/>
     <mergeCell ref="H27:H28"/>
-    <mergeCell ref="A17:I17"/>
-    <mergeCell ref="A19:I19"/>
-    <mergeCell ref="B21:F21"/>
-    <mergeCell ref="B22:F22"/>
-    <mergeCell ref="B23:F23"/>
-    <mergeCell ref="B24:I24"/>
   </mergeCells>
   <conditionalFormatting sqref="H29:H38">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3491,8 +3796,543 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85650EA3-2DDD-4A0A-9B5D-3EC95B3F0ED3}">
+  <dimension ref="A1:L23"/>
+  <sheetFormatPr defaultColWidth="7.625" defaultRowHeight="23.25"/>
+  <cols>
+    <col min="1" max="1" width="19.25" style="8" customWidth="1"/>
+    <col min="2" max="4" width="14.875" style="8" customWidth="1"/>
+    <col min="5" max="5" width="35" style="8" customWidth="1"/>
+    <col min="6" max="6" width="15.75" style="8" customWidth="1"/>
+    <col min="7" max="7" width="14.875" style="8" customWidth="1"/>
+    <col min="8" max="9" width="7.625" style="8"/>
+    <col min="10" max="10" width="8.75" style="8" customWidth="1"/>
+    <col min="11" max="12" width="19.25" style="8" customWidth="1"/>
+    <col min="13" max="16384" width="7.625" style="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" ht="46.5">
+      <c r="A1" s="30" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="15" t="s">
+        <v>222</v>
+      </c>
+      <c r="L1" s="15" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="J2" s="17" t="s">
+        <v>224</v>
+      </c>
+      <c r="K2" s="17" t="s">
+        <v>225</v>
+      </c>
+      <c r="L2" s="17" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B3" s="32" t="s">
+        <v>227</v>
+      </c>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="G3" s="14" t="s">
+        <v>154</v>
+      </c>
+      <c r="J3" s="17" t="s">
+        <v>228</v>
+      </c>
+      <c r="K3" s="17" t="s">
+        <v>229</v>
+      </c>
+      <c r="L3" s="17" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" s="32" t="s">
+        <v>231</v>
+      </c>
+      <c r="C4" s="32"/>
+      <c r="D4" s="32"/>
+      <c r="E4" s="32"/>
+      <c r="F4" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="G4" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="J4" s="17" t="s">
+        <v>232</v>
+      </c>
+      <c r="K4" s="17" t="s">
+        <v>108</v>
+      </c>
+      <c r="L4" s="17" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="46.5">
+      <c r="A5" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B5" s="32" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" s="32"/>
+      <c r="D5" s="32"/>
+      <c r="E5" s="32"/>
+      <c r="F5" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="G5" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="J5" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="K5" s="17" t="s">
+        <v>235</v>
+      </c>
+      <c r="L5" s="17" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="46.5">
+      <c r="A6" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="B6" s="32" t="s">
+        <v>237</v>
+      </c>
+      <c r="C6" s="32"/>
+      <c r="D6" s="32"/>
+      <c r="E6" s="32"/>
+      <c r="F6" s="32"/>
+      <c r="G6" s="32"/>
+      <c r="J6" s="17" t="s">
+        <v>238</v>
+      </c>
+      <c r="K6" s="17" t="s">
+        <v>239</v>
+      </c>
+      <c r="L6" s="17" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="46.5">
+      <c r="A7" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B7" s="32" t="s">
+        <v>243</v>
+      </c>
+      <c r="C7" s="32"/>
+      <c r="D7" s="32"/>
+      <c r="E7" s="32"/>
+      <c r="F7" s="32"/>
+      <c r="G7" s="32"/>
+      <c r="J7" s="17" t="s">
+        <v>244</v>
+      </c>
+      <c r="K7" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="L7" s="17" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="A9" s="31" t="s">
+        <v>72</v>
+      </c>
+      <c r="B9" s="31" t="s">
+        <v>73</v>
+      </c>
+      <c r="C9" s="31"/>
+      <c r="D9" s="31"/>
+      <c r="E9" s="31" t="s">
+        <v>74</v>
+      </c>
+      <c r="F9" s="31" t="s">
+        <v>75</v>
+      </c>
+      <c r="G9" s="31" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="A10" s="31"/>
+      <c r="B10" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>247</v>
+      </c>
+      <c r="D10" s="15" t="s">
+        <v>248</v>
+      </c>
+      <c r="E10" s="31"/>
+      <c r="F10" s="31"/>
+      <c r="G10" s="31"/>
+    </row>
+    <row r="11" spans="1:12" ht="46.5">
+      <c r="A11" s="16" t="s">
+        <v>249</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>250</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>235</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>236</v>
+      </c>
+      <c r="E11" s="13" t="s">
+        <v>251</v>
+      </c>
+      <c r="F11" s="13" t="s">
+        <v>258</v>
+      </c>
+      <c r="G11" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="46.5">
+      <c r="A12" s="16" t="s">
+        <v>252</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>253</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>225</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>254</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>255</v>
+      </c>
+      <c r="F12" s="13" t="s">
+        <v>258</v>
+      </c>
+      <c r="G12" s="17" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="46.5">
+      <c r="A13" s="16" t="s">
+        <v>256</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>257</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>229</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>236</v>
+      </c>
+      <c r="E13" s="13" t="s">
+        <v>258</v>
+      </c>
+      <c r="F13" s="13" t="s">
+        <v>258</v>
+      </c>
+      <c r="G13" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="46.5">
+      <c r="A14" s="16" t="s">
+        <v>259</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>260</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="D14" s="13" t="s">
+        <v>261</v>
+      </c>
+      <c r="E14" s="13" t="s">
+        <v>258</v>
+      </c>
+      <c r="F14" s="13" t="s">
+        <v>258</v>
+      </c>
+      <c r="G14" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="46.5">
+      <c r="A15" s="16" t="s">
+        <v>262</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>263</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>239</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>264</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>258</v>
+      </c>
+      <c r="F15" s="13" t="s">
+        <v>258</v>
+      </c>
+      <c r="G15" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" ht="46.5">
+      <c r="A16" s="16" t="s">
+        <v>265</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>266</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>241</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>267</v>
+      </c>
+      <c r="E16" s="13" t="s">
+        <v>258</v>
+      </c>
+      <c r="F16" s="13" t="s">
+        <v>258</v>
+      </c>
+      <c r="G16" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="46.5">
+      <c r="A17" s="16" t="s">
+        <v>268</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>269</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>245</v>
+      </c>
+      <c r="D17" s="13" t="s">
+        <v>270</v>
+      </c>
+      <c r="E17" s="13" t="s">
+        <v>271</v>
+      </c>
+      <c r="F17" s="13" t="s">
+        <v>258</v>
+      </c>
+      <c r="G17" s="17" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="46.5">
+      <c r="A18" s="16" t="s">
+        <v>272</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>273</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>274</v>
+      </c>
+      <c r="D18" s="13" t="s">
+        <v>226</v>
+      </c>
+      <c r="E18" s="13" t="s">
+        <v>275</v>
+      </c>
+      <c r="F18" s="13" t="s">
+        <v>258</v>
+      </c>
+      <c r="G18" s="17" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="46.5">
+      <c r="A19" s="16" t="s">
+        <v>276</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>277</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>278</v>
+      </c>
+      <c r="D19" s="13" t="s">
+        <v>230</v>
+      </c>
+      <c r="E19" s="13" t="s">
+        <v>258</v>
+      </c>
+      <c r="F19" s="13" t="s">
+        <v>258</v>
+      </c>
+      <c r="G19" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="46.5">
+      <c r="A20" s="16" t="s">
+        <v>279</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>280</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>281</v>
+      </c>
+      <c r="D20" s="13" t="s">
+        <v>233</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>258</v>
+      </c>
+      <c r="F20" s="13" t="s">
+        <v>258</v>
+      </c>
+      <c r="G20" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="46.5">
+      <c r="A21" s="16" t="s">
+        <v>282</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>283</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>284</v>
+      </c>
+      <c r="D21" s="13" t="s">
+        <v>240</v>
+      </c>
+      <c r="E21" s="13" t="s">
+        <v>258</v>
+      </c>
+      <c r="F21" s="13" t="s">
+        <v>258</v>
+      </c>
+      <c r="G21" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="46.5">
+      <c r="A22" s="16" t="s">
+        <v>285</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>287</v>
+      </c>
+      <c r="D22" s="13" t="s">
+        <v>242</v>
+      </c>
+      <c r="E22" s="13" t="s">
+        <v>288</v>
+      </c>
+      <c r="F22" s="13" t="s">
+        <v>258</v>
+      </c>
+      <c r="G22" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="46.5">
+      <c r="A23" s="16" t="s">
+        <v>289</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>290</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>291</v>
+      </c>
+      <c r="D23" s="13" t="s">
+        <v>246</v>
+      </c>
+      <c r="E23" s="13" t="s">
+        <v>292</v>
+      </c>
+      <c r="F23" s="13" t="s">
+        <v>258</v>
+      </c>
+      <c r="G23" s="17" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="B7:G7"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="B6:G6"/>
+  </mergeCells>
+  <conditionalFormatting sqref="G11:G23">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+      <formula>"Pass"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+      <formula>"Fail"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
+      <formula>"Block"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" sqref="G11:G23" xr:uid="{866B5AC5-B25F-4B37-866D-E6C5E90C47BD}">
+      <formula1>"Pass,Fail,No run,Block"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93C8330E-079C-4579-8133-7533964AD0F3}">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr defaultColWidth="7.625" defaultRowHeight="23.25"/>
   <cols>
     <col min="1" max="1" width="5.25" style="8" customWidth="1"/>
@@ -3508,37 +4348,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="46.5">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="36" t="s">
+      <c r="B1" s="22" t="s">
         <v>205</v>
       </c>
-      <c r="C1" s="36" t="s">
+      <c r="C1" s="22" t="s">
         <v>206</v>
       </c>
-      <c r="D1" s="36" t="s">
+      <c r="D1" s="22" t="s">
         <v>207</v>
       </c>
-      <c r="E1" s="36" t="s">
+      <c r="E1" s="22" t="s">
         <v>208</v>
       </c>
-      <c r="F1" s="36" t="s">
+      <c r="F1" s="22" t="s">
         <v>209</v>
       </c>
-      <c r="G1" s="36" t="s">
+      <c r="G1" s="22" t="s">
         <v>210</v>
       </c>
-      <c r="H1" s="36" t="s">
+      <c r="H1" s="22" t="s">
         <v>211</v>
       </c>
-      <c r="I1" s="36" t="s">
+      <c r="I1" s="22" t="s">
         <v>212</v>
       </c>
-      <c r="J1" s="36" t="s">
+      <c r="J1" s="22" t="s">
         <v>213</v>
       </c>
-      <c r="K1" s="36" t="s">
+      <c r="K1" s="22" t="s">
         <v>214</v>
       </c>
     </row>
@@ -3571,6 +4411,37 @@
       <c r="J2" s="13"/>
       <c r="K2" s="13" t="s">
         <v>219</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="85.5" customHeight="1">
+      <c r="A3" s="17">
+        <v>2</v>
+      </c>
+      <c r="B3" s="17" t="s">
+        <v>295</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>296</v>
+      </c>
+      <c r="D3" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="E3" s="13"/>
+      <c r="F3" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="G3" s="17" t="s">
+        <v>216</v>
+      </c>
+      <c r="H3" s="17" t="s">
+        <v>217</v>
+      </c>
+      <c r="I3" s="17" t="s">
+        <v>217</v>
+      </c>
+      <c r="J3" s="13"/>
+      <c r="K3" s="13" t="s">
+        <v>297</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
UnitTest UT05 found bug in method booking Cancel and get money back method
</commit_message>
<xml_diff>
--- a/test/FIWDEE_UnitTest_Report.xlsx
+++ b/test/FIWDEE_UnitTest_Report.xlsx
@@ -8,19 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\ProjectPOS\FIWDEE-CP353002-69_1PrinciplesOfSoftwareDesign\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CD43C00-C407-427A-B4F1-8D5E71DF4907}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39F5FABA-9899-4CB5-88FC-DF6ACEA46236}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9B0ECA1C-B255-4EEE-B7A8-035645CFC3D9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="5" xr2:uid="{9B0ECA1C-B255-4EEE-B7A8-035645CFC3D9}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Summary" sheetId="1" r:id="rId1"/>
     <sheet name="UT01_CreateBooking_EC" sheetId="2" r:id="rId2"/>
     <sheet name="UT02_CreateBooking_DT" sheetId="3" r:id="rId3"/>
     <sheet name="UT03_CreateBooking_Time_BVA" sheetId="5" r:id="rId4"/>
-    <sheet name="Defect Summary" sheetId="4" r:id="rId5"/>
+    <sheet name="UT04_Overlap_Buffer_BVA" sheetId="6" r:id="rId5"/>
+    <sheet name="UT05_CancelBooking_DT" sheetId="7" r:id="rId6"/>
+    <sheet name="Defect Summary" sheetId="4" r:id="rId7"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId6"/>
+    <externalReference r:id="rId8"/>
   </externalReferences>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -68,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="601" uniqueCount="298">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1013" uniqueCount="455">
   <si>
     <t>FIWDEE – Unit Test Design</t>
   </si>
@@ -962,6 +964,477 @@
   </si>
   <si>
     <t>service/impl/BookingServiceImpl.java startDateTime ≠ null • ผิด BR-BKG-02, BR-BKG-03 • UT03-TC002, TC007, TC008, TC013</t>
+  </si>
+  <si>
+    <t>ห้อง: end เดิม→start ใหม่</t>
+  </si>
+  <si>
+    <t>ห้อง: end ใหม่→start เดิม</t>
+  </si>
+  <si>
+    <t>หมอนวด: end เดิม→start ใหม่</t>
+  </si>
+  <si>
+    <t>หมอนวด: end ใหม่→start เดิม</t>
+  </si>
+  <si>
+    <t>ขอบ-1</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>-1</t>
+  </si>
+  <si>
+    <t>BookingRepository.findConflictingRoomBookingsWithCleaningBuffer + createBooking – เวลาทับซ้อน</t>
+  </si>
+  <si>
+    <t>ขอบ</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>Functional testing - Robustness Testing (ขอบด้านเดียว)</t>
+  </si>
+  <si>
+    <t>ขอบ+1</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>120</t>
+  </si>
+  <si>
+    <t>default findConflictingRoomBookingsWithCleaningBuffer(roomId, start, end, 15, excluded) และ findConflictingTherapistBookings(...)</t>
+  </si>
+  <si>
+    <t>ทรัพยากร</t>
+  </si>
+  <si>
+    <t>start ใหม่</t>
+  </si>
+  <si>
+    <t>end ใหม่</t>
+  </si>
+  <si>
+    <t>ระยะห่าง (นาที)</t>
+  </si>
+  <si>
+    <t>UT04-TC001</t>
+  </si>
+  <si>
+    <t>R101 + T1</t>
+  </si>
+  <si>
+    <t>16:00</t>
+  </si>
+  <si>
+    <t>17:00</t>
+  </si>
+  <si>
+    <t>จองสำเร็จ (nom)</t>
+  </si>
+  <si>
+    <t>จองสำเร็จ</t>
+  </si>
+  <si>
+    <t>UT04-TC002</t>
+  </si>
+  <si>
+    <t>ห้อง R101</t>
+  </si>
+  <si>
+    <t>14:14</t>
+  </si>
+  <si>
+    <t>15:14</t>
+  </si>
+  <si>
+    <t>ConflictException ห้องไม่ว่าง (ยังอยู่ใน buffer)</t>
+  </si>
+  <si>
+    <t>UT04-TC003</t>
+  </si>
+  <si>
+    <t>14:15</t>
+  </si>
+  <si>
+    <t>15:15</t>
+  </si>
+  <si>
+    <t>UT04-TC004</t>
+  </si>
+  <si>
+    <t>14:16</t>
+  </si>
+  <si>
+    <t>15:16</t>
+  </si>
+  <si>
+    <t>UT04-TC005</t>
+  </si>
+  <si>
+    <t>11:46</t>
+  </si>
+  <si>
+    <t>12:46</t>
+  </si>
+  <si>
+    <t>ConflictException ห้องไม่ว่าง</t>
+  </si>
+  <si>
+    <t>UT04-TC006</t>
+  </si>
+  <si>
+    <t>11:45</t>
+  </si>
+  <si>
+    <t>12:45</t>
+  </si>
+  <si>
+    <t>UT04-TC007</t>
+  </si>
+  <si>
+    <t>11:44</t>
+  </si>
+  <si>
+    <t>12:44</t>
+  </si>
+  <si>
+    <t>UT04-TC008</t>
+  </si>
+  <si>
+    <t>หมอนวด T1</t>
+  </si>
+  <si>
+    <t>13:59</t>
+  </si>
+  <si>
+    <t>ConflictException หมอนวดไม่ว่าง</t>
+  </si>
+  <si>
+    <t>UT04-TC009</t>
+  </si>
+  <si>
+    <t>14:00</t>
+  </si>
+  <si>
+    <t>UT04-TC010</t>
+  </si>
+  <si>
+    <t>14:01</t>
+  </si>
+  <si>
+    <t>UT04-TC011</t>
+  </si>
+  <si>
+    <t>12:01</t>
+  </si>
+  <si>
+    <t>13:01</t>
+  </si>
+  <si>
+    <t>UT04-TC012</t>
+  </si>
+  <si>
+    <t>12:00</t>
+  </si>
+  <si>
+    <t>13:00</t>
+  </si>
+  <si>
+    <t>UT04-TC013</t>
+  </si>
+  <si>
+    <t>11:59</t>
+  </si>
+  <si>
+    <t>12:59</t>
+  </si>
+  <si>
+    <t>Equivalence class</t>
+  </si>
+  <si>
+    <t>EC1 (ผู้ใช้) = { null, CUSTOMER, STAFF (RECEPTIONIST/OWNER) }</t>
+  </si>
+  <si>
+    <t>EC2 (สถานะ) = { PC = PENDING/CONFIRMED, CI = CHECKED_IN, END = IN_SERVICE/COMPLETED/CANCELLED/NO_SHOW }</t>
+  </si>
+  <si>
+    <t>EC3 (เวลาก่อนเริ่ม) = { ≥ 2 ชม., &lt; 2 ชม. }</t>
+  </si>
+  <si>
+    <t>Rule#9</t>
+  </si>
+  <si>
+    <t>Rule#10</t>
+  </si>
+  <si>
+    <t>C1: currentUser</t>
+  </si>
+  <si>
+    <t>CUST</t>
+  </si>
+  <si>
+    <t>STAFF</t>
+  </si>
+  <si>
+    <t>C2: พบ booking</t>
+  </si>
+  <si>
+    <t>C3: เป็นเจ้าของ booking</t>
+  </si>
+  <si>
+    <t>C4: เวลาก่อนเริ่ม</t>
+  </si>
+  <si>
+    <t>&lt; 2</t>
+  </si>
+  <si>
+    <t>≥ 2</t>
+  </si>
+  <si>
+    <t>C5: สถานะ</t>
+  </si>
+  <si>
+    <t>PC</t>
+  </si>
+  <si>
+    <t>END</t>
+  </si>
+  <si>
+    <t>CI</t>
+  </si>
+  <si>
+    <t>C6: ชำระเงินแล้ว</t>
+  </si>
+  <si>
+    <t>A1: BusinessException 401</t>
+  </si>
+  <si>
+    <t>A2: NotFoundException</t>
+  </si>
+  <si>
+    <t>A3: BusinessException 403</t>
+  </si>
+  <si>
+    <t>A4: ValidationException ยกเลิกกระชั้นชิด</t>
+  </si>
+  <si>
+    <t>A5: ValidationException สถานะยกเลิกไม่ได้ (State)</t>
+  </si>
+  <si>
+    <t>A6: status = CANCELLED + บันทึกเหตุผลใน specialNotes</t>
+  </si>
+  <si>
+    <t>A7: ส่งคืนเงินเต็มจำนวน (RefundService)</t>
+  </si>
+  <si>
+    <t>R1 = null ทำงานก่อนค้นหา booking (โค้ดตรวจ currentUser ก่อน) • A5 มาจาก AbstractBookingState.throwInvalidTransition</t>
+  </si>
+  <si>
+    <t>BookingServiceImpl.cancelBooking – ยกเลิกการจอง</t>
+  </si>
+  <si>
+    <t>Functional testing - Decision Table (Extended Entry)</t>
+  </si>
+  <si>
+    <t>BookingResponseDTO cancelBooking(Long id, CancelBookingRequestDTO dto, User currentUser)</t>
+  </si>
+  <si>
+    <t>bookingId</t>
+  </si>
+  <si>
+    <t>สถานะ / start</t>
+  </si>
+  <si>
+    <t>dto.reason / Payment</t>
+  </si>
+  <si>
+    <t>UT05-TC001</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>CONFIRMED / 03/11 15:00</t>
+  </si>
+  <si>
+    <t>UT05-TC002</t>
+  </si>
+  <si>
+    <t>UT05-TC003</t>
+  </si>
+  <si>
+    <t>Customer#2</t>
+  </si>
+  <si>
+    <t>BusinessException 403 • สถานะคง CONFIRMED • save ไม่ถูกเรียก</t>
+  </si>
+  <si>
+    <t>BusinessException 403</t>
+  </si>
+  <si>
+    <t>UT05-TC004</t>
+  </si>
+  <si>
+    <t>CONFIRMED / 02/11 16:00 (1 ชม.)</t>
+  </si>
+  <si>
+    <t>ValidationException "...at least 2 hours..." • สถานะคงเดิม</t>
+  </si>
+  <si>
+    <t>UT05-TC005</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>PENDING / 03/11 15:00</t>
+  </si>
+  <si>
+    <t>reason = "ติดธุระ" / ไม่มี</t>
+  </si>
+  <si>
+    <t>status = CANCELLED • specialNotes ลงท้าย "[Cancelled by CUSTOMER: ติดธุระ]" • save 1 ครั้ง</t>
+  </si>
+  <si>
+    <t>CANCELLED</t>
+  </si>
+  <si>
+    <t>UT05-TC006</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>CONFIRMED / 03/11 15:00, notes เดิม "ปวดหลัง"</t>
+  </si>
+  <si>
+    <t>dto = null / ไม่มี</t>
+  </si>
+  <si>
+    <t>status = CANCELLED • specialNotes = "ปวดหลัง [Cancelled by CUSTOMER: Cancelled by user]"</t>
+  </si>
+  <si>
+    <t>UT05-TC007</t>
+  </si>
+  <si>
+    <t>− / COMPLETED 600.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">status = CANCELLED และส่งคืนเงิน 600.00 </t>
+  </si>
+  <si>
+    <t>COMPLETED</t>
+  </si>
+  <si>
+    <t>UT05-TC008</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>CANCELLED / 03/11 15:00</t>
+  </si>
+  <si>
+    <t>ValidationException "Cannot execute action 'cancel' from booking status CANCELLED"</t>
+  </si>
+  <si>
+    <t>UT05-TC009</t>
+  </si>
+  <si>
+    <t>status = CANCELLED (พนักงานไม่ติดกฎ 2 ชม.) • note "[Cancelled by RECEPTIONIST: ...]"</t>
+  </si>
+  <si>
+    <t>R9</t>
+  </si>
+  <si>
+    <t>UT05-TC010</t>
+  </si>
+  <si>
+    <t>Owner#60</t>
+  </si>
+  <si>
+    <t>CHECKED_IN / 02/11 15:20</t>
+  </si>
+  <si>
+    <t>status = CANCELLED (ยกเลิกฉุกเฉินหน้าร้าน)</t>
+  </si>
+  <si>
+    <t>R10</t>
+  </si>
+  <si>
+    <t>UT05-TC011</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>COMPLETED / 02/11 10:00</t>
+  </si>
+  <si>
+    <t>ValidationException • สถานะคง COMPLETED</t>
+  </si>
+  <si>
+    <t>UT05-TC012</t>
+  </si>
+  <si>
+    <t>IN_SERVICE / 02/11 14:30</t>
+  </si>
+  <si>
+    <t>ValidationException • สถานะคง IN_SERVICE</t>
+  </si>
+  <si>
+    <t>ยกเลิก booking ที่จ่ายเงินแล้วไม่ส่งเข้ากระบวนการคืนเงิน</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>service/impl/BookingServiceImpl.java cancelBooking (บรรทัด 270–300) • ผิด UC-10 A1 • UT05-TC007</t>
+  </si>
+  <si>
+    <t>cancelBooking / updateBookingStatus ไม่ publish BookingStatusChangedEvent</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>service/impl/BookingServiceImpl.java • Observer (NotificationListener, QueueListener) ไม่ทำงานเมื่อเปลี่ยนสถานะผ่าน 2 เมธอดนี้ • UT05-TC005</t>
+  </si>
+  <si>
+    <t>DEF-003</t>
+  </si>
+  <si>
+    <t>DEF-004</t>
+  </si>
+  <si>
+    <t>UC-10 (Main, A1, E1) • BR-BKG-04 • BR-SEC-01 • UC-5.1 • ดู Q3</t>
+  </si>
+  <si>
+    <t>BR-BKG-01 • BR-RES-03 • UC 6.1–6.2</t>
+  </si>
+  <si>
+    <t>UT04 – BookingRepository.findConflictingRoomBookingsWithCleaningBuffer + createBooking – เวลาทับซ้อน</t>
+  </si>
+  <si>
+    <t>Robustness Testing (ขอบด้านเดียว)</t>
+  </si>
+  <si>
+    <t>UT05 – BookingServiceImpl.cancelBooking – ยกเลิกการจอง</t>
+  </si>
+  <si>
+    <t>Decision Table (Extended Entry)</t>
+  </si>
+  <si>
+    <t>DEF-003, DEF-004</t>
   </si>
 </sst>
 </file>
@@ -1172,7 +1645,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1234,6 +1707,24 @@
     <xf numFmtId="0" fontId="5" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1255,18 +1746,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1280,7 +1759,28 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="15">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1386,8 +1886,8 @@
       <xxl21:relativeUrl r:id="rId3"/>
     </xxl21:alternateUrls>
     <sheetNames>
+      <sheetName val="Test Approach"/>
       <sheetName val="Test Summary"/>
-      <sheetName val="Test Approach"/>
       <sheetName val="Defect Summary"/>
       <sheetName val="UT01_CreateBooking_EC"/>
       <sheetName val="UT02_CreateBooking_DT"/>
@@ -1841,7 +2341,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{659A469D-55E7-4F16-B797-78C1D60B492C}">
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="1" width="5.25" customWidth="1"/>
@@ -1853,14 +2353,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
@@ -1895,17 +2395,17 @@
       </c>
     </row>
     <row r="3" spans="1:9" ht="21">
-      <c r="A3" s="25" t="s">
+      <c r="A3" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="25"/>
-      <c r="C3" s="25"/>
-      <c r="D3" s="25"/>
-      <c r="E3" s="25"/>
-      <c r="F3" s="25"/>
-      <c r="G3" s="25"/>
-      <c r="H3" s="25"/>
-      <c r="I3" s="25"/>
+      <c r="B3" s="31"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
     </row>
     <row r="4" spans="1:9" ht="42">
       <c r="A4" s="3">
@@ -2007,37 +2507,103 @@
         <v>295</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="21">
-      <c r="A7" s="23" t="s">
+    <row r="7" spans="1:9" ht="63">
+      <c r="A7" s="3">
+        <v>4</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>450</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>451</v>
+      </c>
+      <c r="D7" s="3">
+        <f>COUNTA(UT04_Overlap_Buffer_BVA!$A$11:$A$23)</f>
         <v>13</v>
       </c>
-      <c r="B7" s="23"/>
-      <c r="C7" s="23"/>
-      <c r="D7" s="5" cm="1">
-        <f t="array" ref="D7">SUMPRODUCT(ISNUMBER(D4:D5)*D4:D5)</f>
-        <v>25</v>
-      </c>
-      <c r="E7" s="6" cm="1">
-        <f t="array" ref="E7">SUMPRODUCT(ISNUMBER(E4:E6)*E4:E6)</f>
-        <v>33</v>
-      </c>
-      <c r="F7" s="7" cm="1">
-        <f t="array" ref="F7">SUMPRODUCT(ISNUMBER(F4:F6)*F4:F6)</f>
+      <c r="E7" s="3">
+        <f>COUNTIF(UT04_Overlap_Buffer_BVA!$H$11:$H$23,"Pass")</f>
+        <v>13</v>
+      </c>
+      <c r="F7" s="3">
+        <f>COUNTIF(UT04_Overlap_Buffer_BVA!$H$11:$H$23,"Fail")</f>
+        <v>0</v>
+      </c>
+      <c r="G7" s="3">
+        <f>COUNTIF(UT04_Overlap_Buffer_BVA!$H$11:$H$23,"No run")</f>
+        <v>0</v>
+      </c>
+      <c r="H7" s="3">
+        <f>COUNTIF(UT04_Overlap_Buffer_BVA!$H$11:$H$23,"Block")</f>
+        <v>0</v>
+      </c>
+      <c r="I7" s="4"/>
+    </row>
+    <row r="8" spans="1:9" ht="21">
+      <c r="A8" s="3">
         <v>5</v>
       </c>
-      <c r="G7" s="5" cm="1">
-        <f t="array" ref="G7">SUMPRODUCT(ISNUMBER(G4:G5)*G4:G5)</f>
+      <c r="B8" s="4" t="s">
+        <v>452</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>453</v>
+      </c>
+      <c r="D8" s="3">
+        <f>COUNTA(UT05_CancelBooking_DT!$B$34:$B$45)</f>
+        <v>12</v>
+      </c>
+      <c r="E8" s="3">
+        <f>COUNTIF(UT05_CancelBooking_DT!$I$34:$I$45,"Pass")</f>
+        <v>11</v>
+      </c>
+      <c r="F8" s="3">
+        <f>COUNTIF(UT05_CancelBooking_DT!$I$34:$I$45,"Fail")</f>
+        <v>1</v>
+      </c>
+      <c r="G8" s="3">
+        <f>COUNTIF(UT05_CancelBooking_DT!$I$34:$I$45,"No run")</f>
         <v>0</v>
       </c>
-      <c r="H7" s="5" cm="1">
-        <f t="array" ref="H7">SUMPRODUCT(ISNUMBER(H4:H5)*H4:H5)</f>
+      <c r="H8" s="3">
+        <f>COUNTIF(UT05_CancelBooking_DT!$I$34:$I$45,"Block")</f>
         <v>0</v>
       </c>
-      <c r="I7" s="4"/>
+      <c r="I8" s="4" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="21">
+      <c r="A9" s="29" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="29"/>
+      <c r="C9" s="29"/>
+      <c r="D9" s="5" cm="1">
+        <f t="array" ref="D9">SUMPRODUCT(ISNUMBER(D4:D8)*D4:D8)</f>
+        <v>63</v>
+      </c>
+      <c r="E9" s="6" cm="1">
+        <f t="array" ref="E9">SUMPRODUCT(ISNUMBER(E4:E8)*E4:E8)</f>
+        <v>57</v>
+      </c>
+      <c r="F9" s="7" cm="1">
+        <f t="array" ref="F9">SUMPRODUCT(ISNUMBER(F4:F8)*F4:F8)</f>
+        <v>6</v>
+      </c>
+      <c r="G9" s="5" cm="1">
+        <f t="array" ref="G9">SUMPRODUCT(ISNUMBER(G4:G8)*G4:G8)</f>
+        <v>0</v>
+      </c>
+      <c r="H9" s="5" cm="1">
+        <f t="array" ref="H9">SUMPRODUCT(ISNUMBER(H4:H8)*H4:H8)</f>
+        <v>0</v>
+      </c>
+      <c r="I9" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A9:C9"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A3:I3"/>
   </mergeCells>
@@ -2059,265 +2625,265 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="24" thickBot="1">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
-      <c r="J1" s="26"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
     </row>
     <row r="2" spans="1:10" ht="24" thickBot="1">
       <c r="A2" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="27" t="s">
+      <c r="F2" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="27"/>
+      <c r="G2" s="33"/>
     </row>
     <row r="3" spans="1:10" ht="24" thickBot="1">
       <c r="A3" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="28" t="s">
+      <c r="B3" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="28"/>
-      <c r="D3" s="28"/>
+      <c r="C3" s="34"/>
+      <c r="D3" s="34"/>
       <c r="F3" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="28" t="s">
+      <c r="G3" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="28"/>
-      <c r="I3" s="28"/>
-      <c r="J3" s="28"/>
+      <c r="H3" s="34"/>
+      <c r="I3" s="34"/>
+      <c r="J3" s="34"/>
     </row>
     <row r="4" spans="1:10" ht="24" thickBot="1">
       <c r="A4" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="29" t="s">
+      <c r="B4" s="35" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="29"/>
-      <c r="D4" s="29"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
       <c r="F4" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="G4" s="29" t="s">
+      <c r="G4" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="H4" s="29"/>
-      <c r="I4" s="29"/>
-      <c r="J4" s="29"/>
+      <c r="H4" s="35"/>
+      <c r="I4" s="35"/>
+      <c r="J4" s="35"/>
     </row>
     <row r="5" spans="1:10" ht="24" thickBot="1">
       <c r="A5" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="29" t="s">
+      <c r="B5" s="35" t="s">
         <v>24</v>
       </c>
-      <c r="C5" s="29"/>
-      <c r="D5" s="29"/>
+      <c r="C5" s="35"/>
+      <c r="D5" s="35"/>
       <c r="F5" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="G5" s="29" t="s">
+      <c r="G5" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="H5" s="29"/>
-      <c r="I5" s="29"/>
-      <c r="J5" s="29"/>
+      <c r="H5" s="35"/>
+      <c r="I5" s="35"/>
+      <c r="J5" s="35"/>
     </row>
     <row r="6" spans="1:10" ht="24" thickBot="1">
       <c r="A6" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="29" t="s">
+      <c r="B6" s="35" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="29"/>
-      <c r="D6" s="29"/>
+      <c r="C6" s="35"/>
+      <c r="D6" s="35"/>
       <c r="F6" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="G6" s="29" t="s">
+      <c r="G6" s="35" t="s">
         <v>30</v>
       </c>
-      <c r="H6" s="29"/>
-      <c r="I6" s="29"/>
-      <c r="J6" s="29"/>
+      <c r="H6" s="35"/>
+      <c r="I6" s="35"/>
+      <c r="J6" s="35"/>
     </row>
     <row r="7" spans="1:10" ht="24" thickBot="1">
       <c r="A7" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="29" t="s">
+      <c r="B7" s="35" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="29"/>
-      <c r="D7" s="29"/>
+      <c r="C7" s="35"/>
+      <c r="D7" s="35"/>
       <c r="F7" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="G7" s="29" t="s">
+      <c r="G7" s="35" t="s">
         <v>34</v>
       </c>
-      <c r="H7" s="29"/>
-      <c r="I7" s="29"/>
-      <c r="J7" s="29"/>
+      <c r="H7" s="35"/>
+      <c r="I7" s="35"/>
+      <c r="J7" s="35"/>
     </row>
     <row r="8" spans="1:10" ht="24" thickBot="1">
       <c r="A8" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="29" t="s">
+      <c r="B8" s="35" t="s">
         <v>36</v>
       </c>
-      <c r="C8" s="29"/>
-      <c r="D8" s="29"/>
+      <c r="C8" s="35"/>
+      <c r="D8" s="35"/>
       <c r="F8" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="G8" s="29" t="s">
+      <c r="G8" s="35" t="s">
         <v>38</v>
       </c>
-      <c r="H8" s="29"/>
-      <c r="I8" s="29"/>
-      <c r="J8" s="29"/>
+      <c r="H8" s="35"/>
+      <c r="I8" s="35"/>
+      <c r="J8" s="35"/>
     </row>
     <row r="9" spans="1:10" ht="24" thickBot="1">
       <c r="A9" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="B9" s="29" t="s">
+      <c r="B9" s="35" t="s">
         <v>40</v>
       </c>
-      <c r="C9" s="29"/>
-      <c r="D9" s="29"/>
+      <c r="C9" s="35"/>
+      <c r="D9" s="35"/>
       <c r="F9" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="G9" s="29" t="s">
+      <c r="G9" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="H9" s="29"/>
-      <c r="I9" s="29"/>
-      <c r="J9" s="29"/>
+      <c r="H9" s="35"/>
+      <c r="I9" s="35"/>
+      <c r="J9" s="35"/>
     </row>
     <row r="10" spans="1:10" ht="24" thickBot="1">
       <c r="F10" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="G10" s="29" t="s">
+      <c r="G10" s="35" t="s">
         <v>44</v>
       </c>
-      <c r="H10" s="29"/>
-      <c r="I10" s="29"/>
-      <c r="J10" s="29"/>
+      <c r="H10" s="35"/>
+      <c r="I10" s="35"/>
+      <c r="J10" s="35"/>
     </row>
     <row r="11" spans="1:10" ht="24" thickBot="1">
       <c r="F11" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="G11" s="29" t="s">
+      <c r="G11" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="H11" s="29"/>
-      <c r="I11" s="29"/>
-      <c r="J11" s="29"/>
+      <c r="H11" s="35"/>
+      <c r="I11" s="35"/>
+      <c r="J11" s="35"/>
     </row>
     <row r="12" spans="1:10" ht="24" thickBot="1">
       <c r="F12" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="G12" s="29" t="s">
+      <c r="G12" s="35" t="s">
         <v>48</v>
       </c>
-      <c r="H12" s="29"/>
-      <c r="I12" s="29"/>
-      <c r="J12" s="29"/>
+      <c r="H12" s="35"/>
+      <c r="I12" s="35"/>
+      <c r="J12" s="35"/>
     </row>
     <row r="13" spans="1:10" ht="24" thickBot="1">
       <c r="F13" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="G13" s="29" t="s">
+      <c r="G13" s="35" t="s">
         <v>50</v>
       </c>
-      <c r="H13" s="29"/>
-      <c r="I13" s="29"/>
-      <c r="J13" s="29"/>
+      <c r="H13" s="35"/>
+      <c r="I13" s="35"/>
+      <c r="J13" s="35"/>
     </row>
     <row r="14" spans="1:10" ht="24" thickBot="1">
       <c r="F14" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="G14" s="29" t="s">
+      <c r="G14" s="35" t="s">
         <v>52</v>
       </c>
-      <c r="H14" s="29"/>
-      <c r="I14" s="29"/>
-      <c r="J14" s="29"/>
+      <c r="H14" s="35"/>
+      <c r="I14" s="35"/>
+      <c r="J14" s="35"/>
     </row>
     <row r="15" spans="1:10" ht="24" thickBot="1">
       <c r="F15" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="G15" s="29" t="s">
+      <c r="G15" s="35" t="s">
         <v>54</v>
       </c>
-      <c r="H15" s="29"/>
-      <c r="I15" s="29"/>
-      <c r="J15" s="29"/>
+      <c r="H15" s="35"/>
+      <c r="I15" s="35"/>
+      <c r="J15" s="35"/>
     </row>
     <row r="16" spans="1:10" ht="24" thickBot="1">
       <c r="F16" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="G16" s="29" t="s">
+      <c r="G16" s="35" t="s">
         <v>56</v>
       </c>
-      <c r="H16" s="29"/>
-      <c r="I16" s="29"/>
-      <c r="J16" s="29"/>
+      <c r="H16" s="35"/>
+      <c r="I16" s="35"/>
+      <c r="J16" s="35"/>
     </row>
     <row r="18" spans="1:10">
-      <c r="A18" s="30" t="s">
+      <c r="A18" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="B18" s="30"/>
-      <c r="C18" s="30"/>
-      <c r="D18" s="30"/>
-      <c r="E18" s="30"/>
-      <c r="F18" s="30"/>
-      <c r="G18" s="30"/>
-      <c r="H18" s="30"/>
-      <c r="I18" s="30"/>
-      <c r="J18" s="30"/>
+      <c r="B18" s="28"/>
+      <c r="C18" s="28"/>
+      <c r="D18" s="28"/>
+      <c r="E18" s="28"/>
+      <c r="F18" s="28"/>
+      <c r="G18" s="28"/>
+      <c r="H18" s="28"/>
+      <c r="I18" s="28"/>
+      <c r="J18" s="28"/>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="B20" s="32" t="s">
+      <c r="B20" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="C20" s="32"/>
-      <c r="D20" s="32"/>
-      <c r="E20" s="32"/>
-      <c r="F20" s="32"/>
-      <c r="G20" s="32"/>
-      <c r="H20" s="32"/>
+      <c r="C20" s="24"/>
+      <c r="D20" s="24"/>
+      <c r="E20" s="24"/>
+      <c r="F20" s="24"/>
+      <c r="G20" s="24"/>
+      <c r="H20" s="24"/>
       <c r="I20" s="12" t="s">
         <v>60</v>
       </c>
@@ -2329,15 +2895,15 @@
       <c r="A21" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="B21" s="32" t="s">
+      <c r="B21" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="C21" s="32"/>
-      <c r="D21" s="32"/>
-      <c r="E21" s="32"/>
-      <c r="F21" s="32"/>
-      <c r="G21" s="32"/>
-      <c r="H21" s="32"/>
+      <c r="C21" s="24"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="24"/>
+      <c r="F21" s="24"/>
+      <c r="G21" s="24"/>
+      <c r="H21" s="24"/>
       <c r="I21" s="12" t="s">
         <v>63</v>
       </c>
@@ -2349,15 +2915,15 @@
       <c r="A22" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="B22" s="32" t="s">
+      <c r="B22" s="24" t="s">
         <v>65</v>
       </c>
-      <c r="C22" s="32"/>
-      <c r="D22" s="32"/>
-      <c r="E22" s="32"/>
-      <c r="F22" s="32"/>
-      <c r="G22" s="32"/>
-      <c r="H22" s="32"/>
+      <c r="C22" s="24"/>
+      <c r="D22" s="24"/>
+      <c r="E22" s="24"/>
+      <c r="F22" s="24"/>
+      <c r="G22" s="24"/>
+      <c r="H22" s="24"/>
       <c r="I22" s="12" t="s">
         <v>66</v>
       </c>
@@ -2369,58 +2935,58 @@
       <c r="A23" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="B23" s="32" t="s">
+      <c r="B23" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="C23" s="32"/>
-      <c r="D23" s="32"/>
-      <c r="E23" s="32"/>
-      <c r="F23" s="32"/>
-      <c r="G23" s="32"/>
-      <c r="H23" s="32"/>
-      <c r="I23" s="32"/>
-      <c r="J23" s="32"/>
+      <c r="C23" s="24"/>
+      <c r="D23" s="24"/>
+      <c r="E23" s="24"/>
+      <c r="F23" s="24"/>
+      <c r="G23" s="24"/>
+      <c r="H23" s="24"/>
+      <c r="I23" s="24"/>
+      <c r="J23" s="24"/>
     </row>
     <row r="24" spans="1:10" ht="46.5">
       <c r="A24" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="B24" s="32" t="s">
+      <c r="B24" s="24" t="s">
         <v>71</v>
       </c>
-      <c r="C24" s="32"/>
-      <c r="D24" s="32"/>
-      <c r="E24" s="32"/>
-      <c r="F24" s="32"/>
-      <c r="G24" s="32"/>
-      <c r="H24" s="32"/>
-      <c r="I24" s="32"/>
-      <c r="J24" s="32"/>
+      <c r="C24" s="24"/>
+      <c r="D24" s="24"/>
+      <c r="E24" s="24"/>
+      <c r="F24" s="24"/>
+      <c r="G24" s="24"/>
+      <c r="H24" s="24"/>
+      <c r="I24" s="24"/>
+      <c r="J24" s="24"/>
     </row>
     <row r="26" spans="1:10">
-      <c r="A26" s="31" t="s">
+      <c r="A26" s="25" t="s">
         <v>72</v>
       </c>
-      <c r="B26" s="31" t="s">
+      <c r="B26" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="C26" s="31"/>
-      <c r="D26" s="31"/>
-      <c r="E26" s="31"/>
-      <c r="F26" s="31"/>
-      <c r="G26" s="31"/>
-      <c r="H26" s="31" t="s">
+      <c r="C26" s="25"/>
+      <c r="D26" s="25"/>
+      <c r="E26" s="25"/>
+      <c r="F26" s="25"/>
+      <c r="G26" s="25"/>
+      <c r="H26" s="25" t="s">
         <v>74</v>
       </c>
-      <c r="I26" s="31" t="s">
+      <c r="I26" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="J26" s="31" t="s">
+      <c r="J26" s="25" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="46.5">
-      <c r="A27" s="31"/>
+      <c r="A27" s="25"/>
       <c r="B27" s="15" t="s">
         <v>77</v>
       </c>
@@ -2439,9 +3005,9 @@
       <c r="G27" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="H27" s="31"/>
-      <c r="I27" s="31"/>
-      <c r="J27" s="31"/>
+      <c r="H27" s="25"/>
+      <c r="I27" s="25"/>
+      <c r="J27" s="25"/>
     </row>
     <row r="28" spans="1:10" ht="162.75">
       <c r="A28" s="16" t="s">
@@ -2961,13 +3527,13 @@
     <mergeCell ref="G4:J4"/>
   </mergeCells>
   <conditionalFormatting sqref="J28:J42">
-    <cfRule type="cellIs" dxfId="11" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3348,42 +3914,42 @@
       <c r="I16" s="17"/>
     </row>
     <row r="17" spans="1:9">
-      <c r="A17" s="33" t="s">
+      <c r="A17" s="27" t="s">
         <v>152</v>
       </c>
-      <c r="B17" s="33"/>
-      <c r="C17" s="33"/>
-      <c r="D17" s="33"/>
-      <c r="E17" s="33"/>
-      <c r="F17" s="33"/>
-      <c r="G17" s="33"/>
-      <c r="H17" s="33"/>
-      <c r="I17" s="33"/>
+      <c r="B17" s="27"/>
+      <c r="C17" s="27"/>
+      <c r="D17" s="27"/>
+      <c r="E17" s="27"/>
+      <c r="F17" s="27"/>
+      <c r="G17" s="27"/>
+      <c r="H17" s="27"/>
+      <c r="I17" s="27"/>
     </row>
     <row r="19" spans="1:9">
-      <c r="A19" s="30" t="s">
+      <c r="A19" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="B19" s="30"/>
-      <c r="C19" s="30"/>
-      <c r="D19" s="30"/>
-      <c r="E19" s="30"/>
-      <c r="F19" s="30"/>
-      <c r="G19" s="30"/>
-      <c r="H19" s="30"/>
-      <c r="I19" s="30"/>
+      <c r="B19" s="28"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="28"/>
+      <c r="E19" s="28"/>
+      <c r="F19" s="28"/>
+      <c r="G19" s="28"/>
+      <c r="H19" s="28"/>
+      <c r="I19" s="28"/>
     </row>
     <row r="21" spans="1:9" ht="46.5">
       <c r="A21" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="B21" s="32" t="s">
+      <c r="B21" s="24" t="s">
         <v>153</v>
       </c>
-      <c r="C21" s="32"/>
-      <c r="D21" s="32"/>
-      <c r="E21" s="32"/>
-      <c r="F21" s="32"/>
+      <c r="C21" s="24"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="24"/>
+      <c r="F21" s="24"/>
       <c r="G21" s="21"/>
       <c r="H21" s="12" t="s">
         <v>60</v>
@@ -3396,13 +3962,13 @@
       <c r="A22" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="B22" s="32" t="s">
+      <c r="B22" s="24" t="s">
         <v>155</v>
       </c>
-      <c r="C22" s="32"/>
-      <c r="D22" s="32"/>
-      <c r="E22" s="32"/>
-      <c r="F22" s="32"/>
+      <c r="C22" s="24"/>
+      <c r="D22" s="24"/>
+      <c r="E22" s="24"/>
+      <c r="F22" s="24"/>
       <c r="G22" s="21"/>
       <c r="H22" s="12" t="s">
         <v>63</v>
@@ -3415,13 +3981,13 @@
       <c r="A23" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="B23" s="34" t="s">
+      <c r="B23" s="36" t="s">
         <v>65</v>
       </c>
-      <c r="C23" s="35"/>
-      <c r="D23" s="35"/>
-      <c r="E23" s="35"/>
-      <c r="F23" s="36"/>
+      <c r="C23" s="37"/>
+      <c r="D23" s="37"/>
+      <c r="E23" s="37"/>
+      <c r="F23" s="38"/>
       <c r="G23" s="21"/>
       <c r="H23" s="12" t="s">
         <v>66</v>
@@ -3434,57 +4000,57 @@
       <c r="A24" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="B24" s="32" t="s">
+      <c r="B24" s="24" t="s">
         <v>157</v>
       </c>
-      <c r="C24" s="32"/>
-      <c r="D24" s="32"/>
-      <c r="E24" s="32"/>
-      <c r="F24" s="32"/>
-      <c r="G24" s="32"/>
-      <c r="H24" s="32"/>
-      <c r="I24" s="32"/>
+      <c r="C24" s="24"/>
+      <c r="D24" s="24"/>
+      <c r="E24" s="24"/>
+      <c r="F24" s="24"/>
+      <c r="G24" s="24"/>
+      <c r="H24" s="24"/>
+      <c r="I24" s="24"/>
     </row>
     <row r="25" spans="1:9">
       <c r="A25" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="B25" s="32" t="s">
+      <c r="B25" s="24" t="s">
         <v>158</v>
       </c>
-      <c r="C25" s="32"/>
-      <c r="D25" s="32"/>
-      <c r="E25" s="32"/>
-      <c r="F25" s="32"/>
-      <c r="G25" s="32"/>
-      <c r="H25" s="32"/>
-      <c r="I25" s="32"/>
+      <c r="C25" s="24"/>
+      <c r="D25" s="24"/>
+      <c r="E25" s="24"/>
+      <c r="F25" s="24"/>
+      <c r="G25" s="24"/>
+      <c r="H25" s="24"/>
+      <c r="I25" s="24"/>
     </row>
     <row r="27" spans="1:9">
-      <c r="A27" s="31" t="s">
+      <c r="A27" s="25" t="s">
         <v>159</v>
       </c>
-      <c r="B27" s="31" t="s">
+      <c r="B27" s="25" t="s">
         <v>72</v>
       </c>
-      <c r="C27" s="31" t="s">
+      <c r="C27" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="D27" s="31"/>
-      <c r="E27" s="31"/>
-      <c r="F27" s="31" t="s">
+      <c r="D27" s="25"/>
+      <c r="E27" s="25"/>
+      <c r="F27" s="25" t="s">
         <v>74</v>
       </c>
-      <c r="G27" s="31" t="s">
+      <c r="G27" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="H27" s="31" t="s">
+      <c r="H27" s="25" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="28" spans="1:9" ht="46.5">
-      <c r="A28" s="31"/>
-      <c r="B28" s="31"/>
+      <c r="A28" s="25"/>
+      <c r="B28" s="25"/>
       <c r="C28" s="15" t="s">
         <v>81</v>
       </c>
@@ -3494,9 +4060,9 @@
       <c r="E28" s="15" t="s">
         <v>161</v>
       </c>
-      <c r="F28" s="31"/>
-      <c r="G28" s="31"/>
-      <c r="H28" s="31"/>
+      <c r="F28" s="25"/>
+      <c r="G28" s="25"/>
+      <c r="H28" s="25"/>
     </row>
     <row r="29" spans="1:9" ht="69.75">
       <c r="A29" s="17" t="s">
@@ -3775,13 +4341,13 @@
     <mergeCell ref="H27:H28"/>
   </mergeCells>
   <conditionalFormatting sqref="H29:H38">
-    <cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3812,15 +4378,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="46.5">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
       <c r="J1" s="13"/>
       <c r="K1" s="15" t="s">
         <v>222</v>
@@ -3844,12 +4410,12 @@
       <c r="A3" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="B3" s="32" t="s">
+      <c r="B3" s="24" t="s">
         <v>227</v>
       </c>
-      <c r="C3" s="32"/>
-      <c r="D3" s="32"/>
-      <c r="E3" s="32"/>
+      <c r="C3" s="24"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="24"/>
       <c r="F3" s="12" t="s">
         <v>60</v>
       </c>
@@ -3870,12 +4436,12 @@
       <c r="A4" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="B4" s="32" t="s">
+      <c r="B4" s="24" t="s">
         <v>231</v>
       </c>
-      <c r="C4" s="32"/>
-      <c r="D4" s="32"/>
-      <c r="E4" s="32"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
       <c r="F4" s="12" t="s">
         <v>63</v>
       </c>
@@ -3896,12 +4462,12 @@
       <c r="A5" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="B5" s="32" t="s">
+      <c r="B5" s="24" t="s">
         <v>65</v>
       </c>
-      <c r="C5" s="32"/>
-      <c r="D5" s="32"/>
-      <c r="E5" s="32"/>
+      <c r="C5" s="24"/>
+      <c r="D5" s="24"/>
+      <c r="E5" s="24"/>
       <c r="F5" s="12" t="s">
         <v>66</v>
       </c>
@@ -3922,14 +4488,14 @@
       <c r="A6" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="B6" s="32" t="s">
+      <c r="B6" s="24" t="s">
         <v>237</v>
       </c>
-      <c r="C6" s="32"/>
-      <c r="D6" s="32"/>
-      <c r="E6" s="32"/>
-      <c r="F6" s="32"/>
-      <c r="G6" s="32"/>
+      <c r="C6" s="24"/>
+      <c r="D6" s="24"/>
+      <c r="E6" s="24"/>
+      <c r="F6" s="24"/>
+      <c r="G6" s="24"/>
       <c r="J6" s="17" t="s">
         <v>238</v>
       </c>
@@ -3944,14 +4510,14 @@
       <c r="A7" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="B7" s="32" t="s">
+      <c r="B7" s="24" t="s">
         <v>243</v>
       </c>
-      <c r="C7" s="32"/>
-      <c r="D7" s="32"/>
-      <c r="E7" s="32"/>
-      <c r="F7" s="32"/>
-      <c r="G7" s="32"/>
+      <c r="C7" s="24"/>
+      <c r="D7" s="24"/>
+      <c r="E7" s="24"/>
+      <c r="F7" s="24"/>
+      <c r="G7" s="24"/>
       <c r="J7" s="17" t="s">
         <v>244</v>
       </c>
@@ -3963,26 +4529,26 @@
       </c>
     </row>
     <row r="9" spans="1:12">
-      <c r="A9" s="31" t="s">
+      <c r="A9" s="25" t="s">
         <v>72</v>
       </c>
-      <c r="B9" s="31" t="s">
+      <c r="B9" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="C9" s="31"/>
-      <c r="D9" s="31"/>
-      <c r="E9" s="31" t="s">
+      <c r="C9" s="25"/>
+      <c r="D9" s="25"/>
+      <c r="E9" s="25" t="s">
         <v>74</v>
       </c>
-      <c r="F9" s="31" t="s">
+      <c r="F9" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="G9" s="31" t="s">
+      <c r="G9" s="25" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="10" spans="1:12">
-      <c r="A10" s="31"/>
+      <c r="A10" s="25"/>
       <c r="B10" s="15" t="s">
         <v>82</v>
       </c>
@@ -3992,9 +4558,9 @@
       <c r="D10" s="15" t="s">
         <v>248</v>
       </c>
-      <c r="E10" s="31"/>
-      <c r="F10" s="31"/>
-      <c r="G10" s="31"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="25"/>
+      <c r="G10" s="25"/>
     </row>
     <row r="11" spans="1:12" ht="46.5">
       <c r="A11" s="16" t="s">
@@ -4310,13 +4876,13 @@
     <mergeCell ref="B6:G6"/>
   </mergeCells>
   <conditionalFormatting sqref="G11:G23">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4331,8 +4897,1629 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFEC2CCE-24BD-4103-9358-01382E6E8A1D}">
+  <dimension ref="A1:O23"/>
+  <sheetFormatPr defaultColWidth="7.625" defaultRowHeight="23.25"/>
+  <cols>
+    <col min="1" max="1" width="19.25" style="8" customWidth="1"/>
+    <col min="2" max="5" width="12.25" style="8" customWidth="1"/>
+    <col min="6" max="6" width="31.5" style="8" customWidth="1"/>
+    <col min="7" max="7" width="17" style="8" customWidth="1"/>
+    <col min="8" max="8" width="14.875" style="8" customWidth="1"/>
+    <col min="9" max="10" width="7.625" style="8"/>
+    <col min="11" max="11" width="8.75" style="8" customWidth="1"/>
+    <col min="12" max="15" width="15.75" style="8" customWidth="1"/>
+    <col min="16" max="16384" width="7.625" style="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" ht="69.75">
+      <c r="A1" s="28" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="15" t="s">
+        <v>298</v>
+      </c>
+      <c r="M1" s="15" t="s">
+        <v>299</v>
+      </c>
+      <c r="N1" s="15" t="s">
+        <v>300</v>
+      </c>
+      <c r="O1" s="15" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15">
+      <c r="K2" s="17" t="s">
+        <v>302</v>
+      </c>
+      <c r="L2" s="17" t="s">
+        <v>303</v>
+      </c>
+      <c r="M2" s="17" t="s">
+        <v>303</v>
+      </c>
+      <c r="N2" s="17" t="s">
+        <v>304</v>
+      </c>
+      <c r="O2" s="17" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15">
+      <c r="A3" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B3" s="24" t="s">
+        <v>305</v>
+      </c>
+      <c r="C3" s="24"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="24"/>
+      <c r="F3" s="24"/>
+      <c r="G3" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="H3" s="14" t="s">
+        <v>154</v>
+      </c>
+      <c r="K3" s="17" t="s">
+        <v>306</v>
+      </c>
+      <c r="L3" s="17" t="s">
+        <v>307</v>
+      </c>
+      <c r="M3" s="17" t="s">
+        <v>307</v>
+      </c>
+      <c r="N3" s="17" t="s">
+        <v>308</v>
+      </c>
+      <c r="O3" s="17" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15">
+      <c r="A4" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" s="24" t="s">
+        <v>309</v>
+      </c>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="H4" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="K4" s="17" t="s">
+        <v>310</v>
+      </c>
+      <c r="L4" s="17" t="s">
+        <v>311</v>
+      </c>
+      <c r="M4" s="17" t="s">
+        <v>311</v>
+      </c>
+      <c r="N4" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="O4" s="17" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" ht="46.5">
+      <c r="A5" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B5" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" s="24"/>
+      <c r="D5" s="24"/>
+      <c r="E5" s="24"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="H5" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="K5" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="L5" s="17" t="s">
+        <v>312</v>
+      </c>
+      <c r="M5" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="N5" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="O5" s="17" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" ht="46.5">
+      <c r="A6" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="B6" s="24" t="s">
+        <v>313</v>
+      </c>
+      <c r="C6" s="24"/>
+      <c r="D6" s="24"/>
+      <c r="E6" s="24"/>
+      <c r="F6" s="24"/>
+      <c r="G6" s="24"/>
+      <c r="H6" s="24"/>
+    </row>
+    <row r="7" spans="1:15" ht="46.5">
+      <c r="A7" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B7" s="24" t="s">
+        <v>449</v>
+      </c>
+      <c r="C7" s="24"/>
+      <c r="D7" s="24"/>
+      <c r="E7" s="24"/>
+      <c r="F7" s="24"/>
+      <c r="G7" s="24"/>
+      <c r="H7" s="24"/>
+    </row>
+    <row r="9" spans="1:15">
+      <c r="A9" s="25" t="s">
+        <v>72</v>
+      </c>
+      <c r="B9" s="25" t="s">
+        <v>73</v>
+      </c>
+      <c r="C9" s="25"/>
+      <c r="D9" s="25"/>
+      <c r="E9" s="25"/>
+      <c r="F9" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="G9" s="25" t="s">
+        <v>75</v>
+      </c>
+      <c r="H9" s="25" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" ht="46.5">
+      <c r="A10" s="25"/>
+      <c r="B10" s="15" t="s">
+        <v>314</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>315</v>
+      </c>
+      <c r="D10" s="15" t="s">
+        <v>316</v>
+      </c>
+      <c r="E10" s="15" t="s">
+        <v>317</v>
+      </c>
+      <c r="F10" s="25"/>
+      <c r="G10" s="25"/>
+      <c r="H10" s="25"/>
+    </row>
+    <row r="11" spans="1:15">
+      <c r="A11" s="16" t="s">
+        <v>318</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>319</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>320</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>321</v>
+      </c>
+      <c r="E11" s="13" t="s">
+        <v>312</v>
+      </c>
+      <c r="F11" s="13" t="s">
+        <v>322</v>
+      </c>
+      <c r="G11" s="13" t="s">
+        <v>323</v>
+      </c>
+      <c r="H11" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" ht="46.5">
+      <c r="A12" s="16" t="s">
+        <v>324</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>325</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>326</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>327</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>303</v>
+      </c>
+      <c r="F12" s="13" t="s">
+        <v>328</v>
+      </c>
+      <c r="G12" s="13" t="s">
+        <v>201</v>
+      </c>
+      <c r="H12" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15">
+      <c r="A13" s="16" t="s">
+        <v>329</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>325</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>330</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>331</v>
+      </c>
+      <c r="E13" s="13" t="s">
+        <v>307</v>
+      </c>
+      <c r="F13" s="13" t="s">
+        <v>323</v>
+      </c>
+      <c r="G13" s="13" t="s">
+        <v>323</v>
+      </c>
+      <c r="H13" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15">
+      <c r="A14" s="16" t="s">
+        <v>332</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>325</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>333</v>
+      </c>
+      <c r="D14" s="13" t="s">
+        <v>334</v>
+      </c>
+      <c r="E14" s="13" t="s">
+        <v>311</v>
+      </c>
+      <c r="F14" s="13" t="s">
+        <v>323</v>
+      </c>
+      <c r="G14" s="13" t="s">
+        <v>323</v>
+      </c>
+      <c r="H14" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" ht="46.5">
+      <c r="A15" s="16" t="s">
+        <v>335</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>325</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>336</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>337</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>303</v>
+      </c>
+      <c r="F15" s="13" t="s">
+        <v>338</v>
+      </c>
+      <c r="G15" s="13" t="s">
+        <v>201</v>
+      </c>
+      <c r="H15" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15">
+      <c r="A16" s="16" t="s">
+        <v>339</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>325</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>340</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>341</v>
+      </c>
+      <c r="E16" s="13" t="s">
+        <v>307</v>
+      </c>
+      <c r="F16" s="13" t="s">
+        <v>323</v>
+      </c>
+      <c r="G16" s="13" t="s">
+        <v>323</v>
+      </c>
+      <c r="H16" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8">
+      <c r="A17" s="16" t="s">
+        <v>342</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>325</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>343</v>
+      </c>
+      <c r="D17" s="13" t="s">
+        <v>344</v>
+      </c>
+      <c r="E17" s="13" t="s">
+        <v>311</v>
+      </c>
+      <c r="F17" s="13" t="s">
+        <v>323</v>
+      </c>
+      <c r="G17" s="13" t="s">
+        <v>323</v>
+      </c>
+      <c r="H17" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="46.5">
+      <c r="A18" s="16" t="s">
+        <v>345</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>346</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>347</v>
+      </c>
+      <c r="D18" s="13" t="s">
+        <v>264</v>
+      </c>
+      <c r="E18" s="13" t="s">
+        <v>304</v>
+      </c>
+      <c r="F18" s="13" t="s">
+        <v>348</v>
+      </c>
+      <c r="G18" s="13" t="s">
+        <v>201</v>
+      </c>
+      <c r="H18" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8">
+      <c r="A19" s="16" t="s">
+        <v>349</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>346</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>350</v>
+      </c>
+      <c r="D19" s="13" t="s">
+        <v>267</v>
+      </c>
+      <c r="E19" s="13" t="s">
+        <v>308</v>
+      </c>
+      <c r="F19" s="13" t="s">
+        <v>323</v>
+      </c>
+      <c r="G19" s="13" t="s">
+        <v>323</v>
+      </c>
+      <c r="H19" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8">
+      <c r="A20" s="16" t="s">
+        <v>351</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>346</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>352</v>
+      </c>
+      <c r="D20" s="13" t="s">
+        <v>270</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="F20" s="13" t="s">
+        <v>323</v>
+      </c>
+      <c r="G20" s="13" t="s">
+        <v>323</v>
+      </c>
+      <c r="H20" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="46.5">
+      <c r="A21" s="16" t="s">
+        <v>353</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>346</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>354</v>
+      </c>
+      <c r="D21" s="13" t="s">
+        <v>355</v>
+      </c>
+      <c r="E21" s="13" t="s">
+        <v>304</v>
+      </c>
+      <c r="F21" s="13" t="s">
+        <v>348</v>
+      </c>
+      <c r="G21" s="13" t="s">
+        <v>201</v>
+      </c>
+      <c r="H21" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
+      <c r="A22" s="16" t="s">
+        <v>356</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>346</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>357</v>
+      </c>
+      <c r="D22" s="13" t="s">
+        <v>358</v>
+      </c>
+      <c r="E22" s="13" t="s">
+        <v>308</v>
+      </c>
+      <c r="F22" s="13" t="s">
+        <v>323</v>
+      </c>
+      <c r="G22" s="13" t="s">
+        <v>323</v>
+      </c>
+      <c r="H22" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
+      <c r="A23" s="16" t="s">
+        <v>359</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>346</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>360</v>
+      </c>
+      <c r="D23" s="13" t="s">
+        <v>361</v>
+      </c>
+      <c r="E23" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="F23" s="13" t="s">
+        <v>323</v>
+      </c>
+      <c r="G23" s="13" t="s">
+        <v>323</v>
+      </c>
+      <c r="H23" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="B7:H7"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B6:H6"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="H9:H10"/>
+  </mergeCells>
+  <conditionalFormatting sqref="H11:H23">
+    <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
+      <formula>"Pass"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
+      <formula>"Fail"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
+      <formula>"Block"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" sqref="H11:H23" xr:uid="{97BEFB05-6DEC-4720-9336-386699D99661}">
+      <formula1>"Pass,Fail,No run,Block"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB631D1B-CC58-4688-BF52-64335E77E312}">
+  <dimension ref="A1:K45"/>
+  <sheetFormatPr defaultColWidth="7.625" defaultRowHeight="23.25"/>
+  <cols>
+    <col min="1" max="1" width="29.75" style="8" customWidth="1"/>
+    <col min="2" max="2" width="14" style="8" customWidth="1"/>
+    <col min="3" max="6" width="14.875" style="8" customWidth="1"/>
+    <col min="7" max="7" width="38.5" style="8" customWidth="1"/>
+    <col min="8" max="8" width="15.75" style="8" customWidth="1"/>
+    <col min="9" max="9" width="14.875" style="8" customWidth="1"/>
+    <col min="10" max="10" width="8.75" style="8" customWidth="1"/>
+    <col min="11" max="11" width="14.5" style="8" customWidth="1"/>
+    <col min="12" max="16384" width="7.625" style="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11">
+      <c r="A1" s="23" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2" s="26" t="s">
+        <v>363</v>
+      </c>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
+      <c r="I2" s="26"/>
+      <c r="J2" s="26"/>
+      <c r="K2" s="26"/>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" s="26" t="s">
+        <v>364</v>
+      </c>
+      <c r="B3" s="26"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="26"/>
+      <c r="G3" s="26"/>
+      <c r="H3" s="26"/>
+      <c r="I3" s="26"/>
+      <c r="J3" s="26"/>
+      <c r="K3" s="26"/>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" s="26" t="s">
+        <v>365</v>
+      </c>
+      <c r="B4" s="26"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="26"/>
+      <c r="H4" s="26"/>
+      <c r="I4" s="26"/>
+      <c r="J4" s="26"/>
+      <c r="K4" s="26"/>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="19" t="s">
+        <v>126</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>127</v>
+      </c>
+      <c r="D6" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="E6" s="19" t="s">
+        <v>129</v>
+      </c>
+      <c r="F6" s="19" t="s">
+        <v>130</v>
+      </c>
+      <c r="G6" s="19" t="s">
+        <v>131</v>
+      </c>
+      <c r="H6" s="19" t="s">
+        <v>132</v>
+      </c>
+      <c r="I6" s="19" t="s">
+        <v>133</v>
+      </c>
+      <c r="J6" s="19" t="s">
+        <v>366</v>
+      </c>
+      <c r="K6" s="19" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7" s="13" t="s">
+        <v>368</v>
+      </c>
+      <c r="B7" s="17" t="s">
+        <v>93</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="D7" s="17" t="s">
+        <v>369</v>
+      </c>
+      <c r="E7" s="17" t="s">
+        <v>369</v>
+      </c>
+      <c r="F7" s="17" t="s">
+        <v>369</v>
+      </c>
+      <c r="G7" s="17" t="s">
+        <v>369</v>
+      </c>
+      <c r="H7" s="17" t="s">
+        <v>369</v>
+      </c>
+      <c r="I7" s="17" t="s">
+        <v>370</v>
+      </c>
+      <c r="J7" s="17" t="s">
+        <v>370</v>
+      </c>
+      <c r="K7" s="17" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8" s="13" t="s">
+        <v>371</v>
+      </c>
+      <c r="B8" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="C8" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="D8" s="17" t="s">
+        <v>135</v>
+      </c>
+      <c r="E8" s="17" t="s">
+        <v>135</v>
+      </c>
+      <c r="F8" s="17" t="s">
+        <v>135</v>
+      </c>
+      <c r="G8" s="17" t="s">
+        <v>135</v>
+      </c>
+      <c r="H8" s="17" t="s">
+        <v>135</v>
+      </c>
+      <c r="I8" s="17" t="s">
+        <v>135</v>
+      </c>
+      <c r="J8" s="17" t="s">
+        <v>135</v>
+      </c>
+      <c r="K8" s="17" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9" s="13" t="s">
+        <v>372</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="D9" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="E9" s="17" t="s">
+        <v>135</v>
+      </c>
+      <c r="F9" s="17" t="s">
+        <v>135</v>
+      </c>
+      <c r="G9" s="17" t="s">
+        <v>135</v>
+      </c>
+      <c r="H9" s="17" t="s">
+        <v>135</v>
+      </c>
+      <c r="I9" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="J9" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="K9" s="17" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
+      <c r="A10" s="13" t="s">
+        <v>373</v>
+      </c>
+      <c r="B10" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="C10" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="D10" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="E10" s="17" t="s">
+        <v>374</v>
+      </c>
+      <c r="F10" s="17" t="s">
+        <v>375</v>
+      </c>
+      <c r="G10" s="17" t="s">
+        <v>375</v>
+      </c>
+      <c r="H10" s="17" t="s">
+        <v>375</v>
+      </c>
+      <c r="I10" s="17" t="s">
+        <v>374</v>
+      </c>
+      <c r="J10" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="K10" s="17" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11">
+      <c r="A11" s="13" t="s">
+        <v>376</v>
+      </c>
+      <c r="B11" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="C11" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="D11" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="E11" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="F11" s="17" t="s">
+        <v>377</v>
+      </c>
+      <c r="G11" s="17" t="s">
+        <v>377</v>
+      </c>
+      <c r="H11" s="17" t="s">
+        <v>378</v>
+      </c>
+      <c r="I11" s="17" t="s">
+        <v>377</v>
+      </c>
+      <c r="J11" s="17" t="s">
+        <v>379</v>
+      </c>
+      <c r="K11" s="17" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11">
+      <c r="A12" s="13" t="s">
+        <v>380</v>
+      </c>
+      <c r="B12" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="C12" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="D12" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="E12" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="F12" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="G12" s="17" t="s">
+        <v>135</v>
+      </c>
+      <c r="H12" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="I12" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="J12" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="K12" s="17" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
+      <c r="A13" s="18" t="s">
+        <v>143</v>
+      </c>
+      <c r="B13" s="20"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="20"/>
+      <c r="G13" s="20"/>
+      <c r="H13" s="20"/>
+      <c r="I13" s="20"/>
+      <c r="J13" s="20"/>
+      <c r="K13" s="20"/>
+    </row>
+    <row r="14" spans="1:11">
+      <c r="A14" s="13" t="s">
+        <v>381</v>
+      </c>
+      <c r="B14" s="17" t="s">
+        <v>145</v>
+      </c>
+      <c r="C14" s="17"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="17"/>
+      <c r="G14" s="17"/>
+      <c r="H14" s="17"/>
+      <c r="I14" s="17"/>
+      <c r="J14" s="17"/>
+      <c r="K14" s="17"/>
+    </row>
+    <row r="15" spans="1:11">
+      <c r="A15" s="13" t="s">
+        <v>382</v>
+      </c>
+      <c r="B15" s="17"/>
+      <c r="C15" s="17" t="s">
+        <v>145</v>
+      </c>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="17"/>
+      <c r="H15" s="17"/>
+      <c r="I15" s="17"/>
+      <c r="J15" s="17"/>
+      <c r="K15" s="17"/>
+    </row>
+    <row r="16" spans="1:11">
+      <c r="A16" s="13" t="s">
+        <v>383</v>
+      </c>
+      <c r="B16" s="17"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="17" t="s">
+        <v>145</v>
+      </c>
+      <c r="E16" s="17"/>
+      <c r="F16" s="17"/>
+      <c r="G16" s="17"/>
+      <c r="H16" s="17"/>
+      <c r="I16" s="17"/>
+      <c r="J16" s="17"/>
+      <c r="K16" s="17"/>
+    </row>
+    <row r="17" spans="1:11" ht="46.5">
+      <c r="A17" s="13" t="s">
+        <v>384</v>
+      </c>
+      <c r="B17" s="17"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17" t="s">
+        <v>145</v>
+      </c>
+      <c r="F17" s="17"/>
+      <c r="G17" s="17"/>
+      <c r="H17" s="17"/>
+      <c r="I17" s="17"/>
+      <c r="J17" s="17"/>
+      <c r="K17" s="17"/>
+    </row>
+    <row r="18" spans="1:11" ht="46.5">
+      <c r="A18" s="13" t="s">
+        <v>385</v>
+      </c>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="17"/>
+      <c r="H18" s="17" t="s">
+        <v>145</v>
+      </c>
+      <c r="I18" s="17"/>
+      <c r="J18" s="17"/>
+      <c r="K18" s="17" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="46.5">
+      <c r="A19" s="13" t="s">
+        <v>386</v>
+      </c>
+      <c r="B19" s="17"/>
+      <c r="C19" s="17"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="17" t="s">
+        <v>145</v>
+      </c>
+      <c r="G19" s="17" t="s">
+        <v>145</v>
+      </c>
+      <c r="H19" s="17"/>
+      <c r="I19" s="17" t="s">
+        <v>145</v>
+      </c>
+      <c r="J19" s="17" t="s">
+        <v>145</v>
+      </c>
+      <c r="K19" s="17"/>
+    </row>
+    <row r="20" spans="1:11" ht="46.5">
+      <c r="A20" s="13" t="s">
+        <v>387</v>
+      </c>
+      <c r="B20" s="17"/>
+      <c r="C20" s="17"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="17"/>
+      <c r="F20" s="17"/>
+      <c r="G20" s="17" t="s">
+        <v>145</v>
+      </c>
+      <c r="H20" s="17"/>
+      <c r="I20" s="17"/>
+      <c r="J20" s="17"/>
+      <c r="K20" s="17"/>
+    </row>
+    <row r="21" spans="1:11">
+      <c r="A21" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="B21" s="17"/>
+      <c r="C21" s="17"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="17"/>
+      <c r="H21" s="17"/>
+      <c r="I21" s="17"/>
+      <c r="J21" s="17"/>
+      <c r="K21" s="17"/>
+    </row>
+    <row r="22" spans="1:11">
+      <c r="A22" s="27" t="s">
+        <v>388</v>
+      </c>
+      <c r="B22" s="27"/>
+      <c r="C22" s="27"/>
+      <c r="D22" s="27"/>
+      <c r="E22" s="27"/>
+      <c r="F22" s="27"/>
+      <c r="G22" s="27"/>
+      <c r="H22" s="27"/>
+      <c r="I22" s="27"/>
+      <c r="J22" s="27"/>
+      <c r="K22" s="27"/>
+    </row>
+    <row r="24" spans="1:11">
+      <c r="A24" s="28" t="s">
+        <v>57</v>
+      </c>
+      <c r="B24" s="28"/>
+      <c r="C24" s="28"/>
+      <c r="D24" s="28"/>
+      <c r="E24" s="28"/>
+      <c r="F24" s="28"/>
+      <c r="G24" s="28"/>
+      <c r="H24" s="28"/>
+      <c r="I24" s="28"/>
+      <c r="J24" s="28"/>
+      <c r="K24" s="28"/>
+    </row>
+    <row r="26" spans="1:11" ht="46.5">
+      <c r="A26" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B26" s="24" t="s">
+        <v>389</v>
+      </c>
+      <c r="C26" s="24"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="24"/>
+      <c r="F26" s="24"/>
+      <c r="G26" s="24"/>
+      <c r="H26" s="21"/>
+      <c r="I26" s="21"/>
+      <c r="J26" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="K26" s="14" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="46.5">
+      <c r="A27" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="B27" s="24" t="s">
+        <v>390</v>
+      </c>
+      <c r="C27" s="24"/>
+      <c r="D27" s="24"/>
+      <c r="E27" s="24"/>
+      <c r="F27" s="24"/>
+      <c r="G27" s="24"/>
+      <c r="H27" s="21"/>
+      <c r="I27" s="21"/>
+      <c r="J27" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="K27" s="14" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11">
+      <c r="A28" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B28" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="C28" s="24"/>
+      <c r="D28" s="24"/>
+      <c r="E28" s="24"/>
+      <c r="F28" s="24"/>
+      <c r="G28" s="24"/>
+      <c r="H28" s="21"/>
+      <c r="I28" s="21"/>
+      <c r="J28" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="K28" s="13" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11">
+      <c r="A29" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="B29" s="24" t="s">
+        <v>391</v>
+      </c>
+      <c r="C29" s="24"/>
+      <c r="D29" s="24"/>
+      <c r="E29" s="24"/>
+      <c r="F29" s="24"/>
+      <c r="G29" s="24"/>
+      <c r="H29" s="24"/>
+      <c r="I29" s="24"/>
+      <c r="J29" s="24"/>
+      <c r="K29" s="24"/>
+    </row>
+    <row r="30" spans="1:11">
+      <c r="A30" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B30" s="24" t="s">
+        <v>448</v>
+      </c>
+      <c r="C30" s="24"/>
+      <c r="D30" s="24"/>
+      <c r="E30" s="24"/>
+      <c r="F30" s="24"/>
+      <c r="G30" s="24"/>
+      <c r="H30" s="24"/>
+      <c r="I30" s="24"/>
+      <c r="J30" s="24"/>
+      <c r="K30" s="24"/>
+    </row>
+    <row r="32" spans="1:11">
+      <c r="A32" s="25" t="s">
+        <v>159</v>
+      </c>
+      <c r="B32" s="25" t="s">
+        <v>72</v>
+      </c>
+      <c r="C32" s="25" t="s">
+        <v>73</v>
+      </c>
+      <c r="D32" s="25"/>
+      <c r="E32" s="25"/>
+      <c r="F32" s="25"/>
+      <c r="G32" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="H32" s="25" t="s">
+        <v>75</v>
+      </c>
+      <c r="I32" s="25" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="46.5">
+      <c r="A33" s="25"/>
+      <c r="B33" s="25"/>
+      <c r="C33" s="15" t="s">
+        <v>392</v>
+      </c>
+      <c r="D33" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="E33" s="15" t="s">
+        <v>393</v>
+      </c>
+      <c r="F33" s="15" t="s">
+        <v>394</v>
+      </c>
+      <c r="G33" s="25"/>
+      <c r="H33" s="25"/>
+      <c r="I33" s="25"/>
+    </row>
+    <row r="34" spans="1:9" ht="46.5">
+      <c r="A34" s="17" t="s">
+        <v>162</v>
+      </c>
+      <c r="B34" s="16" t="s">
+        <v>395</v>
+      </c>
+      <c r="C34" s="13" t="s">
+        <v>396</v>
+      </c>
+      <c r="D34" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="E34" s="13" t="s">
+        <v>397</v>
+      </c>
+      <c r="F34" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="G34" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="H34" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="I34" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="46.5">
+      <c r="A35" s="17" t="s">
+        <v>167</v>
+      </c>
+      <c r="B35" s="16" t="s">
+        <v>398</v>
+      </c>
+      <c r="C35" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="D35" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="E35" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="F35" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="G35" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="H35" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="I35" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="46.5">
+      <c r="A36" s="17" t="s">
+        <v>171</v>
+      </c>
+      <c r="B36" s="16" t="s">
+        <v>399</v>
+      </c>
+      <c r="C36" s="13" t="s">
+        <v>396</v>
+      </c>
+      <c r="D36" s="13" t="s">
+        <v>400</v>
+      </c>
+      <c r="E36" s="13" t="s">
+        <v>397</v>
+      </c>
+      <c r="F36" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="G36" s="13" t="s">
+        <v>401</v>
+      </c>
+      <c r="H36" s="13" t="s">
+        <v>402</v>
+      </c>
+      <c r="I36" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" ht="69.75">
+      <c r="A37" s="17" t="s">
+        <v>175</v>
+      </c>
+      <c r="B37" s="16" t="s">
+        <v>403</v>
+      </c>
+      <c r="C37" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="D37" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="E37" s="13" t="s">
+        <v>404</v>
+      </c>
+      <c r="F37" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="G37" s="13" t="s">
+        <v>405</v>
+      </c>
+      <c r="H37" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="I37" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" ht="69.75">
+      <c r="A38" s="17" t="s">
+        <v>183</v>
+      </c>
+      <c r="B38" s="16" t="s">
+        <v>406</v>
+      </c>
+      <c r="C38" s="13" t="s">
+        <v>407</v>
+      </c>
+      <c r="D38" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="E38" s="13" t="s">
+        <v>408</v>
+      </c>
+      <c r="F38" s="13" t="s">
+        <v>409</v>
+      </c>
+      <c r="G38" s="13" t="s">
+        <v>410</v>
+      </c>
+      <c r="H38" s="13" t="s">
+        <v>411</v>
+      </c>
+      <c r="I38" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="93">
+      <c r="A39" s="17" t="s">
+        <v>183</v>
+      </c>
+      <c r="B39" s="16" t="s">
+        <v>412</v>
+      </c>
+      <c r="C39" s="13" t="s">
+        <v>413</v>
+      </c>
+      <c r="D39" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="E39" s="13" t="s">
+        <v>414</v>
+      </c>
+      <c r="F39" s="13" t="s">
+        <v>415</v>
+      </c>
+      <c r="G39" s="13" t="s">
+        <v>416</v>
+      </c>
+      <c r="H39" s="13" t="s">
+        <v>411</v>
+      </c>
+      <c r="I39" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" ht="69.75">
+      <c r="A40" s="17" t="s">
+        <v>188</v>
+      </c>
+      <c r="B40" s="16" t="s">
+        <v>417</v>
+      </c>
+      <c r="C40" s="13" t="s">
+        <v>303</v>
+      </c>
+      <c r="D40" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="E40" s="13" t="s">
+        <v>397</v>
+      </c>
+      <c r="F40" s="13" t="s">
+        <v>418</v>
+      </c>
+      <c r="G40" s="13" t="s">
+        <v>419</v>
+      </c>
+      <c r="H40" s="13" t="s">
+        <v>420</v>
+      </c>
+      <c r="I40" s="17" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="69.75">
+      <c r="A41" s="17" t="s">
+        <v>193</v>
+      </c>
+      <c r="B41" s="16" t="s">
+        <v>421</v>
+      </c>
+      <c r="C41" s="13" t="s">
+        <v>422</v>
+      </c>
+      <c r="D41" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="E41" s="13" t="s">
+        <v>423</v>
+      </c>
+      <c r="F41" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="G41" s="13" t="s">
+        <v>424</v>
+      </c>
+      <c r="H41" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="I41" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" ht="69.75">
+      <c r="A42" s="17" t="s">
+        <v>197</v>
+      </c>
+      <c r="B42" s="16" t="s">
+        <v>425</v>
+      </c>
+      <c r="C42" s="13" t="s">
+        <v>307</v>
+      </c>
+      <c r="D42" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="E42" s="13" t="s">
+        <v>404</v>
+      </c>
+      <c r="F42" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="G42" s="13" t="s">
+        <v>426</v>
+      </c>
+      <c r="H42" s="13" t="s">
+        <v>411</v>
+      </c>
+      <c r="I42" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" ht="46.5">
+      <c r="A43" s="17" t="s">
+        <v>427</v>
+      </c>
+      <c r="B43" s="16" t="s">
+        <v>428</v>
+      </c>
+      <c r="C43" s="13" t="s">
+        <v>311</v>
+      </c>
+      <c r="D43" s="13" t="s">
+        <v>429</v>
+      </c>
+      <c r="E43" s="13" t="s">
+        <v>430</v>
+      </c>
+      <c r="F43" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="G43" s="13" t="s">
+        <v>431</v>
+      </c>
+      <c r="H43" s="13" t="s">
+        <v>411</v>
+      </c>
+      <c r="I43" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" ht="46.5">
+      <c r="A44" s="17" t="s">
+        <v>432</v>
+      </c>
+      <c r="B44" s="16" t="s">
+        <v>433</v>
+      </c>
+      <c r="C44" s="13" t="s">
+        <v>434</v>
+      </c>
+      <c r="D44" s="13" t="s">
+        <v>429</v>
+      </c>
+      <c r="E44" s="13" t="s">
+        <v>435</v>
+      </c>
+      <c r="F44" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="G44" s="13" t="s">
+        <v>436</v>
+      </c>
+      <c r="H44" s="13" t="s">
+        <v>420</v>
+      </c>
+      <c r="I44" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" ht="46.5">
+      <c r="A45" s="17" t="s">
+        <v>432</v>
+      </c>
+      <c r="B45" s="16" t="s">
+        <v>437</v>
+      </c>
+      <c r="C45" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="D45" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="E45" s="13" t="s">
+        <v>438</v>
+      </c>
+      <c r="F45" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="G45" s="13" t="s">
+        <v>439</v>
+      </c>
+      <c r="H45" s="13" t="s">
+        <v>420</v>
+      </c>
+      <c r="I45" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="16">
+    <mergeCell ref="B26:G26"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A22:K22"/>
+    <mergeCell ref="A24:K24"/>
+    <mergeCell ref="B27:G27"/>
+    <mergeCell ref="B28:G28"/>
+    <mergeCell ref="B29:K29"/>
+    <mergeCell ref="B30:K30"/>
+    <mergeCell ref="A32:A33"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="C32:F32"/>
+    <mergeCell ref="G32:G33"/>
+    <mergeCell ref="H32:H33"/>
+    <mergeCell ref="I32:I33"/>
+  </mergeCells>
+  <conditionalFormatting sqref="I34:I45">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+      <formula>"Pass"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+      <formula>"Fail"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
+      <formula>"Block"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" sqref="I34:I45" xr:uid="{37897F8D-8509-4E44-A037-2C3E7CBDC1C3}">
+      <formula1>"Pass,Fail,No run,Block"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93C8330E-079C-4579-8133-7533964AD0F3}">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr defaultColWidth="7.625" defaultRowHeight="23.25"/>
   <cols>
     <col min="1" max="1" width="5.25" style="8" customWidth="1"/>
@@ -4444,6 +6631,68 @@
         <v>297</v>
       </c>
     </row>
+    <row r="4" spans="1:11" ht="46.5">
+      <c r="A4" s="17">
+        <v>3</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>446</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>440</v>
+      </c>
+      <c r="D4" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="E4" s="13"/>
+      <c r="F4" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="G4" s="17" t="s">
+        <v>216</v>
+      </c>
+      <c r="H4" s="17" t="s">
+        <v>441</v>
+      </c>
+      <c r="I4" s="17" t="s">
+        <v>441</v>
+      </c>
+      <c r="J4" s="13"/>
+      <c r="K4" s="13" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="69.75">
+      <c r="A5" s="17">
+        <v>4</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>447</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>443</v>
+      </c>
+      <c r="D5" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="E5" s="13"/>
+      <c r="F5" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="G5" s="17" t="s">
+        <v>216</v>
+      </c>
+      <c r="H5" s="17" t="s">
+        <v>444</v>
+      </c>
+      <c r="I5" s="17" t="s">
+        <v>441</v>
+      </c>
+      <c r="J5" s="13"/>
+      <c r="K5" s="13" t="s">
+        <v>445</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
UnitTest UT10, UT11 found bug in BookingService ConfirmedState amd AvailabilityServiceImpl
</commit_message>
<xml_diff>
--- a/test/FIWDEE_UnitTest_Report.xlsx
+++ b/test/FIWDEE_UnitTest_Report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\ProjectPOS\FIWDEE-CP353002-69_1PrinciplesOfSoftwareDesign\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB42AA64-528F-4FC8-A1F6-6AC0387E7895}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12DA990E-553B-4FED-8160-0A90ACC6BDDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9B0ECA1C-B255-4EEE-B7A8-035645CFC3D9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{9B0ECA1C-B255-4EEE-B7A8-035645CFC3D9}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Summary" sheetId="1" r:id="rId1"/>
@@ -24,9 +24,12 @@
     <sheet name="UT07_GetBookingById_DT" sheetId="9" r:id="rId9"/>
     <sheet name="UT08_BookingState_DT" sheetId="10" r:id="rId10"/>
     <sheet name="UT09_StateFactory_EC" sheetId="11" r:id="rId11"/>
+    <sheet name="UT10_Availability_BVA" sheetId="12" r:id="rId12"/>
+    <sheet name="UT11_Availability_EC" sheetId="14" r:id="rId13"/>
+    <sheet name="UT12_BookingMapper_EC" sheetId="15" r:id="rId14"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId12"/>
+    <externalReference r:id="rId15"/>
   </externalReferences>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -74,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1797" uniqueCount="712">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2100" uniqueCount="841">
   <si>
     <t>FIWDEE – Unit Test Design</t>
   </si>
@@ -2210,6 +2213,393 @@
   </si>
   <si>
     <t>Strong Normal Equivalence Class Testing (ทุกค่าใน enum)</t>
+  </si>
+  <si>
+    <t>durationMinutes</t>
+  </si>
+  <si>
+    <t>AvailabilityServiceImpl.checkAvailability – จำนวนรอบเวลาตามระยะเวลาบริการ</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>90</t>
+  </si>
+  <si>
+    <t>AvailabilityResponseDTO checkAvailability(LocalDate date, Long serviceId, Integer durationMinutes)</t>
+  </si>
+  <si>
+    <t>719</t>
+  </si>
+  <si>
+    <t>UC-08 • BR-BKG-02 • SRS 7.2</t>
+  </si>
+  <si>
+    <t>721</t>
+  </si>
+  <si>
+    <t>TC008 เป็นเคส robustness เพิ่มนอกตาราง BVA (ค่าที่ทำให้เวลาวนข้ามวัน)</t>
+  </si>
+  <si>
+    <t>UT10-TC001</t>
+  </si>
+  <si>
+    <t>ใช้ระยะเวลาจาก option แรก = 60 • durationMinutes ใน response = 60 • 12 รอบ (10:00–21:00)</t>
+  </si>
+  <si>
+    <t>UT10-TC002</t>
+  </si>
+  <si>
+    <t>durationMinutes = 1 • 12 รอบ (10:00–21:00) รอบสุดท้ายจบ 21:01</t>
+  </si>
+  <si>
+    <t>UT10-TC003</t>
+  </si>
+  <si>
+    <t>12 รอบ</t>
+  </si>
+  <si>
+    <t>UT10-TC004</t>
+  </si>
+  <si>
+    <t>11 รอบ (10:00–20:00) • ไม่มีรอบ 21:00 เพราะจะจบ 22:30</t>
+  </si>
+  <si>
+    <t>UT10-TC005</t>
+  </si>
+  <si>
+    <t>1 รอบ (10:00–21:59)</t>
+  </si>
+  <si>
+    <t>UT10-TC006</t>
+  </si>
+  <si>
+    <t>720</t>
+  </si>
+  <si>
+    <t>UT10-TC007</t>
+  </si>
+  <si>
+    <t>0 รอบ (availableSlots ว่าง) ไม่เกิด Exception</t>
+  </si>
+  <si>
+    <t>UT10-TC008</t>
+  </si>
+  <si>
+    <t>900 (นอกโดเมน: เกินเที่ยงคืน)</t>
+  </si>
+  <si>
+    <t>0 รอบ</t>
+  </si>
+  <si>
+    <t>22 รอบ</t>
+  </si>
+  <si>
+    <t>1 รอบ</t>
+  </si>
+  <si>
+    <t>11 รอบ</t>
+  </si>
+  <si>
+    <t>1 รอบ (10:00–22:00)</t>
+  </si>
+  <si>
+    <t>UT10 – AvailabilityServiceImpl.checkAvailability – จำนวนรอบเวลาตามระยะเวลาบริการ</t>
+  </si>
+  <si>
+    <t>DEF-012</t>
+  </si>
+  <si>
+    <t>UT11 – AvailabilityServiceImpl.checkAvailability – สภาพร้านและทรัพยากร</t>
+  </si>
+  <si>
+    <t>DEF-006</t>
+  </si>
+  <si>
+    <t>UT12 – BookingMapper (toMyBookingResponse / toBookingResponse / list)</t>
+  </si>
+  <si>
+    <t>Weak Normal Equivalence Class Testing</t>
+  </si>
+  <si>
+    <t>date ระบุมา</t>
+  </si>
+  <si>
+    <t>date = null → ใช้วันนี้</t>
+  </si>
+  <si>
+    <t>service inactive</t>
+  </si>
+  <si>
+    <t>service มีอยู่และ active</t>
+  </si>
+  <si>
+    <t>วันนั้นร้านปิด (isClosed = true)</t>
+  </si>
+  <si>
+    <t>มี BusinessHours ของวันนั้นและเปิด</t>
+  </si>
+  <si>
+    <t>ไม่มี BusinessHours ของวันนั้น → ใช้ค่าเริ่มต้น 10:00–21:00</t>
+  </si>
+  <si>
+    <t>หมอนวดหยุดถูกตัดออกจาก availableTherapists</t>
+  </si>
+  <si>
+    <t>รอบที่ไม่มีห้องว่าง → available = false</t>
+  </si>
+  <si>
+    <t>booking เดิมสถานะ COMPLETED/CANCELLED/NO_SHOW ไม่ล็อกทรัพยากร</t>
+  </si>
+  <si>
+    <t>AvailabilityServiceImpl.checkAvailability – สภาพร้านและทรัพยากร</t>
+  </si>
+  <si>
+    <t>checkAvailability(date, serviceId, durationMinutes)</t>
+  </si>
+  <si>
+    <t>UC-08, UC-08a, UC-08b • SRS 7.2</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>UT11-TC001</t>
+  </si>
+  <si>
+    <t>2026-11-09</t>
+  </si>
+  <si>
+    <t>ร้านเปิด 10–22, T5 + R101 ว่าง</t>
+  </si>
+  <si>
+    <t>(V1,V3,V4) 12 รอบ ทุกรอบ available = true, availableTherapists มี T5, availableRooms มี R101</t>
+  </si>
+  <si>
+    <t>UT11-TC002</t>
+  </si>
+  <si>
+    <t>ร้านเปิด</t>
+  </si>
+  <si>
+    <t>(V2) date ใน response = วันนี้</t>
+  </si>
+  <si>
+    <t>UT11-TC003</t>
+  </si>
+  <si>
+    <t>ไม่มีแถว BusinessHours วันจันทร์</t>
+  </si>
+  <si>
+    <t>(V5) 11 รอบ (10:00–20:00)</t>
+  </si>
+  <si>
+    <t>UT11-TC004</t>
+  </si>
+  <si>
+    <t>T5 isDayOff, T8 ว่าง</t>
+  </si>
+  <si>
+    <t>(V6) availableTherapists ทุกรอบมีแค่ T8</t>
+  </si>
+  <si>
+    <t>UT11-TC005</t>
+  </si>
+  <si>
+    <t>R101 มีคิว 13:00–14:00 (ห้องเดียว)</t>
+  </si>
+  <si>
+    <t>(V7) รอบ 12:00, 13:00, 14:00 available = false (12:00 จบ 13:00 + buffer 15 ชนคิว, 14:00 ติด buffer ถึง 14:15) • รอบอื่น true</t>
+  </si>
+  <si>
+    <t>UT11-TC006</t>
+  </si>
+  <si>
+    <t>R101 (ห้องเดียว) มีคิว 13:00–14:00 สถานะ COMPLETED</t>
+  </si>
+  <si>
+    <t>UT11-TC007</t>
+  </si>
+  <si>
+    <t>(I1) NotFoundException</t>
+  </si>
+  <si>
+    <t>UT11-TC008</t>
+  </si>
+  <si>
+    <t>S3 inactive</t>
+  </si>
+  <si>
+    <t>(I2) ValidationException "Selected service is currently inactive"</t>
+  </si>
+  <si>
+    <t>UT11-TC009</t>
+  </si>
+  <si>
+    <t>BusinessHours MONDAY isClosed = true</t>
+  </si>
+  <si>
+    <t>(I3) availableSlots ว่าง ไม่เกิด Exception</t>
+  </si>
+  <si>
+    <t>date ใน response = วันนี้</t>
+  </si>
+  <si>
+    <t>availableTherapists ทุกรอบมีแค่ T8</t>
+  </si>
+  <si>
+    <t>12 รอบ ทุกรอบ available = true, availableTherapists มี T5, availableRooms มี R101</t>
+  </si>
+  <si>
+    <t>รอบ 12:00, 13:00, 14:00 available = false (12:00 จบ 13:00 + buffer 15 ชนคิว, 14:00 ติด buffer ถึง 14:15) • รอบอื่น true</t>
+  </si>
+  <si>
+    <t>availableSlots ว่าง</t>
+  </si>
+  <si>
+    <t>(V8) รอบ 13:00 available = true เพราะ COMPLETED ไม่ล็อกทรัพยากร</t>
+  </si>
+  <si>
+    <t>available = flase</t>
+  </si>
+  <si>
+    <t>Booking มีครบทุก relation</t>
+  </si>
+  <si>
+    <t>ไม่มี: ทุกกรณีต้องไม่โยน Exception</t>
+  </si>
+  <si>
+    <t>therapist = null</t>
+  </si>
+  <si>
+    <t>service, room, durationOption, customer = null</t>
+  </si>
+  <si>
+    <t>status = null</t>
+  </si>
+  <si>
+    <t>room มีแต่ roomType = null</t>
+  </si>
+  <si>
+    <t>booking = null</t>
+  </si>
+  <si>
+    <t>List = null หรือว่าง</t>
+  </si>
+  <si>
+    <t>BookingMapper (toMyBookingResponse / toBookingResponse / list)</t>
+  </si>
+  <si>
+    <t>Functional testing - Weak Normal Equivalence Class Testing</t>
+  </si>
+  <si>
+    <t>toMyBookingResponse, toMyBookingResponses, toBookingResponse, toBookingResponses</t>
+  </si>
+  <si>
+    <t>เมธอด</t>
+  </si>
+  <si>
+    <t>Booking ที่ส่งเข้า</t>
+  </si>
+  <si>
+    <t>UT12-TC001</t>
+  </si>
+  <si>
+    <t>toBookingResponse</t>
+  </si>
+  <si>
+    <t>ครบทุก relation</t>
+  </si>
+  <si>
+    <t>(V1) map ครบทุก field: customerId/Name/Phone, serviceId/Name, therapistId/Name, roomId/Number/Type, status, channel, notes</t>
+  </si>
+  <si>
+    <t>UT12-TC002</t>
+  </si>
+  <si>
+    <t>toMyBookingResponse</t>
+  </si>
+  <si>
+    <t>(V1) serviceName, therapistName, roomNumber, durationMinutes = 60, status = "CONFIRMED"</t>
+  </si>
+  <si>
+    <t>UT12-TC003</t>
+  </si>
+  <si>
+    <t>(V2) therapistId และ therapistName = null</t>
+  </si>
+  <si>
+    <t>UT12-TC004</t>
+  </si>
+  <si>
+    <t>service/room/option/customer = null</t>
+  </si>
+  <si>
+    <t>(V3) field ที่เกี่ยวข้องเป็น null</t>
+  </si>
+  <si>
+    <t>UT12-TC005</t>
+  </si>
+  <si>
+    <t>(V4) status = null</t>
+  </si>
+  <si>
+    <t>UT12-TC006</t>
+  </si>
+  <si>
+    <t>room.roomType = null</t>
+  </si>
+  <si>
+    <t>(V5) roomNumber มีค่า, roomType = null</t>
+  </si>
+  <si>
+    <t>UT12-TC007</t>
+  </si>
+  <si>
+    <t>toBookingResponse / toMyBookingResponse</t>
+  </si>
+  <si>
+    <t>(V6) คืน null</t>
+  </si>
+  <si>
+    <t>UT12-TC008</t>
+  </si>
+  <si>
+    <t>toBookingResponses / toMyBookingResponses</t>
+  </si>
+  <si>
+    <t>null และ []</t>
+  </si>
+  <si>
+    <t>(V7) คืน List ว่าง</t>
+  </si>
+  <si>
+    <t>UC-09 • DTO Pattern + Mapper</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> คืน List ว่าง</t>
+  </si>
+  <si>
+    <t>roomNumber มีค่า, roomType = null</t>
+  </si>
+  <si>
+    <t>field ที่เกี่ยวข้องเป็น null</t>
+  </si>
+  <si>
+    <t>therapistId และ therapistName = null</t>
+  </si>
+  <si>
+    <t>serviceName, therapistName, roomNumber, durationMinutes = 60, status = "CONFIRMED"</t>
+  </si>
+  <si>
+    <t>map ครบทุก field</t>
+  </si>
+  <si>
+    <t>Booking ที่ COMPLETED ยังล็อกห้องและหมอนวด</t>
+  </si>
+  <si>
+    <t>service/impl/BookingServiceImpl.java และ AvailabilityServiceImpl.java : EXCLUDED_STATUSES มีแค่ CANCELLED, NO_SHOW • UC-08 ข้อ 4 ระบุว่า COMPLETED ไม่ใช่ active • UT11-TC006</t>
   </si>
 </sst>
 </file>
@@ -2485,21 +2875,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2507,9 +2882,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2521,6 +2893,21 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -2530,11 +2917,56 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="30">
+  <dxfs count="36">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -3221,7 +3653,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{659A469D-55E7-4F16-B797-78C1D60B492C}">
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="1" width="5.25" customWidth="1"/>
@@ -3233,14 +3665,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
@@ -3275,17 +3707,17 @@
       </c>
     </row>
     <row r="3" spans="1:9" ht="21">
-      <c r="A3" s="31" t="s">
+      <c r="A3" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="31"/>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="31"/>
-      <c r="G3" s="31"/>
-      <c r="H3" s="31"/>
-      <c r="I3" s="31"/>
+      <c r="B3" s="26"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="26"/>
+      <c r="G3" s="26"/>
+      <c r="H3" s="26"/>
+      <c r="I3" s="26"/>
     </row>
     <row r="4" spans="1:9" ht="42">
       <c r="A4" s="3">
@@ -3583,37 +4015,137 @@
       </c>
       <c r="I12" s="4"/>
     </row>
-    <row r="13" spans="1:9" ht="21">
-      <c r="A13" s="29" t="s">
+    <row r="13" spans="1:9" ht="64.5" customHeight="1">
+      <c r="A13" s="3">
+        <v>10</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>742</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D13" s="3">
+        <f>COUNTA(UT10_Availability_BVA!$A$12:$A$19)</f>
+        <v>8</v>
+      </c>
+      <c r="E13" s="3">
+        <f>COUNTIF(UT10_Availability_BVA!$E$12:$E$19,"Pass")</f>
+        <v>7</v>
+      </c>
+      <c r="F13" s="3">
+        <f>COUNTIF(UT10_Availability_BVA!$E$12:$E$19,"Fail")</f>
+        <v>1</v>
+      </c>
+      <c r="G13" s="3">
+        <f>COUNTIF(UT10_Availability_BVA!$E$12:$E$19,"No run")</f>
+        <v>0</v>
+      </c>
+      <c r="H13" s="3">
+        <f>COUNTIF(UT10_Availability_BVA!$E$12:$E$19,"Block")</f>
+        <v>0</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="64.5" customHeight="1">
+      <c r="A14" s="3">
+        <v>11</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>744</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D14" s="3">
+        <f>COUNTA(UT11_Availability_EC!$A$24:$A$32)</f>
+        <v>8</v>
+      </c>
+      <c r="E14" s="3">
+        <f>COUNTIF(UT11_Availability_EC!$G$24:$G$32,"Pass")</f>
+        <v>7</v>
+      </c>
+      <c r="F14" s="3">
+        <f>COUNTIF(UT11_Availability_EC!$G$24:$G$32,"Fail")</f>
+        <v>1</v>
+      </c>
+      <c r="G14" s="3">
+        <f>COUNTIF(UT11_Availability_EC!$G$24:$G$32,"No run")</f>
+        <v>0</v>
+      </c>
+      <c r="H14" s="3">
+        <f>COUNTIF(UT11_Availability_EC!$G$24:$G$32,"Block")</f>
+        <v>0</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>745</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="64.5" customHeight="1">
+      <c r="A15" s="3">
+        <v>12</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>746</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>747</v>
+      </c>
+      <c r="D15" s="3">
+        <f>COUNTA(UT12_BookingMapper_EC!$A$23:$A$30)</f>
+        <v>7</v>
+      </c>
+      <c r="E15" s="3">
+        <f>COUNTIF(UT12_BookingMapper_EC!$F$23:$F$30,"Pass")</f>
+        <v>7</v>
+      </c>
+      <c r="F15" s="3">
+        <f>COUNTIF(UT12_BookingMapper_EC!$F$23:$F$30,"Fail")</f>
+        <v>0</v>
+      </c>
+      <c r="G15" s="3">
+        <f>COUNTIF(UT12_BookingMapper_EC!$F$23:$F$30,"No run")</f>
+        <v>0</v>
+      </c>
+      <c r="H15" s="3">
+        <f>COUNTIF(UT12_BookingMapper_EC!$F$23:$F$30,"Block")</f>
+        <v>0</v>
+      </c>
+      <c r="I15" s="4"/>
+    </row>
+    <row r="16" spans="1:9" ht="21">
+      <c r="A16" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="29"/>
-      <c r="C13" s="29"/>
-      <c r="D13" s="5" cm="1">
-        <f t="array" ref="D13">SUMPRODUCT(ISNUMBER(D4:D12)*D4:D12)</f>
-        <v>126</v>
-      </c>
-      <c r="E13" s="6" cm="1">
-        <f t="array" ref="E13">SUMPRODUCT(ISNUMBER(E4:E12)*E4:E12)</f>
-        <v>119</v>
-      </c>
-      <c r="F13" s="7" cm="1">
-        <f t="array" ref="F13">SUMPRODUCT(ISNUMBER(F4:F12)*F4:F12)</f>
-        <v>7</v>
-      </c>
-      <c r="G13" s="5" cm="1">
-        <f t="array" ref="G13">SUMPRODUCT(ISNUMBER(G4:G12)*G4:G12)</f>
+      <c r="B16" s="24"/>
+      <c r="C16" s="24"/>
+      <c r="D16" s="5" cm="1">
+        <f t="array" ref="D16">SUMPRODUCT(ISNUMBER(D4:D15)*D4:D15)</f>
+        <v>149</v>
+      </c>
+      <c r="E16" s="6" cm="1">
+        <f t="array" ref="E16">SUMPRODUCT(ISNUMBER(E4:E15)*E4:E15)</f>
+        <v>140</v>
+      </c>
+      <c r="F16" s="7" cm="1">
+        <f t="array" ref="F16">SUMPRODUCT(ISNUMBER(F4:F15)*F4:F15)</f>
+        <v>9</v>
+      </c>
+      <c r="G16" s="5" cm="1">
+        <f t="array" ref="G16">SUMPRODUCT(ISNUMBER(G4:G15)*G4:G15)</f>
         <v>0</v>
       </c>
-      <c r="H13" s="5" cm="1">
-        <f t="array" ref="H13">SUMPRODUCT(ISNUMBER(H4:H12)*H4:H12)</f>
+      <c r="H16" s="5" cm="1">
+        <f t="array" ref="H16">SUMPRODUCT(ISNUMBER(H4:H15)*H4:H15)</f>
         <v>0</v>
       </c>
-      <c r="I13" s="4"/>
+      <c r="I16" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A16:C16"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A3:I3"/>
   </mergeCells>
@@ -3640,40 +4172,40 @@
       </c>
     </row>
     <row r="2" spans="1:8" ht="22.5" customHeight="1">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="38" t="s">
         <v>501</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
+      <c r="B2" s="38"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="38"/>
+      <c r="F2" s="38"/>
+      <c r="G2" s="38"/>
+      <c r="H2" s="38"/>
     </row>
     <row r="3" spans="1:8" ht="22.5" customHeight="1">
-      <c r="A3" s="25" t="s">
+      <c r="A3" s="38" t="s">
         <v>502</v>
       </c>
-      <c r="B3" s="25"/>
-      <c r="C3" s="25"/>
-      <c r="D3" s="25"/>
-      <c r="E3" s="25"/>
-      <c r="F3" s="25"/>
-      <c r="G3" s="25"/>
-      <c r="H3" s="25"/>
+      <c r="B3" s="38"/>
+      <c r="C3" s="38"/>
+      <c r="D3" s="38"/>
+      <c r="E3" s="38"/>
+      <c r="F3" s="38"/>
+      <c r="G3" s="38"/>
+      <c r="H3" s="38"/>
     </row>
     <row r="4" spans="1:8" ht="22.5" customHeight="1">
-      <c r="A4" s="25" t="s">
+      <c r="A4" s="38" t="s">
         <v>503</v>
       </c>
-      <c r="B4" s="25"/>
-      <c r="C4" s="25"/>
-      <c r="D4" s="25"/>
-      <c r="E4" s="25"/>
-      <c r="F4" s="25"/>
-      <c r="G4" s="25"/>
-      <c r="H4" s="25"/>
+      <c r="B4" s="38"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="38"/>
+      <c r="E4" s="38"/>
+      <c r="F4" s="38"/>
+      <c r="G4" s="38"/>
+      <c r="H4" s="38"/>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="18" t="s">
@@ -3960,40 +4492,40 @@
       <c r="H17" s="17"/>
     </row>
     <row r="18" spans="1:8" ht="22.5" customHeight="1">
-      <c r="A18" s="26" t="s">
+      <c r="A18" s="34" t="s">
         <v>525</v>
       </c>
-      <c r="B18" s="26"/>
-      <c r="C18" s="26"/>
-      <c r="D18" s="26"/>
-      <c r="E18" s="26"/>
-      <c r="F18" s="26"/>
-      <c r="G18" s="26"/>
-      <c r="H18" s="26"/>
+      <c r="B18" s="34"/>
+      <c r="C18" s="34"/>
+      <c r="D18" s="34"/>
+      <c r="E18" s="34"/>
+      <c r="F18" s="34"/>
+      <c r="G18" s="34"/>
+      <c r="H18" s="34"/>
     </row>
     <row r="20" spans="1:8" ht="20.100000000000001" customHeight="1">
-      <c r="A20" s="27" t="s">
+      <c r="A20" s="31" t="s">
         <v>57</v>
       </c>
-      <c r="B20" s="27"/>
-      <c r="C20" s="27"/>
-      <c r="D20" s="27"/>
-      <c r="E20" s="27"/>
-      <c r="F20" s="27"/>
-      <c r="G20" s="27"/>
-      <c r="H20" s="27"/>
+      <c r="B20" s="31"/>
+      <c r="C20" s="31"/>
+      <c r="D20" s="31"/>
+      <c r="E20" s="31"/>
+      <c r="F20" s="31"/>
+      <c r="G20" s="31"/>
+      <c r="H20" s="31"/>
     </row>
     <row r="22" spans="1:8" ht="22.5" customHeight="1">
       <c r="A22" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="B22" s="24" t="s">
+      <c r="B22" s="33" t="s">
         <v>526</v>
       </c>
-      <c r="C22" s="24"/>
-      <c r="D22" s="24"/>
-      <c r="E22" s="24"/>
-      <c r="F22" s="24"/>
+      <c r="C22" s="33"/>
+      <c r="D22" s="33"/>
+      <c r="E22" s="33"/>
+      <c r="F22" s="33"/>
       <c r="G22" s="12" t="s">
         <v>60</v>
       </c>
@@ -4005,13 +4537,13 @@
       <c r="A23" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="B23" s="24" t="s">
+      <c r="B23" s="33" t="s">
         <v>527</v>
       </c>
-      <c r="C23" s="24"/>
-      <c r="D23" s="24"/>
-      <c r="E23" s="24"/>
-      <c r="F23" s="24"/>
+      <c r="C23" s="33"/>
+      <c r="D23" s="33"/>
+      <c r="E23" s="33"/>
+      <c r="F23" s="33"/>
       <c r="G23" s="12" t="s">
         <v>63</v>
       </c>
@@ -4023,13 +4555,13 @@
       <c r="A24" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="B24" s="24" t="s">
+      <c r="B24" s="33" t="s">
         <v>65</v>
       </c>
-      <c r="C24" s="24"/>
-      <c r="D24" s="24"/>
-      <c r="E24" s="24"/>
-      <c r="F24" s="24"/>
+      <c r="C24" s="33"/>
+      <c r="D24" s="33"/>
+      <c r="E24" s="33"/>
+      <c r="F24" s="33"/>
       <c r="G24" s="12" t="s">
         <v>66</v>
       </c>
@@ -4041,55 +4573,55 @@
       <c r="A25" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="B25" s="24" t="s">
+      <c r="B25" s="33" t="s">
         <v>528</v>
       </c>
-      <c r="C25" s="24"/>
-      <c r="D25" s="24"/>
-      <c r="E25" s="24"/>
-      <c r="F25" s="24"/>
-      <c r="G25" s="24"/>
-      <c r="H25" s="24"/>
+      <c r="C25" s="33"/>
+      <c r="D25" s="33"/>
+      <c r="E25" s="33"/>
+      <c r="F25" s="33"/>
+      <c r="G25" s="33"/>
+      <c r="H25" s="33"/>
     </row>
     <row r="26" spans="1:8" ht="22.5" customHeight="1">
       <c r="A26" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="B26" s="24" t="s">
+      <c r="B26" s="33" t="s">
         <v>529</v>
       </c>
-      <c r="C26" s="24"/>
-      <c r="D26" s="24"/>
-      <c r="E26" s="24"/>
-      <c r="F26" s="24"/>
-      <c r="G26" s="24"/>
-      <c r="H26" s="24"/>
+      <c r="C26" s="33"/>
+      <c r="D26" s="33"/>
+      <c r="E26" s="33"/>
+      <c r="F26" s="33"/>
+      <c r="G26" s="33"/>
+      <c r="H26" s="33"/>
     </row>
     <row r="28" spans="1:8" ht="24" customHeight="1">
-      <c r="A28" s="28" t="s">
+      <c r="A28" s="32" t="s">
         <v>159</v>
       </c>
-      <c r="B28" s="28" t="s">
+      <c r="B28" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="C28" s="28" t="s">
+      <c r="C28" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="D28" s="28"/>
-      <c r="E28" s="28"/>
-      <c r="F28" s="28" t="s">
+      <c r="D28" s="32"/>
+      <c r="E28" s="32"/>
+      <c r="F28" s="32" t="s">
         <v>74</v>
       </c>
-      <c r="G28" s="28" t="s">
+      <c r="G28" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="H28" s="28" t="s">
+      <c r="H28" s="32" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="64.5" customHeight="1">
-      <c r="A29" s="28"/>
-      <c r="B29" s="28"/>
+      <c r="A29" s="32"/>
+      <c r="B29" s="32"/>
       <c r="C29" s="15" t="s">
         <v>530</v>
       </c>
@@ -4099,9 +4631,9 @@
       <c r="E29" s="15" t="s">
         <v>531</v>
       </c>
-      <c r="F29" s="28"/>
-      <c r="G29" s="28"/>
-      <c r="H29" s="28"/>
+      <c r="F29" s="32"/>
+      <c r="G29" s="32"/>
+      <c r="H29" s="32"/>
     </row>
     <row r="30" spans="1:8" ht="22.5" customHeight="1">
       <c r="A30" s="17" t="s">
@@ -5271,31 +5803,31 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="B22:F22"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A18:H18"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="C28:E28"/>
+    <mergeCell ref="F28:F29"/>
+    <mergeCell ref="G28:G29"/>
     <mergeCell ref="H28:H29"/>
     <mergeCell ref="B23:F23"/>
     <mergeCell ref="B24:F24"/>
     <mergeCell ref="B25:H25"/>
     <mergeCell ref="B26:H26"/>
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="B28:B29"/>
-    <mergeCell ref="C28:E28"/>
-    <mergeCell ref="F28:F29"/>
-    <mergeCell ref="G28:G29"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A18:H18"/>
-    <mergeCell ref="A20:H20"/>
-    <mergeCell ref="B22:F22"/>
   </mergeCells>
   <conditionalFormatting sqref="H30:H74">
-    <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5325,147 +5857,147 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="24" thickBot="1">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="33"/>
-      <c r="I1" s="33"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
     </row>
     <row r="2" spans="1:9" ht="24" thickBot="1">
       <c r="A2" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="34" t="s">
+      <c r="E2" s="28" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="34"/>
+      <c r="F2" s="28"/>
     </row>
     <row r="3" spans="1:9" ht="24" thickBot="1">
       <c r="A3" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="35" t="s">
+      <c r="B3" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="35"/>
+      <c r="C3" s="29"/>
       <c r="E3" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="35" t="s">
+      <c r="F3" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="G3" s="35"/>
-      <c r="H3" s="35"/>
-      <c r="I3" s="35"/>
+      <c r="G3" s="29"/>
+      <c r="H3" s="29"/>
+      <c r="I3" s="29"/>
     </row>
     <row r="4" spans="1:9" ht="24" thickBot="1">
       <c r="A4" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="32" t="s">
+      <c r="B4" s="30" t="s">
         <v>681</v>
       </c>
-      <c r="C4" s="32"/>
+      <c r="C4" s="30"/>
       <c r="E4" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="F4" s="32" t="s">
+      <c r="F4" s="30" t="s">
         <v>682</v>
       </c>
-      <c r="G4" s="32"/>
-      <c r="H4" s="32"/>
-      <c r="I4" s="32"/>
+      <c r="G4" s="30"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="30"/>
     </row>
     <row r="5" spans="1:9" ht="24" thickBot="1">
       <c r="A5" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="32" t="s">
+      <c r="B5" s="30" t="s">
         <v>535</v>
       </c>
-      <c r="C5" s="32"/>
+      <c r="C5" s="30"/>
     </row>
     <row r="6" spans="1:9" ht="24" thickBot="1">
       <c r="A6" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="32" t="s">
+      <c r="B6" s="30" t="s">
         <v>560</v>
       </c>
-      <c r="C6" s="32"/>
+      <c r="C6" s="30"/>
     </row>
     <row r="7" spans="1:9" ht="24" thickBot="1">
       <c r="A7" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="32" t="s">
+      <c r="B7" s="30" t="s">
         <v>683</v>
       </c>
-      <c r="C7" s="32"/>
+      <c r="C7" s="30"/>
     </row>
     <row r="8" spans="1:9" ht="24" thickBot="1">
       <c r="A8" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="32" t="s">
+      <c r="B8" s="30" t="s">
         <v>684</v>
       </c>
-      <c r="C8" s="32"/>
+      <c r="C8" s="30"/>
     </row>
     <row r="9" spans="1:9" ht="24" thickBot="1">
       <c r="A9" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="B9" s="32" t="s">
+      <c r="B9" s="30" t="s">
         <v>466</v>
       </c>
-      <c r="C9" s="32"/>
+      <c r="C9" s="30"/>
     </row>
     <row r="10" spans="1:9" ht="24" thickBot="1">
       <c r="A10" s="11" t="s">
         <v>685</v>
       </c>
-      <c r="B10" s="32" t="s">
+      <c r="B10" s="30" t="s">
         <v>571</v>
       </c>
-      <c r="C10" s="32"/>
+      <c r="C10" s="30"/>
     </row>
     <row r="11" spans="1:9" ht="24" thickBot="1">
       <c r="A11" s="11" t="s">
         <v>686</v>
       </c>
-      <c r="B11" s="32" t="s">
+      <c r="B11" s="30" t="s">
         <v>687</v>
       </c>
-      <c r="C11" s="32"/>
+      <c r="C11" s="30"/>
     </row>
     <row r="13" spans="1:9">
-      <c r="A13" s="27" t="s">
+      <c r="A13" s="31" t="s">
         <v>57</v>
       </c>
-      <c r="B13" s="27"/>
-      <c r="C13" s="27"/>
-      <c r="D13" s="27"/>
-      <c r="E13" s="27"/>
-      <c r="F13" s="27"/>
-      <c r="G13" s="27"/>
-      <c r="H13" s="27"/>
-      <c r="I13" s="27"/>
+      <c r="B13" s="31"/>
+      <c r="C13" s="31"/>
+      <c r="D13" s="31"/>
+      <c r="E13" s="31"/>
+      <c r="F13" s="31"/>
+      <c r="G13" s="31"/>
+      <c r="H13" s="31"/>
+      <c r="I13" s="31"/>
     </row>
     <row r="15" spans="1:9">
       <c r="A15" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="B15" s="24" t="s">
+      <c r="B15" s="33" t="s">
         <v>688</v>
       </c>
-      <c r="C15" s="24"/>
+      <c r="C15" s="33"/>
       <c r="D15" s="21"/>
       <c r="E15" s="21"/>
       <c r="F15" s="21"/>
@@ -5481,10 +6013,10 @@
       <c r="A16" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="B16" s="24" t="s">
+      <c r="B16" s="33" t="s">
         <v>689</v>
       </c>
-      <c r="C16" s="24"/>
+      <c r="C16" s="33"/>
       <c r="D16" s="21"/>
       <c r="E16" s="21"/>
       <c r="F16" s="21"/>
@@ -5500,10 +6032,10 @@
       <c r="A17" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="B17" s="24" t="s">
+      <c r="B17" s="33" t="s">
         <v>65</v>
       </c>
-      <c r="C17" s="24"/>
+      <c r="C17" s="33"/>
       <c r="D17" s="21"/>
       <c r="E17" s="21"/>
       <c r="F17" s="21"/>
@@ -5519,57 +6051,57 @@
       <c r="A18" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="B18" s="24" t="s">
+      <c r="B18" s="33" t="s">
         <v>690</v>
       </c>
-      <c r="C18" s="24"/>
-      <c r="D18" s="24"/>
-      <c r="E18" s="24"/>
-      <c r="F18" s="24"/>
-      <c r="G18" s="24"/>
-      <c r="H18" s="24"/>
-      <c r="I18" s="24"/>
+      <c r="C18" s="33"/>
+      <c r="D18" s="33"/>
+      <c r="E18" s="33"/>
+      <c r="F18" s="33"/>
+      <c r="G18" s="33"/>
+      <c r="H18" s="33"/>
+      <c r="I18" s="33"/>
     </row>
     <row r="19" spans="1:9" ht="46.5">
       <c r="A19" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="B19" s="24" t="s">
+      <c r="B19" s="33" t="s">
         <v>691</v>
       </c>
-      <c r="C19" s="24"/>
-      <c r="D19" s="24"/>
-      <c r="E19" s="24"/>
-      <c r="F19" s="24"/>
-      <c r="G19" s="24"/>
-      <c r="H19" s="24"/>
-      <c r="I19" s="24"/>
+      <c r="C19" s="33"/>
+      <c r="D19" s="33"/>
+      <c r="E19" s="33"/>
+      <c r="F19" s="33"/>
+      <c r="G19" s="33"/>
+      <c r="H19" s="33"/>
+      <c r="I19" s="33"/>
     </row>
     <row r="21" spans="1:9">
-      <c r="A21" s="28" t="s">
+      <c r="A21" s="32" t="s">
         <v>72</v>
       </c>
       <c r="B21" s="15" t="s">
         <v>73</v>
       </c>
-      <c r="C21" s="28" t="s">
+      <c r="C21" s="32" t="s">
         <v>74</v>
       </c>
-      <c r="D21" s="28" t="s">
+      <c r="D21" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="E21" s="28" t="s">
+      <c r="E21" s="32" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="22" spans="1:9">
-      <c r="A22" s="28"/>
+      <c r="A22" s="32"/>
       <c r="B22" s="15" t="s">
         <v>692</v>
       </c>
-      <c r="C22" s="28"/>
-      <c r="D22" s="28"/>
-      <c r="E22" s="28"/>
+      <c r="C22" s="32"/>
+      <c r="D22" s="32"/>
+      <c r="E22" s="32"/>
     </row>
     <row r="23" spans="1:9" ht="46.5">
       <c r="A23" s="16" t="s">
@@ -5709,17 +6241,1362 @@
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="F3:I3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="F4:I4"/>
+    <mergeCell ref="B18:I18"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="A13:I13"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
     <mergeCell ref="B19:I19"/>
     <mergeCell ref="A21:A22"/>
     <mergeCell ref="C21:C22"/>
     <mergeCell ref="D21:D22"/>
     <mergeCell ref="E21:E22"/>
+  </mergeCells>
+  <conditionalFormatting sqref="E23:E30">
+    <cfRule type="cellIs" dxfId="11" priority="1" operator="equal">
+      <formula>"Pass"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="10" priority="2" operator="equal">
+      <formula>"Fail"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="9" priority="3" operator="equal">
+      <formula>"Block"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" sqref="E23:E30" xr:uid="{63AF4BCA-D9D3-4060-939A-5EB7E4EBD518}">
+      <formula1>"Pass,Fail,No run,Block"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CEC8779-48C7-4989-A948-D292DD8E6ED3}">
+  <dimension ref="A1:I19"/>
+  <sheetFormatPr defaultColWidth="7.625" defaultRowHeight="23.25"/>
+  <cols>
+    <col min="1" max="1" width="19.25" style="8" customWidth="1"/>
+    <col min="2" max="2" width="15.75" style="8" customWidth="1"/>
+    <col min="3" max="3" width="49" style="8" customWidth="1"/>
+    <col min="4" max="4" width="15.75" style="8" customWidth="1"/>
+    <col min="5" max="5" width="14.875" style="8" customWidth="1"/>
+    <col min="6" max="7" width="7.625" style="8"/>
+    <col min="8" max="8" width="8.75" style="8" customWidth="1"/>
+    <col min="9" max="9" width="19.25" style="8" customWidth="1"/>
+    <col min="10" max="16384" width="7.625" style="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="31" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="15" t="s">
+        <v>712</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="H2" s="17" t="s">
+        <v>224</v>
+      </c>
+      <c r="I2" s="17" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B3" s="33" t="s">
+        <v>713</v>
+      </c>
+      <c r="C3" s="33"/>
+      <c r="D3" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="E3" s="14" t="s">
+        <v>154</v>
+      </c>
+      <c r="H3" s="17" t="s">
+        <v>228</v>
+      </c>
+      <c r="I3" s="17" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" s="33" t="s">
+        <v>231</v>
+      </c>
+      <c r="C4" s="33"/>
+      <c r="D4" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="E4" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="H4" s="17" t="s">
+        <v>232</v>
+      </c>
+      <c r="I4" s="17" t="s">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="46.5">
+      <c r="A5" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B5" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" s="33"/>
+      <c r="D5" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="H5" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="I5" s="17" t="s">
+        <v>715</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="46.5">
+      <c r="A6" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="B6" s="33" t="s">
+        <v>716</v>
+      </c>
+      <c r="C6" s="33"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
+      <c r="H6" s="17" t="s">
+        <v>238</v>
+      </c>
+      <c r="I6" s="17" t="s">
+        <v>717</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="46.5">
+      <c r="A7" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B7" s="33" t="s">
+        <v>718</v>
+      </c>
+      <c r="C7" s="33"/>
+      <c r="D7" s="33"/>
+      <c r="E7" s="33"/>
+      <c r="H7" s="17" t="s">
+        <v>244</v>
+      </c>
+      <c r="I7" s="17" t="s">
+        <v>719</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" s="34" t="s">
+        <v>720</v>
+      </c>
+      <c r="B8" s="34"/>
+      <c r="C8" s="34"/>
+      <c r="D8" s="34"/>
+      <c r="E8" s="34"/>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="C10" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="D10" s="32" t="s">
+        <v>75</v>
+      </c>
+      <c r="E10" s="32" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="46.5">
+      <c r="A11" s="32"/>
+      <c r="B11" s="15" t="s">
+        <v>712</v>
+      </c>
+      <c r="C11" s="32"/>
+      <c r="D11" s="32"/>
+      <c r="E11" s="32"/>
+    </row>
+    <row r="12" spans="1:9" ht="46.5">
+      <c r="A12" s="16" t="s">
+        <v>721</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>308</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>722</v>
+      </c>
+      <c r="D12" s="13"/>
+      <c r="E12" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="46.5">
+      <c r="A13" s="16" t="s">
+        <v>723</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>724</v>
+      </c>
+      <c r="D13" s="13"/>
+      <c r="E13" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" s="16" t="s">
+        <v>725</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>714</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>726</v>
+      </c>
+      <c r="D14" s="13" t="s">
+        <v>726</v>
+      </c>
+      <c r="E14" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="46.5">
+      <c r="A15" s="16" t="s">
+        <v>727</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>715</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>728</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>740</v>
+      </c>
+      <c r="E15" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16" s="16" t="s">
+        <v>729</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>717</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>730</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>739</v>
+      </c>
+      <c r="E16" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" s="16" t="s">
+        <v>731</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>732</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>741</v>
+      </c>
+      <c r="D17" s="13" t="s">
+        <v>739</v>
+      </c>
+      <c r="E17" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" s="16" t="s">
+        <v>733</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>719</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>734</v>
+      </c>
+      <c r="D18" s="13" t="s">
+        <v>737</v>
+      </c>
+      <c r="E18" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="46.5">
+      <c r="A19" s="16" t="s">
+        <v>735</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>736</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>737</v>
+      </c>
+      <c r="D19" s="13" t="s">
+        <v>738</v>
+      </c>
+      <c r="E19" s="17" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="A8:E8"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="D10:D11"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="B7:E7"/>
+  </mergeCells>
+  <conditionalFormatting sqref="E12:E19">
+    <cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
+      <formula>"Pass"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="7" priority="2" operator="equal">
+      <formula>"Fail"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="3" operator="equal">
+      <formula>"Block"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" sqref="E12:E19" xr:uid="{F5693CEB-D577-4041-A6F3-A39A911857DF}">
+      <formula1>"Pass,Fail,No run,Block"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{093C7D2F-D01A-4762-98C7-079E027DDEF2}">
+  <dimension ref="A1:I31"/>
+  <sheetFormatPr defaultColWidth="7.625" defaultRowHeight="23.25"/>
+  <cols>
+    <col min="1" max="1" width="19.25" style="8" customWidth="1"/>
+    <col min="2" max="4" width="14" style="8" customWidth="1"/>
+    <col min="5" max="5" width="42" style="8" customWidth="1"/>
+    <col min="6" max="6" width="29.25" style="8" customWidth="1"/>
+    <col min="7" max="7" width="14.875" style="8" customWidth="1"/>
+    <col min="8" max="8" width="12.25" style="8" customWidth="1"/>
+    <col min="9" max="9" width="14.375" style="8" customWidth="1"/>
+    <col min="10" max="16384" width="7.625" style="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="24" thickBot="1">
+      <c r="A1" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+    </row>
+    <row r="2" spans="1:9" ht="24" thickBot="1">
+      <c r="A2" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" s="28" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" s="28"/>
+    </row>
+    <row r="3" spans="1:9" ht="24" thickBot="1">
+      <c r="A3" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="29" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="29"/>
+      <c r="E3" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="29" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" s="29"/>
+      <c r="H3" s="29"/>
+      <c r="I3" s="29"/>
+    </row>
+    <row r="4" spans="1:9" ht="24" thickBot="1">
+      <c r="A4" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="30" t="s">
+        <v>748</v>
+      </c>
+      <c r="C4" s="30"/>
+      <c r="E4" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="G4" s="30"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="30"/>
+    </row>
+    <row r="5" spans="1:9" ht="24" thickBot="1">
+      <c r="A5" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="30" t="s">
+        <v>749</v>
+      </c>
+      <c r="C5" s="30"/>
+      <c r="E5" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" s="30" t="s">
+        <v>750</v>
+      </c>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+    </row>
+    <row r="6" spans="1:9" ht="24" thickBot="1">
+      <c r="A6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="30" t="s">
+        <v>751</v>
+      </c>
+      <c r="C6" s="30"/>
+      <c r="E6" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="F6" s="30" t="s">
+        <v>752</v>
+      </c>
+      <c r="G6" s="30"/>
+      <c r="H6" s="30"/>
+      <c r="I6" s="30"/>
+    </row>
+    <row r="7" spans="1:9" ht="24" thickBot="1">
+      <c r="A7" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="30" t="s">
+        <v>753</v>
+      </c>
+      <c r="C7" s="30"/>
+    </row>
+    <row r="8" spans="1:9" ht="24" thickBot="1">
+      <c r="A8" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" s="30" t="s">
+        <v>754</v>
+      </c>
+      <c r="C8" s="30"/>
+    </row>
+    <row r="9" spans="1:9" ht="24" thickBot="1">
+      <c r="A9" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="B9" s="30" t="s">
+        <v>755</v>
+      </c>
+      <c r="C9" s="30"/>
+    </row>
+    <row r="10" spans="1:9" ht="24" thickBot="1">
+      <c r="A10" s="11" t="s">
+        <v>685</v>
+      </c>
+      <c r="B10" s="30" t="s">
+        <v>756</v>
+      </c>
+      <c r="C10" s="30"/>
+    </row>
+    <row r="11" spans="1:9" ht="24" thickBot="1">
+      <c r="A11" s="11" t="s">
+        <v>686</v>
+      </c>
+      <c r="B11" s="30" t="s">
+        <v>757</v>
+      </c>
+      <c r="C11" s="30"/>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" s="31" t="s">
+        <v>57</v>
+      </c>
+      <c r="B13" s="31"/>
+      <c r="C13" s="31"/>
+      <c r="D13" s="31"/>
+      <c r="E13" s="31"/>
+      <c r="F13" s="31"/>
+      <c r="G13" s="31"/>
+      <c r="H13" s="31"/>
+      <c r="I13" s="31"/>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B15" s="33" t="s">
+        <v>758</v>
+      </c>
+      <c r="C15" s="33"/>
+      <c r="D15" s="33"/>
+      <c r="E15" s="33"/>
+      <c r="F15" s="21"/>
+      <c r="G15" s="21"/>
+      <c r="H15" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="I15" s="14" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="B16" s="33" t="s">
+        <v>62</v>
+      </c>
+      <c r="C16" s="33"/>
+      <c r="D16" s="33"/>
+      <c r="E16" s="33"/>
+      <c r="F16" s="21"/>
+      <c r="G16" s="21"/>
+      <c r="H16" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="I16" s="14" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="46.5">
+      <c r="A17" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B17" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="C17" s="33"/>
+      <c r="D17" s="33"/>
+      <c r="E17" s="33"/>
+      <c r="F17" s="21"/>
+      <c r="G17" s="21"/>
+      <c r="H17" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="I17" s="13" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="46.5">
+      <c r="A18" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="B18" s="33" t="s">
+        <v>759</v>
+      </c>
+      <c r="C18" s="33"/>
+      <c r="D18" s="33"/>
+      <c r="E18" s="33"/>
+      <c r="F18" s="33"/>
+      <c r="G18" s="33"/>
+      <c r="H18" s="33"/>
+      <c r="I18" s="33"/>
+    </row>
+    <row r="19" spans="1:9" ht="46.5">
+      <c r="A19" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B19" s="33" t="s">
+        <v>760</v>
+      </c>
+      <c r="C19" s="33"/>
+      <c r="D19" s="33"/>
+      <c r="E19" s="33"/>
+      <c r="F19" s="33"/>
+      <c r="G19" s="33"/>
+      <c r="H19" s="33"/>
+      <c r="I19" s="33"/>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="B21" s="32" t="s">
+        <v>73</v>
+      </c>
+      <c r="C21" s="32"/>
+      <c r="D21" s="32"/>
+      <c r="E21" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="F21" s="32" t="s">
+        <v>75</v>
+      </c>
+      <c r="G21" s="32" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="46.5">
+      <c r="A22" s="32"/>
+      <c r="B22" s="15" t="s">
+        <v>761</v>
+      </c>
+      <c r="C22" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="D22" s="15" t="s">
+        <v>161</v>
+      </c>
+      <c r="E22" s="32"/>
+      <c r="F22" s="32"/>
+      <c r="G22" s="32"/>
+    </row>
+    <row r="23" spans="1:9" ht="97.5" customHeight="1">
+      <c r="A23" s="16" t="s">
+        <v>762</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>763</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="D23" s="13" t="s">
+        <v>764</v>
+      </c>
+      <c r="E23" s="13" t="s">
+        <v>765</v>
+      </c>
+      <c r="F23" s="13" t="s">
+        <v>790</v>
+      </c>
+      <c r="G23" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="46.5">
+      <c r="A24" s="16" t="s">
+        <v>766</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="D24" s="13" t="s">
+        <v>767</v>
+      </c>
+      <c r="E24" s="13" t="s">
+        <v>768</v>
+      </c>
+      <c r="F24" s="13" t="s">
+        <v>788</v>
+      </c>
+      <c r="G24" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="69.75">
+      <c r="A25" s="16" t="s">
+        <v>769</v>
+      </c>
+      <c r="B25" s="13" t="s">
+        <v>763</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="D25" s="13" t="s">
+        <v>770</v>
+      </c>
+      <c r="E25" s="13" t="s">
+        <v>771</v>
+      </c>
+      <c r="F25" s="13" t="s">
+        <v>740</v>
+      </c>
+      <c r="G25" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="46.5">
+      <c r="A26" s="16" t="s">
+        <v>772</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>763</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="D26" s="13" t="s">
+        <v>773</v>
+      </c>
+      <c r="E26" s="13" t="s">
+        <v>774</v>
+      </c>
+      <c r="F26" s="13" t="s">
+        <v>789</v>
+      </c>
+      <c r="G26" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="116.25">
+      <c r="A27" s="16" t="s">
+        <v>775</v>
+      </c>
+      <c r="B27" s="13" t="s">
+        <v>763</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="D27" s="13" t="s">
+        <v>776</v>
+      </c>
+      <c r="E27" s="13" t="s">
+        <v>777</v>
+      </c>
+      <c r="F27" s="13" t="s">
+        <v>791</v>
+      </c>
+      <c r="G27" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="116.25">
+      <c r="A28" s="16" t="s">
+        <v>778</v>
+      </c>
+      <c r="B28" s="13" t="s">
+        <v>763</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="D28" s="13" t="s">
+        <v>779</v>
+      </c>
+      <c r="E28" s="13" t="s">
+        <v>793</v>
+      </c>
+      <c r="F28" s="13" t="s">
+        <v>794</v>
+      </c>
+      <c r="G28" s="17" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9">
+      <c r="A29" s="16" t="s">
+        <v>780</v>
+      </c>
+      <c r="B29" s="13" t="s">
+        <v>763</v>
+      </c>
+      <c r="C29" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="D29" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="E29" s="13" t="s">
+        <v>781</v>
+      </c>
+      <c r="F29" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="G29" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="46.5">
+      <c r="A30" s="16" t="s">
+        <v>782</v>
+      </c>
+      <c r="B30" s="13" t="s">
+        <v>763</v>
+      </c>
+      <c r="C30" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="D30" s="13" t="s">
+        <v>783</v>
+      </c>
+      <c r="E30" s="13" t="s">
+        <v>784</v>
+      </c>
+      <c r="F30" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="G30" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" ht="93">
+      <c r="A31" s="16" t="s">
+        <v>785</v>
+      </c>
+      <c r="B31" s="13" t="s">
+        <v>763</v>
+      </c>
+      <c r="C31" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="D31" s="13" t="s">
+        <v>786</v>
+      </c>
+      <c r="E31" s="13" t="s">
+        <v>787</v>
+      </c>
+      <c r="F31" s="13" t="s">
+        <v>792</v>
+      </c>
+      <c r="G31" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="26">
+    <mergeCell ref="B17:E17"/>
+    <mergeCell ref="B18:I18"/>
+    <mergeCell ref="B19:I19"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="G21:G22"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="A13:I13"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="B16:E16"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="F5:I5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="F6:I6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="F3:I3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="F4:I4"/>
+  </mergeCells>
+  <conditionalFormatting sqref="G23:G31">
+    <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
+      <formula>"Pass"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
+      <formula>"Fail"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
+      <formula>"Block"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" sqref="G23:G31" xr:uid="{4B692064-9C1A-4960-8717-E4AA58133272}">
+      <formula1>"Pass,Fail,No run,Block"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD0DBD97-2BD1-46BE-A1EF-D9D2695D3435}">
+  <dimension ref="A1:I29"/>
+  <sheetFormatPr defaultColWidth="7.625" defaultRowHeight="23.25"/>
+  <cols>
+    <col min="1" max="1" width="19.25" style="8" customWidth="1"/>
+    <col min="2" max="3" width="17.5" style="8" customWidth="1"/>
+    <col min="4" max="4" width="40.25" style="8" customWidth="1"/>
+    <col min="5" max="5" width="28.25" style="8" customWidth="1"/>
+    <col min="6" max="6" width="14.875" style="8" customWidth="1"/>
+    <col min="7" max="8" width="12.25" style="8" customWidth="1"/>
+    <col min="9" max="9" width="16.625" style="8" customWidth="1"/>
+    <col min="10" max="16384" width="7.625" style="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="24" thickBot="1">
+      <c r="A1" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+    </row>
+    <row r="2" spans="1:9" ht="24" thickBot="1">
+      <c r="A2" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" s="28" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" s="28"/>
+    </row>
+    <row r="3" spans="1:9" ht="24" thickBot="1">
+      <c r="A3" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="29" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="29"/>
+      <c r="E3" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="29" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" s="29"/>
+      <c r="H3" s="29"/>
+      <c r="I3" s="29"/>
+    </row>
+    <row r="4" spans="1:9" ht="24" thickBot="1">
+      <c r="A4" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="30" t="s">
+        <v>795</v>
+      </c>
+      <c r="C4" s="30"/>
+      <c r="E4" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="F4" s="30" t="s">
+        <v>796</v>
+      </c>
+      <c r="G4" s="30"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="30"/>
+    </row>
+    <row r="5" spans="1:9" ht="24" thickBot="1">
+      <c r="A5" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="30" t="s">
+        <v>797</v>
+      </c>
+      <c r="C5" s="30"/>
+    </row>
+    <row r="6" spans="1:9" ht="24" thickBot="1">
+      <c r="A6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="30" t="s">
+        <v>798</v>
+      </c>
+      <c r="C6" s="30"/>
+    </row>
+    <row r="7" spans="1:9" ht="24" thickBot="1">
+      <c r="A7" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="30" t="s">
+        <v>799</v>
+      </c>
+      <c r="C7" s="30"/>
+    </row>
+    <row r="8" spans="1:9" ht="24" thickBot="1">
+      <c r="A8" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" s="30" t="s">
+        <v>800</v>
+      </c>
+      <c r="C8" s="30"/>
+    </row>
+    <row r="9" spans="1:9" ht="24" thickBot="1">
+      <c r="A9" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="B9" s="30" t="s">
+        <v>801</v>
+      </c>
+      <c r="C9" s="30"/>
+    </row>
+    <row r="10" spans="1:9" ht="24" thickBot="1">
+      <c r="A10" s="11" t="s">
+        <v>685</v>
+      </c>
+      <c r="B10" s="30" t="s">
+        <v>802</v>
+      </c>
+      <c r="C10" s="30"/>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" s="31" t="s">
+        <v>57</v>
+      </c>
+      <c r="B12" s="31"/>
+      <c r="C12" s="31"/>
+      <c r="D12" s="31"/>
+      <c r="E12" s="31"/>
+      <c r="F12" s="31"/>
+      <c r="G12" s="31"/>
+      <c r="H12" s="31"/>
+      <c r="I12" s="31"/>
+    </row>
+    <row r="14" spans="1:9" ht="46.5">
+      <c r="A14" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B14" s="33" t="s">
+        <v>803</v>
+      </c>
+      <c r="C14" s="33"/>
+      <c r="D14" s="33"/>
+      <c r="E14" s="21"/>
+      <c r="F14" s="21"/>
+      <c r="G14" s="21"/>
+      <c r="H14" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="I14" s="14" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="B15" s="33" t="s">
+        <v>804</v>
+      </c>
+      <c r="C15" s="33"/>
+      <c r="D15" s="33"/>
+      <c r="E15" s="21"/>
+      <c r="F15" s="21"/>
+      <c r="G15" s="21"/>
+      <c r="H15" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="I15" s="14" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="46.5">
+      <c r="A16" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B16" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="C16" s="33"/>
+      <c r="D16" s="33"/>
+      <c r="E16" s="21"/>
+      <c r="F16" s="21"/>
+      <c r="G16" s="21"/>
+      <c r="H16" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="I16" s="13" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="46.5">
+      <c r="A17" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="B17" s="33" t="s">
+        <v>805</v>
+      </c>
+      <c r="C17" s="33"/>
+      <c r="D17" s="33"/>
+      <c r="E17" s="33"/>
+      <c r="F17" s="33"/>
+      <c r="G17" s="33"/>
+      <c r="H17" s="33"/>
+      <c r="I17" s="33"/>
+    </row>
+    <row r="18" spans="1:9" ht="46.5">
+      <c r="A18" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B18" s="33" t="s">
+        <v>832</v>
+      </c>
+      <c r="C18" s="33"/>
+      <c r="D18" s="33"/>
+      <c r="E18" s="33"/>
+      <c r="F18" s="33"/>
+      <c r="G18" s="33"/>
+      <c r="H18" s="33"/>
+      <c r="I18" s="33"/>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="B20" s="32" t="s">
+        <v>73</v>
+      </c>
+      <c r="C20" s="32"/>
+      <c r="D20" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="E20" s="32" t="s">
+        <v>75</v>
+      </c>
+      <c r="F20" s="32" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" s="32"/>
+      <c r="B21" s="15" t="s">
+        <v>806</v>
+      </c>
+      <c r="C21" s="15" t="s">
+        <v>807</v>
+      </c>
+      <c r="D21" s="32"/>
+      <c r="E21" s="32"/>
+      <c r="F21" s="32"/>
+    </row>
+    <row r="22" spans="1:9" ht="116.25">
+      <c r="A22" s="16" t="s">
+        <v>808</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>809</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>810</v>
+      </c>
+      <c r="D22" s="13" t="s">
+        <v>811</v>
+      </c>
+      <c r="E22" s="13" t="s">
+        <v>838</v>
+      </c>
+      <c r="F22" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="99" customHeight="1">
+      <c r="A23" s="16" t="s">
+        <v>812</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>813</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>810</v>
+      </c>
+      <c r="D23" s="13" t="s">
+        <v>814</v>
+      </c>
+      <c r="E23" s="13" t="s">
+        <v>837</v>
+      </c>
+      <c r="F23" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="53.25" customHeight="1">
+      <c r="A24" s="16" t="s">
+        <v>815</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>809</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>797</v>
+      </c>
+      <c r="D24" s="13" t="s">
+        <v>816</v>
+      </c>
+      <c r="E24" s="13" t="s">
+        <v>836</v>
+      </c>
+      <c r="F24" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="69.75">
+      <c r="A25" s="16" t="s">
+        <v>817</v>
+      </c>
+      <c r="B25" s="13" t="s">
+        <v>809</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>818</v>
+      </c>
+      <c r="D25" s="13" t="s">
+        <v>819</v>
+      </c>
+      <c r="E25" s="13" t="s">
+        <v>835</v>
+      </c>
+      <c r="F25" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="46.5">
+      <c r="A26" s="16" t="s">
+        <v>820</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>813</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>799</v>
+      </c>
+      <c r="D26" s="13" t="s">
+        <v>821</v>
+      </c>
+      <c r="E26" s="13" t="s">
+        <v>799</v>
+      </c>
+      <c r="F26" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="55.5" customHeight="1">
+      <c r="A27" s="16" t="s">
+        <v>822</v>
+      </c>
+      <c r="B27" s="13" t="s">
+        <v>809</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>823</v>
+      </c>
+      <c r="D27" s="13" t="s">
+        <v>824</v>
+      </c>
+      <c r="E27" s="13" t="s">
+        <v>834</v>
+      </c>
+      <c r="F27" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="93">
+      <c r="A28" s="16" t="s">
+        <v>825</v>
+      </c>
+      <c r="B28" s="13" t="s">
+        <v>826</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="D28" s="13" t="s">
+        <v>827</v>
+      </c>
+      <c r="E28" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="F28" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="93">
+      <c r="A29" s="16" t="s">
+        <v>828</v>
+      </c>
+      <c r="B29" s="13" t="s">
+        <v>829</v>
+      </c>
+      <c r="C29" s="13" t="s">
+        <v>830</v>
+      </c>
+      <c r="D29" s="13" t="s">
+        <v>831</v>
+      </c>
+      <c r="E29" s="13" t="s">
+        <v>833</v>
+      </c>
+      <c r="F29" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="23">
     <mergeCell ref="B18:I18"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="E20:E21"/>
+    <mergeCell ref="F20:F21"/>
+    <mergeCell ref="A12:I12"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="B17:I17"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B7:C7"/>
@@ -5733,7 +7610,7 @@
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="F4:I4"/>
   </mergeCells>
-  <conditionalFormatting sqref="E23:E30">
+  <conditionalFormatting sqref="F22:F29">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
@@ -5745,7 +7622,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="E23:E30" xr:uid="{63AF4BCA-D9D3-4060-939A-5EB7E4EBD518}">
+    <dataValidation type="list" allowBlank="1" sqref="F22:F29" xr:uid="{FFB14C75-2281-4BC8-BEDD-EB79111A9A0D}">
       <formula1>"Pass,Fail,No run,Block"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -5756,7 +7633,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93C8330E-079C-4579-8133-7533964AD0F3}">
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr defaultColWidth="7.625" defaultRowHeight="23.25"/>
   <cols>
     <col min="1" max="1" width="5.25" style="8" customWidth="1"/>
@@ -5959,6 +7836,37 @@
       <c r="J6" s="13"/>
       <c r="K6" s="13" t="s">
         <v>676</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="85.5" customHeight="1">
+      <c r="A7" s="17">
+        <v>6</v>
+      </c>
+      <c r="B7" s="17" t="s">
+        <v>745</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>839</v>
+      </c>
+      <c r="D7" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="E7" s="13"/>
+      <c r="F7" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="G7" s="17" t="s">
+        <v>216</v>
+      </c>
+      <c r="H7" s="17" t="s">
+        <v>444</v>
+      </c>
+      <c r="I7" s="17" t="s">
+        <v>444</v>
+      </c>
+      <c r="J7" s="13"/>
+      <c r="K7" s="13" t="s">
+        <v>840</v>
       </c>
     </row>
   </sheetData>
@@ -5980,265 +7888,265 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="24" thickBot="1">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="33"/>
-      <c r="I1" s="33"/>
-      <c r="J1" s="33"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
     </row>
     <row r="2" spans="1:10" ht="24" thickBot="1">
       <c r="A2" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="34" t="s">
+      <c r="F2" s="28" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="34"/>
+      <c r="G2" s="28"/>
     </row>
     <row r="3" spans="1:10" ht="24" thickBot="1">
       <c r="A3" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="35" t="s">
+      <c r="B3" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="35"/>
-      <c r="D3" s="35"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
       <c r="F3" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="35" t="s">
+      <c r="G3" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="35"/>
-      <c r="I3" s="35"/>
-      <c r="J3" s="35"/>
+      <c r="H3" s="29"/>
+      <c r="I3" s="29"/>
+      <c r="J3" s="29"/>
     </row>
     <row r="4" spans="1:10" ht="24" thickBot="1">
       <c r="A4" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="32" t="s">
+      <c r="B4" s="30" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="32"/>
-      <c r="D4" s="32"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
       <c r="F4" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="G4" s="32" t="s">
+      <c r="G4" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="H4" s="32"/>
-      <c r="I4" s="32"/>
-      <c r="J4" s="32"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="30"/>
+      <c r="J4" s="30"/>
     </row>
     <row r="5" spans="1:10" ht="24" thickBot="1">
       <c r="A5" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="32" t="s">
+      <c r="B5" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="C5" s="32"/>
-      <c r="D5" s="32"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
       <c r="F5" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="G5" s="32" t="s">
+      <c r="G5" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="H5" s="32"/>
-      <c r="I5" s="32"/>
-      <c r="J5" s="32"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+      <c r="J5" s="30"/>
     </row>
     <row r="6" spans="1:10" ht="24" thickBot="1">
       <c r="A6" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="32" t="s">
+      <c r="B6" s="30" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="32"/>
-      <c r="D6" s="32"/>
+      <c r="C6" s="30"/>
+      <c r="D6" s="30"/>
       <c r="F6" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="G6" s="32" t="s">
+      <c r="G6" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="H6" s="32"/>
-      <c r="I6" s="32"/>
-      <c r="J6" s="32"/>
+      <c r="H6" s="30"/>
+      <c r="I6" s="30"/>
+      <c r="J6" s="30"/>
     </row>
     <row r="7" spans="1:10" ht="24" thickBot="1">
       <c r="A7" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="32" t="s">
+      <c r="B7" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="32"/>
-      <c r="D7" s="32"/>
+      <c r="C7" s="30"/>
+      <c r="D7" s="30"/>
       <c r="F7" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="G7" s="32" t="s">
+      <c r="G7" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="H7" s="32"/>
-      <c r="I7" s="32"/>
-      <c r="J7" s="32"/>
+      <c r="H7" s="30"/>
+      <c r="I7" s="30"/>
+      <c r="J7" s="30"/>
     </row>
     <row r="8" spans="1:10" ht="24" thickBot="1">
       <c r="A8" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="32" t="s">
+      <c r="B8" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="C8" s="32"/>
-      <c r="D8" s="32"/>
+      <c r="C8" s="30"/>
+      <c r="D8" s="30"/>
       <c r="F8" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="G8" s="32" t="s">
+      <c r="G8" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="H8" s="32"/>
-      <c r="I8" s="32"/>
-      <c r="J8" s="32"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="30"/>
+      <c r="J8" s="30"/>
     </row>
     <row r="9" spans="1:10" ht="24" thickBot="1">
       <c r="A9" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="B9" s="32" t="s">
+      <c r="B9" s="30" t="s">
         <v>40</v>
       </c>
-      <c r="C9" s="32"/>
-      <c r="D9" s="32"/>
+      <c r="C9" s="30"/>
+      <c r="D9" s="30"/>
       <c r="F9" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="G9" s="32" t="s">
+      <c r="G9" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="H9" s="32"/>
-      <c r="I9" s="32"/>
-      <c r="J9" s="32"/>
+      <c r="H9" s="30"/>
+      <c r="I9" s="30"/>
+      <c r="J9" s="30"/>
     </row>
     <row r="10" spans="1:10" ht="24" thickBot="1">
       <c r="F10" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="G10" s="32" t="s">
+      <c r="G10" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="H10" s="32"/>
-      <c r="I10" s="32"/>
-      <c r="J10" s="32"/>
+      <c r="H10" s="30"/>
+      <c r="I10" s="30"/>
+      <c r="J10" s="30"/>
     </row>
     <row r="11" spans="1:10" ht="24" thickBot="1">
       <c r="F11" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="G11" s="32" t="s">
+      <c r="G11" s="30" t="s">
         <v>46</v>
       </c>
-      <c r="H11" s="32"/>
-      <c r="I11" s="32"/>
-      <c r="J11" s="32"/>
+      <c r="H11" s="30"/>
+      <c r="I11" s="30"/>
+      <c r="J11" s="30"/>
     </row>
     <row r="12" spans="1:10" ht="24" thickBot="1">
       <c r="F12" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="G12" s="32" t="s">
+      <c r="G12" s="30" t="s">
         <v>48</v>
       </c>
-      <c r="H12" s="32"/>
-      <c r="I12" s="32"/>
-      <c r="J12" s="32"/>
+      <c r="H12" s="30"/>
+      <c r="I12" s="30"/>
+      <c r="J12" s="30"/>
     </row>
     <row r="13" spans="1:10" ht="24" thickBot="1">
       <c r="F13" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="G13" s="32" t="s">
+      <c r="G13" s="30" t="s">
         <v>50</v>
       </c>
-      <c r="H13" s="32"/>
-      <c r="I13" s="32"/>
-      <c r="J13" s="32"/>
+      <c r="H13" s="30"/>
+      <c r="I13" s="30"/>
+      <c r="J13" s="30"/>
     </row>
     <row r="14" spans="1:10" ht="24" thickBot="1">
       <c r="F14" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="G14" s="32" t="s">
+      <c r="G14" s="30" t="s">
         <v>52</v>
       </c>
-      <c r="H14" s="32"/>
-      <c r="I14" s="32"/>
-      <c r="J14" s="32"/>
+      <c r="H14" s="30"/>
+      <c r="I14" s="30"/>
+      <c r="J14" s="30"/>
     </row>
     <row r="15" spans="1:10" ht="24" thickBot="1">
       <c r="F15" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="G15" s="32" t="s">
+      <c r="G15" s="30" t="s">
         <v>54</v>
       </c>
-      <c r="H15" s="32"/>
-      <c r="I15" s="32"/>
-      <c r="J15" s="32"/>
+      <c r="H15" s="30"/>
+      <c r="I15" s="30"/>
+      <c r="J15" s="30"/>
     </row>
     <row r="16" spans="1:10" ht="24" thickBot="1">
       <c r="F16" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="G16" s="32" t="s">
+      <c r="G16" s="30" t="s">
         <v>56</v>
       </c>
-      <c r="H16" s="32"/>
-      <c r="I16" s="32"/>
-      <c r="J16" s="32"/>
+      <c r="H16" s="30"/>
+      <c r="I16" s="30"/>
+      <c r="J16" s="30"/>
     </row>
     <row r="18" spans="1:10">
-      <c r="A18" s="27" t="s">
+      <c r="A18" s="31" t="s">
         <v>57</v>
       </c>
-      <c r="B18" s="27"/>
-      <c r="C18" s="27"/>
-      <c r="D18" s="27"/>
-      <c r="E18" s="27"/>
-      <c r="F18" s="27"/>
-      <c r="G18" s="27"/>
-      <c r="H18" s="27"/>
-      <c r="I18" s="27"/>
-      <c r="J18" s="27"/>
+      <c r="B18" s="31"/>
+      <c r="C18" s="31"/>
+      <c r="D18" s="31"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="31"/>
+      <c r="G18" s="31"/>
+      <c r="H18" s="31"/>
+      <c r="I18" s="31"/>
+      <c r="J18" s="31"/>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="B20" s="24" t="s">
+      <c r="B20" s="33" t="s">
         <v>59</v>
       </c>
-      <c r="C20" s="24"/>
-      <c r="D20" s="24"/>
-      <c r="E20" s="24"/>
-      <c r="F20" s="24"/>
-      <c r="G20" s="24"/>
-      <c r="H20" s="24"/>
+      <c r="C20" s="33"/>
+      <c r="D20" s="33"/>
+      <c r="E20" s="33"/>
+      <c r="F20" s="33"/>
+      <c r="G20" s="33"/>
+      <c r="H20" s="33"/>
       <c r="I20" s="12" t="s">
         <v>60</v>
       </c>
@@ -6250,15 +8158,15 @@
       <c r="A21" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="B21" s="24" t="s">
+      <c r="B21" s="33" t="s">
         <v>62</v>
       </c>
-      <c r="C21" s="24"/>
-      <c r="D21" s="24"/>
-      <c r="E21" s="24"/>
-      <c r="F21" s="24"/>
-      <c r="G21" s="24"/>
-      <c r="H21" s="24"/>
+      <c r="C21" s="33"/>
+      <c r="D21" s="33"/>
+      <c r="E21" s="33"/>
+      <c r="F21" s="33"/>
+      <c r="G21" s="33"/>
+      <c r="H21" s="33"/>
       <c r="I21" s="12" t="s">
         <v>63</v>
       </c>
@@ -6270,15 +8178,15 @@
       <c r="A22" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="B22" s="24" t="s">
+      <c r="B22" s="33" t="s">
         <v>65</v>
       </c>
-      <c r="C22" s="24"/>
-      <c r="D22" s="24"/>
-      <c r="E22" s="24"/>
-      <c r="F22" s="24"/>
-      <c r="G22" s="24"/>
-      <c r="H22" s="24"/>
+      <c r="C22" s="33"/>
+      <c r="D22" s="33"/>
+      <c r="E22" s="33"/>
+      <c r="F22" s="33"/>
+      <c r="G22" s="33"/>
+      <c r="H22" s="33"/>
       <c r="I22" s="12" t="s">
         <v>66</v>
       </c>
@@ -6290,58 +8198,58 @@
       <c r="A23" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="B23" s="24" t="s">
+      <c r="B23" s="33" t="s">
         <v>69</v>
       </c>
-      <c r="C23" s="24"/>
-      <c r="D23" s="24"/>
-      <c r="E23" s="24"/>
-      <c r="F23" s="24"/>
-      <c r="G23" s="24"/>
-      <c r="H23" s="24"/>
-      <c r="I23" s="24"/>
-      <c r="J23" s="24"/>
+      <c r="C23" s="33"/>
+      <c r="D23" s="33"/>
+      <c r="E23" s="33"/>
+      <c r="F23" s="33"/>
+      <c r="G23" s="33"/>
+      <c r="H23" s="33"/>
+      <c r="I23" s="33"/>
+      <c r="J23" s="33"/>
     </row>
     <row r="24" spans="1:10" ht="46.5">
       <c r="A24" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="B24" s="24" t="s">
+      <c r="B24" s="33" t="s">
         <v>71</v>
       </c>
-      <c r="C24" s="24"/>
-      <c r="D24" s="24"/>
-      <c r="E24" s="24"/>
-      <c r="F24" s="24"/>
-      <c r="G24" s="24"/>
-      <c r="H24" s="24"/>
-      <c r="I24" s="24"/>
-      <c r="J24" s="24"/>
+      <c r="C24" s="33"/>
+      <c r="D24" s="33"/>
+      <c r="E24" s="33"/>
+      <c r="F24" s="33"/>
+      <c r="G24" s="33"/>
+      <c r="H24" s="33"/>
+      <c r="I24" s="33"/>
+      <c r="J24" s="33"/>
     </row>
     <row r="26" spans="1:10">
-      <c r="A26" s="28" t="s">
+      <c r="A26" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="B26" s="28" t="s">
+      <c r="B26" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="C26" s="28"/>
-      <c r="D26" s="28"/>
-      <c r="E26" s="28"/>
-      <c r="F26" s="28"/>
-      <c r="G26" s="28"/>
-      <c r="H26" s="28" t="s">
+      <c r="C26" s="32"/>
+      <c r="D26" s="32"/>
+      <c r="E26" s="32"/>
+      <c r="F26" s="32"/>
+      <c r="G26" s="32"/>
+      <c r="H26" s="32" t="s">
         <v>74</v>
       </c>
-      <c r="I26" s="28" t="s">
+      <c r="I26" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="J26" s="28" t="s">
+      <c r="J26" s="32" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="46.5">
-      <c r="A27" s="28"/>
+      <c r="A27" s="32"/>
       <c r="B27" s="15" t="s">
         <v>77</v>
       </c>
@@ -6360,9 +8268,9 @@
       <c r="G27" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="H27" s="28"/>
-      <c r="I27" s="28"/>
-      <c r="J27" s="28"/>
+      <c r="H27" s="32"/>
+      <c r="I27" s="32"/>
+      <c r="J27" s="32"/>
     </row>
     <row r="28" spans="1:10" ht="162.75">
       <c r="A28" s="16" t="s">
@@ -6846,18 +8754,16 @@
     </row>
   </sheetData>
   <mergeCells count="34">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="G3:J3"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="G4:J4"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="G5:J5"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="G6:J6"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="G7:J7"/>
+    <mergeCell ref="B20:H20"/>
+    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="B22:H22"/>
+    <mergeCell ref="B23:J23"/>
+    <mergeCell ref="B24:J24"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="B26:G26"/>
+    <mergeCell ref="H26:H27"/>
+    <mergeCell ref="I26:I27"/>
+    <mergeCell ref="J26:J27"/>
     <mergeCell ref="A18:J18"/>
     <mergeCell ref="B8:D8"/>
     <mergeCell ref="G8:J8"/>
@@ -6870,25 +8776,27 @@
     <mergeCell ref="G14:J14"/>
     <mergeCell ref="G15:J15"/>
     <mergeCell ref="G16:J16"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="B26:G26"/>
-    <mergeCell ref="H26:H27"/>
-    <mergeCell ref="I26:I27"/>
-    <mergeCell ref="J26:J27"/>
-    <mergeCell ref="B20:H20"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="B22:H22"/>
-    <mergeCell ref="B23:J23"/>
-    <mergeCell ref="B24:J24"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="G5:J5"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="G6:J6"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="G7:J7"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="G3:J3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="G4:J4"/>
   </mergeCells>
   <conditionalFormatting sqref="J28:J42">
-    <cfRule type="cellIs" dxfId="29" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="35" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="34" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="27" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="33" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7269,42 +9177,42 @@
       <c r="I16" s="17"/>
     </row>
     <row r="17" spans="1:9">
-      <c r="A17" s="26" t="s">
+      <c r="A17" s="34" t="s">
         <v>152</v>
       </c>
-      <c r="B17" s="26"/>
-      <c r="C17" s="26"/>
-      <c r="D17" s="26"/>
-      <c r="E17" s="26"/>
-      <c r="F17" s="26"/>
-      <c r="G17" s="26"/>
-      <c r="H17" s="26"/>
-      <c r="I17" s="26"/>
+      <c r="B17" s="34"/>
+      <c r="C17" s="34"/>
+      <c r="D17" s="34"/>
+      <c r="E17" s="34"/>
+      <c r="F17" s="34"/>
+      <c r="G17" s="34"/>
+      <c r="H17" s="34"/>
+      <c r="I17" s="34"/>
     </row>
     <row r="19" spans="1:9">
-      <c r="A19" s="27" t="s">
+      <c r="A19" s="31" t="s">
         <v>57</v>
       </c>
-      <c r="B19" s="27"/>
-      <c r="C19" s="27"/>
-      <c r="D19" s="27"/>
-      <c r="E19" s="27"/>
-      <c r="F19" s="27"/>
-      <c r="G19" s="27"/>
-      <c r="H19" s="27"/>
-      <c r="I19" s="27"/>
+      <c r="B19" s="31"/>
+      <c r="C19" s="31"/>
+      <c r="D19" s="31"/>
+      <c r="E19" s="31"/>
+      <c r="F19" s="31"/>
+      <c r="G19" s="31"/>
+      <c r="H19" s="31"/>
+      <c r="I19" s="31"/>
     </row>
     <row r="21" spans="1:9" ht="46.5">
       <c r="A21" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="B21" s="24" t="s">
+      <c r="B21" s="33" t="s">
         <v>153</v>
       </c>
-      <c r="C21" s="24"/>
-      <c r="D21" s="24"/>
-      <c r="E21" s="24"/>
-      <c r="F21" s="24"/>
+      <c r="C21" s="33"/>
+      <c r="D21" s="33"/>
+      <c r="E21" s="33"/>
+      <c r="F21" s="33"/>
       <c r="G21" s="21"/>
       <c r="H21" s="12" t="s">
         <v>60</v>
@@ -7317,13 +9225,13 @@
       <c r="A22" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="B22" s="24" t="s">
+      <c r="B22" s="33" t="s">
         <v>155</v>
       </c>
-      <c r="C22" s="24"/>
-      <c r="D22" s="24"/>
-      <c r="E22" s="24"/>
-      <c r="F22" s="24"/>
+      <c r="C22" s="33"/>
+      <c r="D22" s="33"/>
+      <c r="E22" s="33"/>
+      <c r="F22" s="33"/>
       <c r="G22" s="21"/>
       <c r="H22" s="12" t="s">
         <v>63</v>
@@ -7336,13 +9244,13 @@
       <c r="A23" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="B23" s="36" t="s">
+      <c r="B23" s="35" t="s">
         <v>65</v>
       </c>
-      <c r="C23" s="37"/>
-      <c r="D23" s="37"/>
-      <c r="E23" s="37"/>
-      <c r="F23" s="38"/>
+      <c r="C23" s="36"/>
+      <c r="D23" s="36"/>
+      <c r="E23" s="36"/>
+      <c r="F23" s="37"/>
       <c r="G23" s="21"/>
       <c r="H23" s="12" t="s">
         <v>66</v>
@@ -7355,57 +9263,57 @@
       <c r="A24" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="B24" s="24" t="s">
+      <c r="B24" s="33" t="s">
         <v>157</v>
       </c>
-      <c r="C24" s="24"/>
-      <c r="D24" s="24"/>
-      <c r="E24" s="24"/>
-      <c r="F24" s="24"/>
-      <c r="G24" s="24"/>
-      <c r="H24" s="24"/>
-      <c r="I24" s="24"/>
+      <c r="C24" s="33"/>
+      <c r="D24" s="33"/>
+      <c r="E24" s="33"/>
+      <c r="F24" s="33"/>
+      <c r="G24" s="33"/>
+      <c r="H24" s="33"/>
+      <c r="I24" s="33"/>
     </row>
     <row r="25" spans="1:9">
       <c r="A25" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="B25" s="24" t="s">
+      <c r="B25" s="33" t="s">
         <v>158</v>
       </c>
-      <c r="C25" s="24"/>
-      <c r="D25" s="24"/>
-      <c r="E25" s="24"/>
-      <c r="F25" s="24"/>
-      <c r="G25" s="24"/>
-      <c r="H25" s="24"/>
-      <c r="I25" s="24"/>
+      <c r="C25" s="33"/>
+      <c r="D25" s="33"/>
+      <c r="E25" s="33"/>
+      <c r="F25" s="33"/>
+      <c r="G25" s="33"/>
+      <c r="H25" s="33"/>
+      <c r="I25" s="33"/>
     </row>
     <row r="27" spans="1:9">
-      <c r="A27" s="28" t="s">
+      <c r="A27" s="32" t="s">
         <v>159</v>
       </c>
-      <c r="B27" s="28" t="s">
+      <c r="B27" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="C27" s="28" t="s">
+      <c r="C27" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="D27" s="28"/>
-      <c r="E27" s="28"/>
-      <c r="F27" s="28" t="s">
+      <c r="D27" s="32"/>
+      <c r="E27" s="32"/>
+      <c r="F27" s="32" t="s">
         <v>74</v>
       </c>
-      <c r="G27" s="28" t="s">
+      <c r="G27" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="H27" s="28" t="s">
+      <c r="H27" s="32" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="28" spans="1:9" ht="46.5">
-      <c r="A28" s="28"/>
-      <c r="B28" s="28"/>
+      <c r="A28" s="32"/>
+      <c r="B28" s="32"/>
       <c r="C28" s="15" t="s">
         <v>81</v>
       </c>
@@ -7415,9 +9323,9 @@
       <c r="E28" s="15" t="s">
         <v>161</v>
       </c>
-      <c r="F28" s="28"/>
-      <c r="G28" s="28"/>
-      <c r="H28" s="28"/>
+      <c r="F28" s="32"/>
+      <c r="G28" s="32"/>
+      <c r="H28" s="32"/>
     </row>
     <row r="29" spans="1:9" ht="69.75">
       <c r="A29" s="17" t="s">
@@ -7681,6 +9589,12 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="B24:I24"/>
+    <mergeCell ref="A17:I17"/>
+    <mergeCell ref="A19:I19"/>
+    <mergeCell ref="B21:F21"/>
+    <mergeCell ref="B22:F22"/>
+    <mergeCell ref="B23:F23"/>
     <mergeCell ref="B25:I25"/>
     <mergeCell ref="A27:A28"/>
     <mergeCell ref="B27:B28"/>
@@ -7688,21 +9602,15 @@
     <mergeCell ref="F27:F28"/>
     <mergeCell ref="G27:G28"/>
     <mergeCell ref="H27:H28"/>
-    <mergeCell ref="B24:I24"/>
-    <mergeCell ref="A17:I17"/>
-    <mergeCell ref="A19:I19"/>
-    <mergeCell ref="B21:F21"/>
-    <mergeCell ref="B22:F22"/>
-    <mergeCell ref="B23:F23"/>
   </mergeCells>
   <conditionalFormatting sqref="H29:H38">
-    <cfRule type="cellIs" dxfId="26" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="32" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="31" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="30" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7733,15 +9641,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="46.5">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="31" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
       <c r="J1" s="13"/>
       <c r="K1" s="15" t="s">
         <v>222</v>
@@ -7765,12 +9673,12 @@
       <c r="A3" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="B3" s="24" t="s">
+      <c r="B3" s="33" t="s">
         <v>227</v>
       </c>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="24"/>
+      <c r="C3" s="33"/>
+      <c r="D3" s="33"/>
+      <c r="E3" s="33"/>
       <c r="F3" s="12" t="s">
         <v>60</v>
       </c>
@@ -7791,12 +9699,12 @@
       <c r="A4" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="B4" s="24" t="s">
+      <c r="B4" s="33" t="s">
         <v>231</v>
       </c>
-      <c r="C4" s="24"/>
-      <c r="D4" s="24"/>
-      <c r="E4" s="24"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="33"/>
       <c r="F4" s="12" t="s">
         <v>63</v>
       </c>
@@ -7817,12 +9725,12 @@
       <c r="A5" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="B5" s="24" t="s">
+      <c r="B5" s="33" t="s">
         <v>65</v>
       </c>
-      <c r="C5" s="24"/>
-      <c r="D5" s="24"/>
-      <c r="E5" s="24"/>
+      <c r="C5" s="33"/>
+      <c r="D5" s="33"/>
+      <c r="E5" s="33"/>
       <c r="F5" s="12" t="s">
         <v>66</v>
       </c>
@@ -7843,14 +9751,14 @@
       <c r="A6" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="33" t="s">
         <v>237</v>
       </c>
-      <c r="C6" s="24"/>
-      <c r="D6" s="24"/>
-      <c r="E6" s="24"/>
-      <c r="F6" s="24"/>
-      <c r="G6" s="24"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
+      <c r="F6" s="33"/>
+      <c r="G6" s="33"/>
       <c r="J6" s="17" t="s">
         <v>238</v>
       </c>
@@ -7865,14 +9773,14 @@
       <c r="A7" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="B7" s="24" t="s">
+      <c r="B7" s="33" t="s">
         <v>243</v>
       </c>
-      <c r="C7" s="24"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24"/>
-      <c r="F7" s="24"/>
-      <c r="G7" s="24"/>
+      <c r="C7" s="33"/>
+      <c r="D7" s="33"/>
+      <c r="E7" s="33"/>
+      <c r="F7" s="33"/>
+      <c r="G7" s="33"/>
       <c r="J7" s="17" t="s">
         <v>244</v>
       </c>
@@ -7884,26 +9792,26 @@
       </c>
     </row>
     <row r="9" spans="1:12">
-      <c r="A9" s="28" t="s">
+      <c r="A9" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="B9" s="28" t="s">
+      <c r="B9" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="C9" s="28"/>
-      <c r="D9" s="28"/>
-      <c r="E9" s="28" t="s">
+      <c r="C9" s="32"/>
+      <c r="D9" s="32"/>
+      <c r="E9" s="32" t="s">
         <v>74</v>
       </c>
-      <c r="F9" s="28" t="s">
+      <c r="F9" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="G9" s="28" t="s">
+      <c r="G9" s="32" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="10" spans="1:12">
-      <c r="A10" s="28"/>
+      <c r="A10" s="32"/>
       <c r="B10" s="15" t="s">
         <v>82</v>
       </c>
@@ -7913,9 +9821,9 @@
       <c r="D10" s="15" t="s">
         <v>248</v>
       </c>
-      <c r="E10" s="28"/>
-      <c r="F10" s="28"/>
-      <c r="G10" s="28"/>
+      <c r="E10" s="32"/>
+      <c r="F10" s="32"/>
+      <c r="G10" s="32"/>
     </row>
     <row r="11" spans="1:12" ht="46.5">
       <c r="A11" s="16" t="s">
@@ -8218,26 +10126,26 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="B6:G6"/>
     <mergeCell ref="B7:G7"/>
     <mergeCell ref="A9:A10"/>
     <mergeCell ref="B9:D9"/>
     <mergeCell ref="E9:E10"/>
     <mergeCell ref="F9:F10"/>
     <mergeCell ref="G9:G10"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="B6:G6"/>
   </mergeCells>
   <conditionalFormatting sqref="G11:G23">
-    <cfRule type="cellIs" dxfId="23" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="29" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="28" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="27" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8268,16 +10176,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="69.75">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="31" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
       <c r="K1" s="13"/>
       <c r="L1" s="15" t="s">
         <v>298</v>
@@ -8313,13 +10221,13 @@
       <c r="A3" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="B3" s="24" t="s">
+      <c r="B3" s="33" t="s">
         <v>305</v>
       </c>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="24"/>
-      <c r="F3" s="24"/>
+      <c r="C3" s="33"/>
+      <c r="D3" s="33"/>
+      <c r="E3" s="33"/>
+      <c r="F3" s="33"/>
       <c r="G3" s="12" t="s">
         <v>60</v>
       </c>
@@ -8346,13 +10254,13 @@
       <c r="A4" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="B4" s="24" t="s">
+      <c r="B4" s="33" t="s">
         <v>309</v>
       </c>
-      <c r="C4" s="24"/>
-      <c r="D4" s="24"/>
-      <c r="E4" s="24"/>
-      <c r="F4" s="24"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="33"/>
+      <c r="F4" s="33"/>
       <c r="G4" s="12" t="s">
         <v>63</v>
       </c>
@@ -8379,13 +10287,13 @@
       <c r="A5" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="B5" s="24" t="s">
+      <c r="B5" s="33" t="s">
         <v>65</v>
       </c>
-      <c r="C5" s="24"/>
-      <c r="D5" s="24"/>
-      <c r="E5" s="24"/>
-      <c r="F5" s="24"/>
+      <c r="C5" s="33"/>
+      <c r="D5" s="33"/>
+      <c r="E5" s="33"/>
+      <c r="F5" s="33"/>
       <c r="G5" s="12" t="s">
         <v>66</v>
       </c>
@@ -8412,52 +10320,52 @@
       <c r="A6" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="33" t="s">
         <v>313</v>
       </c>
-      <c r="C6" s="24"/>
-      <c r="D6" s="24"/>
-      <c r="E6" s="24"/>
-      <c r="F6" s="24"/>
-      <c r="G6" s="24"/>
-      <c r="H6" s="24"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
+      <c r="F6" s="33"/>
+      <c r="G6" s="33"/>
+      <c r="H6" s="33"/>
     </row>
     <row r="7" spans="1:15" ht="46.5">
       <c r="A7" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="B7" s="24" t="s">
+      <c r="B7" s="33" t="s">
         <v>449</v>
       </c>
-      <c r="C7" s="24"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24"/>
-      <c r="F7" s="24"/>
-      <c r="G7" s="24"/>
-      <c r="H7" s="24"/>
+      <c r="C7" s="33"/>
+      <c r="D7" s="33"/>
+      <c r="E7" s="33"/>
+      <c r="F7" s="33"/>
+      <c r="G7" s="33"/>
+      <c r="H7" s="33"/>
     </row>
     <row r="9" spans="1:15">
-      <c r="A9" s="28" t="s">
+      <c r="A9" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="B9" s="28" t="s">
+      <c r="B9" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="C9" s="28"/>
-      <c r="D9" s="28"/>
-      <c r="E9" s="28"/>
-      <c r="F9" s="28" t="s">
+      <c r="C9" s="32"/>
+      <c r="D9" s="32"/>
+      <c r="E9" s="32"/>
+      <c r="F9" s="32" t="s">
         <v>74</v>
       </c>
-      <c r="G9" s="28" t="s">
+      <c r="G9" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="H9" s="28" t="s">
+      <c r="H9" s="32" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="10" spans="1:15" ht="46.5">
-      <c r="A10" s="28"/>
+      <c r="A10" s="32"/>
       <c r="B10" s="15" t="s">
         <v>314</v>
       </c>
@@ -8470,9 +10378,9 @@
       <c r="E10" s="15" t="s">
         <v>317</v>
       </c>
-      <c r="F10" s="28"/>
-      <c r="G10" s="28"/>
-      <c r="H10" s="28"/>
+      <c r="F10" s="32"/>
+      <c r="G10" s="32"/>
+      <c r="H10" s="32"/>
     </row>
     <row r="11" spans="1:15">
       <c r="A11" s="16" t="s">
@@ -8814,26 +10722,26 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B9:E9"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="G9:G10"/>
-    <mergeCell ref="H9:H10"/>
     <mergeCell ref="B7:H7"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="B6:H6"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="H9:H10"/>
   </mergeCells>
   <conditionalFormatting sqref="H11:H23">
-    <cfRule type="cellIs" dxfId="20" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="26" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="19" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="25" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="24" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8869,49 +10777,49 @@
       </c>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="38" t="s">
         <v>363</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
-      <c r="J2" s="25"/>
-      <c r="K2" s="25"/>
+      <c r="B2" s="38"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="38"/>
+      <c r="F2" s="38"/>
+      <c r="G2" s="38"/>
+      <c r="H2" s="38"/>
+      <c r="I2" s="38"/>
+      <c r="J2" s="38"/>
+      <c r="K2" s="38"/>
     </row>
     <row r="3" spans="1:11">
-      <c r="A3" s="25" t="s">
+      <c r="A3" s="38" t="s">
         <v>364</v>
       </c>
-      <c r="B3" s="25"/>
-      <c r="C3" s="25"/>
-      <c r="D3" s="25"/>
-      <c r="E3" s="25"/>
-      <c r="F3" s="25"/>
-      <c r="G3" s="25"/>
-      <c r="H3" s="25"/>
-      <c r="I3" s="25"/>
-      <c r="J3" s="25"/>
-      <c r="K3" s="25"/>
+      <c r="B3" s="38"/>
+      <c r="C3" s="38"/>
+      <c r="D3" s="38"/>
+      <c r="E3" s="38"/>
+      <c r="F3" s="38"/>
+      <c r="G3" s="38"/>
+      <c r="H3" s="38"/>
+      <c r="I3" s="38"/>
+      <c r="J3" s="38"/>
+      <c r="K3" s="38"/>
     </row>
     <row r="4" spans="1:11">
-      <c r="A4" s="25" t="s">
+      <c r="A4" s="38" t="s">
         <v>365</v>
       </c>
-      <c r="B4" s="25"/>
-      <c r="C4" s="25"/>
-      <c r="D4" s="25"/>
-      <c r="E4" s="25"/>
-      <c r="F4" s="25"/>
-      <c r="G4" s="25"/>
-      <c r="H4" s="25"/>
-      <c r="I4" s="25"/>
-      <c r="J4" s="25"/>
-      <c r="K4" s="25"/>
+      <c r="B4" s="38"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="38"/>
+      <c r="E4" s="38"/>
+      <c r="F4" s="38"/>
+      <c r="G4" s="38"/>
+      <c r="H4" s="38"/>
+      <c r="I4" s="38"/>
+      <c r="J4" s="38"/>
+      <c r="K4" s="38"/>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" s="18" t="s">
@@ -9316,47 +11224,47 @@
       <c r="K21" s="17"/>
     </row>
     <row r="22" spans="1:11">
-      <c r="A22" s="26" t="s">
+      <c r="A22" s="34" t="s">
         <v>388</v>
       </c>
-      <c r="B22" s="26"/>
-      <c r="C22" s="26"/>
-      <c r="D22" s="26"/>
-      <c r="E22" s="26"/>
-      <c r="F22" s="26"/>
-      <c r="G22" s="26"/>
-      <c r="H22" s="26"/>
-      <c r="I22" s="26"/>
-      <c r="J22" s="26"/>
-      <c r="K22" s="26"/>
+      <c r="B22" s="34"/>
+      <c r="C22" s="34"/>
+      <c r="D22" s="34"/>
+      <c r="E22" s="34"/>
+      <c r="F22" s="34"/>
+      <c r="G22" s="34"/>
+      <c r="H22" s="34"/>
+      <c r="I22" s="34"/>
+      <c r="J22" s="34"/>
+      <c r="K22" s="34"/>
     </row>
     <row r="24" spans="1:11">
-      <c r="A24" s="27" t="s">
+      <c r="A24" s="31" t="s">
         <v>57</v>
       </c>
-      <c r="B24" s="27"/>
-      <c r="C24" s="27"/>
-      <c r="D24" s="27"/>
-      <c r="E24" s="27"/>
-      <c r="F24" s="27"/>
-      <c r="G24" s="27"/>
-      <c r="H24" s="27"/>
-      <c r="I24" s="27"/>
-      <c r="J24" s="27"/>
-      <c r="K24" s="27"/>
+      <c r="B24" s="31"/>
+      <c r="C24" s="31"/>
+      <c r="D24" s="31"/>
+      <c r="E24" s="31"/>
+      <c r="F24" s="31"/>
+      <c r="G24" s="31"/>
+      <c r="H24" s="31"/>
+      <c r="I24" s="31"/>
+      <c r="J24" s="31"/>
+      <c r="K24" s="31"/>
     </row>
     <row r="26" spans="1:11" ht="46.5">
       <c r="A26" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="B26" s="24" t="s">
+      <c r="B26" s="33" t="s">
         <v>389</v>
       </c>
-      <c r="C26" s="24"/>
-      <c r="D26" s="24"/>
-      <c r="E26" s="24"/>
-      <c r="F26" s="24"/>
-      <c r="G26" s="24"/>
+      <c r="C26" s="33"/>
+      <c r="D26" s="33"/>
+      <c r="E26" s="33"/>
+      <c r="F26" s="33"/>
+      <c r="G26" s="33"/>
       <c r="H26" s="21"/>
       <c r="I26" s="21"/>
       <c r="J26" s="12" t="s">
@@ -9370,14 +11278,14 @@
       <c r="A27" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="B27" s="24" t="s">
+      <c r="B27" s="33" t="s">
         <v>390</v>
       </c>
-      <c r="C27" s="24"/>
-      <c r="D27" s="24"/>
-      <c r="E27" s="24"/>
-      <c r="F27" s="24"/>
-      <c r="G27" s="24"/>
+      <c r="C27" s="33"/>
+      <c r="D27" s="33"/>
+      <c r="E27" s="33"/>
+      <c r="F27" s="33"/>
+      <c r="G27" s="33"/>
       <c r="H27" s="21"/>
       <c r="I27" s="21"/>
       <c r="J27" s="12" t="s">
@@ -9391,14 +11299,14 @@
       <c r="A28" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="B28" s="24" t="s">
+      <c r="B28" s="33" t="s">
         <v>65</v>
       </c>
-      <c r="C28" s="24"/>
-      <c r="D28" s="24"/>
-      <c r="E28" s="24"/>
-      <c r="F28" s="24"/>
-      <c r="G28" s="24"/>
+      <c r="C28" s="33"/>
+      <c r="D28" s="33"/>
+      <c r="E28" s="33"/>
+      <c r="F28" s="33"/>
+      <c r="G28" s="33"/>
       <c r="H28" s="21"/>
       <c r="I28" s="21"/>
       <c r="J28" s="12" t="s">
@@ -9412,62 +11320,62 @@
       <c r="A29" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="B29" s="24" t="s">
+      <c r="B29" s="33" t="s">
         <v>391</v>
       </c>
-      <c r="C29" s="24"/>
-      <c r="D29" s="24"/>
-      <c r="E29" s="24"/>
-      <c r="F29" s="24"/>
-      <c r="G29" s="24"/>
-      <c r="H29" s="24"/>
-      <c r="I29" s="24"/>
-      <c r="J29" s="24"/>
-      <c r="K29" s="24"/>
+      <c r="C29" s="33"/>
+      <c r="D29" s="33"/>
+      <c r="E29" s="33"/>
+      <c r="F29" s="33"/>
+      <c r="G29" s="33"/>
+      <c r="H29" s="33"/>
+      <c r="I29" s="33"/>
+      <c r="J29" s="33"/>
+      <c r="K29" s="33"/>
     </row>
     <row r="30" spans="1:11">
       <c r="A30" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="B30" s="24" t="s">
+      <c r="B30" s="33" t="s">
         <v>448</v>
       </c>
-      <c r="C30" s="24"/>
-      <c r="D30" s="24"/>
-      <c r="E30" s="24"/>
-      <c r="F30" s="24"/>
-      <c r="G30" s="24"/>
-      <c r="H30" s="24"/>
-      <c r="I30" s="24"/>
-      <c r="J30" s="24"/>
-      <c r="K30" s="24"/>
+      <c r="C30" s="33"/>
+      <c r="D30" s="33"/>
+      <c r="E30" s="33"/>
+      <c r="F30" s="33"/>
+      <c r="G30" s="33"/>
+      <c r="H30" s="33"/>
+      <c r="I30" s="33"/>
+      <c r="J30" s="33"/>
+      <c r="K30" s="33"/>
     </row>
     <row r="32" spans="1:11">
-      <c r="A32" s="28" t="s">
+      <c r="A32" s="32" t="s">
         <v>159</v>
       </c>
-      <c r="B32" s="28" t="s">
+      <c r="B32" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="C32" s="28" t="s">
+      <c r="C32" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="D32" s="28"/>
-      <c r="E32" s="28"/>
-      <c r="F32" s="28"/>
-      <c r="G32" s="28" t="s">
+      <c r="D32" s="32"/>
+      <c r="E32" s="32"/>
+      <c r="F32" s="32"/>
+      <c r="G32" s="32" t="s">
         <v>74</v>
       </c>
-      <c r="H32" s="28" t="s">
+      <c r="H32" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="I32" s="28" t="s">
+      <c r="I32" s="32" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="33" spans="1:9" ht="46.5">
-      <c r="A33" s="28"/>
-      <c r="B33" s="28"/>
+      <c r="A33" s="32"/>
+      <c r="B33" s="32"/>
       <c r="C33" s="15" t="s">
         <v>392</v>
       </c>
@@ -9480,9 +11388,9 @@
       <c r="F33" s="15" t="s">
         <v>394</v>
       </c>
-      <c r="G33" s="28"/>
-      <c r="H33" s="28"/>
-      <c r="I33" s="28"/>
+      <c r="G33" s="32"/>
+      <c r="H33" s="32"/>
+      <c r="I33" s="32"/>
     </row>
     <row r="34" spans="1:9" ht="46.5">
       <c r="A34" s="17" t="s">
@@ -9834,6 +11742,12 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="B26:G26"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A22:K22"/>
+    <mergeCell ref="A24:K24"/>
     <mergeCell ref="B27:G27"/>
     <mergeCell ref="B28:G28"/>
     <mergeCell ref="B29:K29"/>
@@ -9844,21 +11758,15 @@
     <mergeCell ref="G32:G33"/>
     <mergeCell ref="H32:H33"/>
     <mergeCell ref="I32:I33"/>
-    <mergeCell ref="B26:G26"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A22:K22"/>
-    <mergeCell ref="A24:K24"/>
   </mergeCells>
   <conditionalFormatting sqref="I34:I45">
-    <cfRule type="cellIs" dxfId="17" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="23" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="22" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="21" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9889,14 +11797,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="23.25" customHeight="1">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="31" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
       <c r="I1" s="13"/>
       <c r="J1" s="15" t="s">
         <v>455</v>
@@ -9914,11 +11822,11 @@
       <c r="A3" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="B3" s="24" t="s">
+      <c r="B3" s="33" t="s">
         <v>458</v>
       </c>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
+      <c r="C3" s="33"/>
+      <c r="D3" s="33"/>
       <c r="E3" s="12" t="s">
         <v>60</v>
       </c>
@@ -9936,11 +11844,11 @@
       <c r="A4" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="B4" s="24" t="s">
+      <c r="B4" s="33" t="s">
         <v>309</v>
       </c>
-      <c r="C4" s="24"/>
-      <c r="D4" s="24"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
       <c r="E4" s="12" t="s">
         <v>63</v>
       </c>
@@ -9958,11 +11866,11 @@
       <c r="A5" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="B5" s="24" t="s">
+      <c r="B5" s="33" t="s">
         <v>65</v>
       </c>
-      <c r="C5" s="24"/>
-      <c r="D5" s="24"/>
+      <c r="C5" s="33"/>
+      <c r="D5" s="33"/>
       <c r="E5" s="12" t="s">
         <v>66</v>
       </c>
@@ -9980,13 +11888,13 @@
       <c r="A6" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="33" t="s">
         <v>477</v>
       </c>
-      <c r="C6" s="24"/>
-      <c r="D6" s="24"/>
-      <c r="E6" s="24"/>
-      <c r="F6" s="24"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
+      <c r="F6" s="33"/>
       <c r="I6" s="17" t="s">
         <v>234</v>
       </c>
@@ -9998,43 +11906,43 @@
       <c r="A7" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="B7" s="24" t="s">
+      <c r="B7" s="33" t="s">
         <v>462</v>
       </c>
-      <c r="C7" s="24"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24"/>
-      <c r="F7" s="24"/>
+      <c r="C7" s="33"/>
+      <c r="D7" s="33"/>
+      <c r="E7" s="33"/>
+      <c r="F7" s="33"/>
     </row>
     <row r="9" spans="1:10" ht="23.25" customHeight="1">
-      <c r="A9" s="28" t="s">
+      <c r="A9" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="B9" s="28" t="s">
+      <c r="B9" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="C9" s="28"/>
-      <c r="D9" s="28" t="s">
+      <c r="C9" s="32"/>
+      <c r="D9" s="32" t="s">
         <v>74</v>
       </c>
-      <c r="E9" s="28" t="s">
+      <c r="E9" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="F9" s="28" t="s">
+      <c r="F9" s="32" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="46.5">
-      <c r="A10" s="28"/>
+      <c r="A10" s="32"/>
       <c r="B10" s="15" t="s">
         <v>463</v>
       </c>
       <c r="C10" s="15" t="s">
         <v>455</v>
       </c>
-      <c r="D10" s="28"/>
-      <c r="E10" s="28"/>
-      <c r="F10" s="28"/>
+      <c r="D10" s="32"/>
+      <c r="E10" s="32"/>
+      <c r="F10" s="32"/>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" s="16" t="s">
@@ -10138,26 +12046,26 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B6:F6"/>
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="A9:A10"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="D9:D10"/>
     <mergeCell ref="E9:E10"/>
     <mergeCell ref="F9:F10"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B6:F6"/>
   </mergeCells>
   <conditionalFormatting sqref="F11:F15">
-    <cfRule type="cellIs" dxfId="11" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="20" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="18" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10429,39 +12337,39 @@
       <c r="H12" s="17"/>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" s="26" t="s">
+      <c r="A13" s="34" t="s">
         <v>483</v>
       </c>
-      <c r="B13" s="26"/>
-      <c r="C13" s="26"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="26"/>
-      <c r="F13" s="26"/>
-      <c r="G13" s="26"/>
-      <c r="H13" s="26"/>
+      <c r="B13" s="34"/>
+      <c r="C13" s="34"/>
+      <c r="D13" s="34"/>
+      <c r="E13" s="34"/>
+      <c r="F13" s="34"/>
+      <c r="G13" s="34"/>
+      <c r="H13" s="34"/>
     </row>
     <row r="15" spans="1:8">
-      <c r="A15" s="27" t="s">
+      <c r="A15" s="31" t="s">
         <v>57</v>
       </c>
-      <c r="B15" s="27"/>
-      <c r="C15" s="27"/>
-      <c r="D15" s="27"/>
-      <c r="E15" s="27"/>
-      <c r="F15" s="27"/>
-      <c r="G15" s="27"/>
-      <c r="H15" s="27"/>
-    </row>
-    <row r="17" spans="1:8" ht="46.5">
+      <c r="B15" s="31"/>
+      <c r="C15" s="31"/>
+      <c r="D15" s="31"/>
+      <c r="E15" s="31"/>
+      <c r="F15" s="31"/>
+      <c r="G15" s="31"/>
+      <c r="H15" s="31"/>
+    </row>
+    <row r="17" spans="1:8">
       <c r="A17" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="B17" s="24" t="s">
+      <c r="B17" s="33" t="s">
         <v>484</v>
       </c>
-      <c r="C17" s="24"/>
-      <c r="D17" s="24"/>
-      <c r="E17" s="24"/>
+      <c r="C17" s="33"/>
+      <c r="D17" s="33"/>
+      <c r="E17" s="33"/>
       <c r="F17" s="21"/>
       <c r="G17" s="12" t="s">
         <v>60</v>
@@ -10474,12 +12382,12 @@
       <c r="A18" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="B18" s="24" t="s">
+      <c r="B18" s="33" t="s">
         <v>155</v>
       </c>
-      <c r="C18" s="24"/>
-      <c r="D18" s="24"/>
-      <c r="E18" s="24"/>
+      <c r="C18" s="33"/>
+      <c r="D18" s="33"/>
+      <c r="E18" s="33"/>
       <c r="F18" s="21"/>
       <c r="G18" s="12" t="s">
         <v>63</v>
@@ -10492,12 +12400,12 @@
       <c r="A19" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="B19" s="24" t="s">
+      <c r="B19" s="33" t="s">
         <v>65</v>
       </c>
-      <c r="C19" s="24"/>
-      <c r="D19" s="24"/>
-      <c r="E19" s="24"/>
+      <c r="C19" s="33"/>
+      <c r="D19" s="33"/>
+      <c r="E19" s="33"/>
       <c r="F19" s="21"/>
       <c r="G19" s="12" t="s">
         <v>66</v>
@@ -10510,65 +12418,65 @@
       <c r="A20" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="B20" s="24" t="s">
+      <c r="B20" s="33" t="s">
         <v>485</v>
       </c>
-      <c r="C20" s="24"/>
-      <c r="D20" s="24"/>
-      <c r="E20" s="24"/>
-      <c r="F20" s="24"/>
-      <c r="G20" s="24"/>
-      <c r="H20" s="24"/>
+      <c r="C20" s="33"/>
+      <c r="D20" s="33"/>
+      <c r="E20" s="33"/>
+      <c r="F20" s="33"/>
+      <c r="G20" s="33"/>
+      <c r="H20" s="33"/>
     </row>
     <row r="21" spans="1:8">
       <c r="A21" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="B21" s="24" t="s">
+      <c r="B21" s="33" t="s">
         <v>486</v>
       </c>
-      <c r="C21" s="24"/>
-      <c r="D21" s="24"/>
-      <c r="E21" s="24"/>
-      <c r="F21" s="24"/>
-      <c r="G21" s="24"/>
-      <c r="H21" s="24"/>
+      <c r="C21" s="33"/>
+      <c r="D21" s="33"/>
+      <c r="E21" s="33"/>
+      <c r="F21" s="33"/>
+      <c r="G21" s="33"/>
+      <c r="H21" s="33"/>
     </row>
     <row r="23" spans="1:8">
-      <c r="A23" s="28" t="s">
+      <c r="A23" s="32" t="s">
         <v>159</v>
       </c>
-      <c r="B23" s="28" t="s">
+      <c r="B23" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="C23" s="28" t="s">
+      <c r="C23" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="D23" s="28"/>
-      <c r="E23" s="28" t="s">
+      <c r="D23" s="32"/>
+      <c r="E23" s="32" t="s">
         <v>74</v>
       </c>
-      <c r="F23" s="28" t="s">
+      <c r="F23" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="G23" s="28" t="s">
+      <c r="G23" s="32" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="24" spans="1:8">
-      <c r="A24" s="28"/>
-      <c r="B24" s="28"/>
+      <c r="A24" s="32"/>
+      <c r="B24" s="32"/>
       <c r="C24" s="15" t="s">
         <v>487</v>
       </c>
       <c r="D24" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="E24" s="28"/>
-      <c r="F24" s="28"/>
-      <c r="G24" s="28"/>
-    </row>
-    <row r="25" spans="1:8" ht="46.5">
+      <c r="E24" s="32"/>
+      <c r="F24" s="32"/>
+      <c r="G24" s="32"/>
+    </row>
+    <row r="25" spans="1:8">
       <c r="A25" s="17" t="s">
         <v>162</v>
       </c>
@@ -10754,6 +12662,12 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="B20:H20"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A15:H15"/>
+    <mergeCell ref="B17:E17"/>
+    <mergeCell ref="B18:E18"/>
+    <mergeCell ref="B19:E19"/>
     <mergeCell ref="B21:H21"/>
     <mergeCell ref="A23:A24"/>
     <mergeCell ref="B23:B24"/>
@@ -10761,21 +12675,15 @@
     <mergeCell ref="E23:E24"/>
     <mergeCell ref="F23:F24"/>
     <mergeCell ref="G23:G24"/>
-    <mergeCell ref="A13:H13"/>
-    <mergeCell ref="A15:H15"/>
-    <mergeCell ref="B17:E17"/>
-    <mergeCell ref="B18:E18"/>
-    <mergeCell ref="B19:E19"/>
-    <mergeCell ref="B20:H20"/>
   </mergeCells>
   <conditionalFormatting sqref="G25:G32">
-    <cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="17" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Edit Unit Test Report
</commit_message>
<xml_diff>
--- a/test/FIWDEE_UnitTest_Report.xlsx
+++ b/test/FIWDEE_UnitTest_Report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\ProjectPOS\FIWDEE-CP353002-69_1PrinciplesOfSoftwareDesign\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC37DD3C-22CA-49B2-A730-DA146FE1F5C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E9E9B8E-352F-4837-96A2-587992B4F267}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="14" activeTab="14" xr2:uid="{9B0ECA1C-B255-4EEE-B7A8-035645CFC3D9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{9B0ECA1C-B255-4EEE-B7A8-035645CFC3D9}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Summary" sheetId="1" r:id="rId1"/>
@@ -83,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2850" uniqueCount="1115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2874" uniqueCount="1123">
   <si>
     <t>FIWDEE – Unit Test Design</t>
   </si>
@@ -3428,6 +3428,30 @@
   </si>
   <si>
     <t>Payment ใหม่ COMPLETED</t>
+  </si>
+  <si>
+    <t>ชำระเงินตอน CHECKED_IN แล้ว Booking กลายเป็น COMPLETED (ข้าม IN_SERVICE)</t>
+  </si>
+  <si>
+    <t>เปลี่ยนสถานะ Booking ตอนชำระเงินแต่ไม่ publish BookingStatusChangedEvent</t>
+  </si>
+  <si>
+    <t>service/impl/PaymentServiceImpl.java (ไม่มี ApplicationEventPublisher) • ลูกค้าไม่ได้รับแจ้งเตือน (UC-07 ข้อ 13) • UT14-TC007, TC008</t>
+  </si>
+  <si>
+    <t>รับชำระเงินของ Booking ที่ CANCELLED / NO_SHOW ได้</t>
+  </si>
+  <si>
+    <t>DEF-007</t>
+  </si>
+  <si>
+    <t>DEF-008</t>
+  </si>
+  <si>
+    <t>service/impl/PaymentServiceImpl.java  ผิด BR-QUE-03 และ State diagram • ข้าม completeService() ห้องไม่เข้า CLEANING, คิวไม่ COMPLETED • ยืนยันด้วย UT14-TC009</t>
+  </si>
+  <si>
+    <t>service/impl/PaymentServiceImpl.java processPayment ไม่ตรวจสถานะ booking • ผิด SRS 7.1 (end state) • UT14-TC010, TC011</t>
   </si>
 </sst>
 </file>
@@ -12074,13 +12098,13 @@
     <mergeCell ref="F4:I4"/>
   </mergeCells>
   <conditionalFormatting sqref="F19:F26">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12096,7 +12120,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93C8330E-079C-4579-8133-7533964AD0F3}">
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr defaultColWidth="7.625" defaultRowHeight="23.25"/>
   <cols>
     <col min="1" max="1" width="5.25" style="8" customWidth="1"/>
@@ -12330,6 +12354,99 @@
       <c r="J7" s="13"/>
       <c r="K7" s="13" t="s">
         <v>840</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="69.75">
+      <c r="A8" s="17">
+        <v>7</v>
+      </c>
+      <c r="B8" s="17" t="s">
+        <v>1119</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>1115</v>
+      </c>
+      <c r="D8" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="E8" s="13"/>
+      <c r="F8" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="G8" s="17" t="s">
+        <v>216</v>
+      </c>
+      <c r="H8" s="17" t="s">
+        <v>217</v>
+      </c>
+      <c r="I8" s="17" t="s">
+        <v>217</v>
+      </c>
+      <c r="J8" s="13"/>
+      <c r="K8" s="13" t="s">
+        <v>1121</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="69.75">
+      <c r="A9" s="17">
+        <v>8</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>1120</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>1116</v>
+      </c>
+      <c r="D9" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="E9" s="13"/>
+      <c r="F9" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="G9" s="17" t="s">
+        <v>216</v>
+      </c>
+      <c r="H9" s="17" t="s">
+        <v>441</v>
+      </c>
+      <c r="I9" s="17" t="s">
+        <v>441</v>
+      </c>
+      <c r="J9" s="13"/>
+      <c r="K9" s="13" t="s">
+        <v>1117</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="46.5">
+      <c r="A10" s="17">
+        <v>9</v>
+      </c>
+      <c r="B10" s="17" t="s">
+        <v>673</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>1118</v>
+      </c>
+      <c r="D10" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="E10" s="13"/>
+      <c r="F10" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="G10" s="17" t="s">
+        <v>216</v>
+      </c>
+      <c r="H10" s="17" t="s">
+        <v>441</v>
+      </c>
+      <c r="I10" s="17" t="s">
+        <v>441</v>
+      </c>
+      <c r="J10" s="13"/>
+      <c r="K10" s="13" t="s">
+        <v>1122</v>
       </c>
     </row>
   </sheetData>
@@ -12831,13 +12948,13 @@
     <mergeCell ref="F4:I4"/>
   </mergeCells>
   <conditionalFormatting sqref="F20:F29">
-    <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Unit Test in RefundServiceImpl
</commit_message>
<xml_diff>
--- a/test/FIWDEE_UnitTest_Report.xlsx
+++ b/test/FIWDEE_UnitTest_Report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\ProjectPOS\FIWDEE-CP353002-69_1PrinciplesOfSoftwareDesign\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDC74CAF-D168-48D6-99A6-9B6A77A9C7A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88DF55BB-EC1B-4820-B5C5-AE93591DE559}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9B0ECA1C-B255-4EEE-B7A8-035645CFC3D9}"/>
   </bookViews>
@@ -33,9 +33,11 @@
     <sheet name="UT16_PercentDiscount_EC" sheetId="19" r:id="rId18"/>
     <sheet name="UT17_DiscountFactory_EC" sheetId="20" r:id="rId19"/>
     <sheet name="UT18_PaymentStrategy_EC" sheetId="21" r:id="rId20"/>
+    <sheet name="UT19_Refund_Amount_BVA" sheetId="22" r:id="rId21"/>
+    <sheet name="UT20_Refund_EC" sheetId="23" r:id="rId22"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId21"/>
+    <externalReference r:id="rId23"/>
   </externalReferences>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -83,7 +85,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2874" uniqueCount="1123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3061" uniqueCount="1201">
   <si>
     <t>FIWDEE – Unit Test Design</t>
   </si>
@@ -3452,6 +3454,240 @@
   </si>
   <si>
     <t>service/impl/PaymentServiceImpl.java processPayment ไม่ตรวจสถานะ booking • ผิด SRS 7.1 (end state) • UT14-TC010, TC011</t>
+  </si>
+  <si>
+    <t>Refund</t>
+  </si>
+  <si>
+    <t>UT19 – RefundServiceImpl.processRefund – จำนวนเงินคืน</t>
+  </si>
+  <si>
+    <t>UT20 – RefundServiceImpl – เงื่อนไขอื่นของการคืนเงิน</t>
+  </si>
+  <si>
+    <t>refundAmount</t>
+  </si>
+  <si>
+    <t>RefundServiceImpl.processRefund – จำนวนเงินคืน</t>
+  </si>
+  <si>
+    <t>RefundResponseDTO processRefund(RefundRequestDTO request) : 0 &lt; refundAmount ≤ net − คืนไปแล้ว</t>
+  </si>
+  <si>
+    <t>599.99</t>
+  </si>
+  <si>
+    <t>UC-10 A1 • BR-PAY-02 (Refund เป็น record แยก)</t>
+  </si>
+  <si>
+    <t>600.01</t>
+  </si>
+  <si>
+    <t>UT19-TC001</t>
+  </si>
+  <si>
+    <t>ValidationException "Refund amount must be greater than zero"</t>
+  </si>
+  <si>
+    <t>UT19-TC002</t>
+  </si>
+  <si>
+    <t>บันทึก Refund COMPLETED 0.01 • Payment คง COMPLETED</t>
+  </si>
+  <si>
+    <t>UT19-TC003</t>
+  </si>
+  <si>
+    <t>บันทึก Refund • Payment คง COMPLETED</t>
+  </si>
+  <si>
+    <t>UT19-TC004</t>
+  </si>
+  <si>
+    <t>UT19-TC005</t>
+  </si>
+  <si>
+    <t>UT19-TC006</t>
+  </si>
+  <si>
+    <t>บันทึก Refund • Payment เปลี่ยนเป็น REFUNDED และถูก save</t>
+  </si>
+  <si>
+    <t>UT19-TC007</t>
+  </si>
+  <si>
+    <t>ValidationException "...exceeds maximum remaining refundable balance (600.00)"</t>
+  </si>
+  <si>
+    <t>Payment COMPLETED เคยคืนแล้ว 200 (COMPLETED) → คงเหลือ 400</t>
+  </si>
+  <si>
+    <t>request = null หรือ paymentId = null</t>
+  </si>
+  <si>
+    <t>Refund เก่าสถานะ FAILED ไม่นับ</t>
+  </si>
+  <si>
+    <t>ไม่พบ Payment</t>
+  </si>
+  <si>
+    <t>processedByStaff ว่าง → "Staff"</t>
+  </si>
+  <si>
+    <t>Payment PENDING / FAILED</t>
+  </si>
+  <si>
+    <t>ดึง refund ล่าสุดของ payment ที่มี refund</t>
+  </si>
+  <si>
+    <t>คืนเกินยอดคงเหลือหลังคืนบางส่วน</t>
+  </si>
+  <si>
+    <t>getRefundByPaymentId ไม่มี refund</t>
+  </si>
+  <si>
+    <t>id = null ในเมธอด get</t>
+  </si>
+  <si>
+    <t>RefundServiceImpl – เงื่อนไขอื่นของการคืนเงิน</t>
+  </si>
+  <si>
+    <t>processRefund(...), getRefundByPaymentId(...), getRefundsByBookingId(...)</t>
+  </si>
+  <si>
+    <t>UC-10 A1 • BR-PAY-02</t>
+  </si>
+  <si>
+    <t>สภาพ Payment / refund เดิม</t>
+  </si>
+  <si>
+    <t>request</t>
+  </si>
+  <si>
+    <t>UT20-TC001</t>
+  </si>
+  <si>
+    <t>COMPLETED, คืนแล้ว 200 (COMPLETED)</t>
+  </si>
+  <si>
+    <t>refund 400.00</t>
+  </si>
+  <si>
+    <t>(V1) สำเร็จ • Payment → REFUNDED</t>
+  </si>
+  <si>
+    <t>UT20-TC002</t>
+  </si>
+  <si>
+    <t>COMPLETED, refund เก่า 200 สถานะ FAILED</t>
+  </si>
+  <si>
+    <t>refund 600.00</t>
+  </si>
+  <si>
+    <t>(V2) สำเร็จ (คงเหลือ 600) • Payment → REFUNDED</t>
+  </si>
+  <si>
+    <t>UT20-TC003</t>
+  </si>
+  <si>
+    <t>refund 100, processedByStaff = "  "</t>
+  </si>
+  <si>
+    <t>(V3) processedByStaff = "Staff"</t>
+  </si>
+  <si>
+    <t>UT20-TC004</t>
+  </si>
+  <si>
+    <t>มี refund 2 รายการ</t>
+  </si>
+  <si>
+    <t>getRefundByPaymentId(1)</t>
+  </si>
+  <si>
+    <t>(V4) คืนรายการ id ล่าสุด</t>
+  </si>
+  <si>
+    <t>UT20-TC005</t>
+  </si>
+  <si>
+    <t>request = null</t>
+  </si>
+  <si>
+    <t>(I1) ValidationException "Payment ID is required..."</t>
+  </si>
+  <si>
+    <t>UT20-TC006</t>
+  </si>
+  <si>
+    <t>ไม่พบ Payment#999</t>
+  </si>
+  <si>
+    <t>paymentId 999, 100.00</t>
+  </si>
+  <si>
+    <t>(I2) NotFoundException</t>
+  </si>
+  <si>
+    <t>UT20-TC007</t>
+  </si>
+  <si>
+    <t>refund 100.00</t>
+  </si>
+  <si>
+    <t>(I3) ConflictException "...not COMPLETED..."</t>
+  </si>
+  <si>
+    <t>UT20-TC008</t>
+  </si>
+  <si>
+    <t>COMPLETED, คืนแล้ว 200</t>
+  </si>
+  <si>
+    <t>refund 400.01</t>
+  </si>
+  <si>
+    <t>(I4) ValidationException เกินยอดคงเหลือ 400.00</t>
+  </si>
+  <si>
+    <t>UT20-TC009</t>
+  </si>
+  <si>
+    <t>ไม่มี refund</t>
+  </si>
+  <si>
+    <t>(I5) NotFoundException</t>
+  </si>
+  <si>
+    <t>UT20-TC010</t>
+  </si>
+  <si>
+    <t>getRefundsByBookingId(null)</t>
+  </si>
+  <si>
+    <t>(I6) ValidationException</t>
+  </si>
+  <si>
+    <t>บันทึก Refund COMPLETED 0.01 Payment คง COMPLETED</t>
+  </si>
+  <si>
+    <t>บันทึก Refund Payment คง COMPLETED</t>
+  </si>
+  <si>
+    <t>บันทึก Refund Payment เปลี่ยนเป็น REFUNDED และถูก save</t>
+  </si>
+  <si>
+    <t>สำเร็จ • Payment → REFUNDED</t>
+  </si>
+  <si>
+    <t>processedByStaff = "Staff"</t>
+  </si>
+  <si>
+    <t>คืนรายการ id ล่าสุด</t>
+  </si>
+  <si>
+    <t>สำเร็จ (คงเหลือ 600) • Payment → REFUNDED</t>
   </si>
 </sst>
 </file>
@@ -3790,7 +4026,49 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="54">
+  <dxfs count="60">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -4645,7 +4923,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{659A469D-55E7-4F16-B797-78C1D60B492C}">
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="1" width="5.25" customWidth="1"/>
@@ -5315,39 +5593,117 @@
       <c r="I22" s="4"/>
     </row>
     <row r="23" spans="1:9" ht="21">
-      <c r="A23" s="24" t="s">
+      <c r="A23" s="26" t="s">
+        <v>1123</v>
+      </c>
+      <c r="B23" s="26"/>
+      <c r="C23" s="26"/>
+      <c r="D23" s="26"/>
+      <c r="E23" s="26"/>
+      <c r="F23" s="26"/>
+      <c r="G23" s="26"/>
+      <c r="H23" s="26"/>
+      <c r="I23" s="26"/>
+    </row>
+    <row r="24" spans="1:9" ht="21">
+      <c r="A24" s="3">
+        <v>19</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>1124</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D24" s="3">
+        <f>COUNTA(UT19_Refund_Amount_BVA!$A$12:$A$18)</f>
+        <v>6</v>
+      </c>
+      <c r="E24" s="3">
+        <f>COUNTIF(UT19_Refund_Amount_BVA!$E$12:$E$18,"Pass")</f>
+        <v>6</v>
+      </c>
+      <c r="F24" s="3">
+        <f>COUNTIF(UT19_Refund_Amount_BVA!$E$12:$E$18,"Fail")</f>
+        <v>0</v>
+      </c>
+      <c r="G24" s="3">
+        <f>COUNTIF(UT19_Refund_Amount_BVA!$E$12:$E$18,"No run")</f>
+        <v>0</v>
+      </c>
+      <c r="H24" s="3">
+        <f>COUNTIF(UT19_Refund_Amount_BVA!$E$12:$E$18,"Block")</f>
+        <v>0</v>
+      </c>
+      <c r="I24" s="4"/>
+    </row>
+    <row r="25" spans="1:9" ht="21">
+      <c r="A25" s="3">
+        <v>20</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>1125</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D25" s="3">
+        <f>COUNTA(UT20_Refund_EC!$A$22:$A$31)</f>
+        <v>9</v>
+      </c>
+      <c r="E25" s="3">
+        <f>COUNTIF(UT20_Refund_EC!$F$22:$F$31,"Pass")</f>
+        <v>9</v>
+      </c>
+      <c r="F25" s="3">
+        <f>COUNTIF(UT20_Refund_EC!$F$22:$F$31,"Fail")</f>
+        <v>0</v>
+      </c>
+      <c r="G25" s="3">
+        <f>COUNTIF(UT20_Refund_EC!$F$22:$F$31,"No run")</f>
+        <v>0</v>
+      </c>
+      <c r="H25" s="3">
+        <f>COUNTIF(UT20_Refund_EC!$F$22:$F$31,"Block")</f>
+        <v>0</v>
+      </c>
+      <c r="I25" s="4"/>
+    </row>
+    <row r="26" spans="1:9" ht="21">
+      <c r="A26" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="B23" s="24"/>
-      <c r="C23" s="24"/>
-      <c r="D23" s="5" cm="1">
-        <f t="array" ref="D23">SUMPRODUCT(ISNUMBER(D4:D22)*D4:D22)</f>
-        <v>203</v>
-      </c>
-      <c r="E23" s="6" cm="1">
-        <f t="array" ref="E23">SUMPRODUCT(ISNUMBER(E4:E22)*E4:E22)</f>
-        <v>191</v>
-      </c>
-      <c r="F23" s="7" cm="1">
-        <f t="array" ref="F23">SUMPRODUCT(ISNUMBER(F4:F22)*F4:F22)</f>
+      <c r="B26" s="24"/>
+      <c r="C26" s="24"/>
+      <c r="D26" s="5" cm="1">
+        <f t="array" ref="D26">SUMPRODUCT(ISNUMBER(D4:D25)*D4:D25)</f>
+        <v>218</v>
+      </c>
+      <c r="E26" s="6" cm="1">
+        <f t="array" ref="E26">SUMPRODUCT(ISNUMBER(E4:E25)*E4:E25)</f>
+        <v>206</v>
+      </c>
+      <c r="F26" s="7" cm="1">
+        <f t="array" ref="F26">SUMPRODUCT(ISNUMBER(F4:F25)*F4:F25)</f>
         <v>12</v>
       </c>
-      <c r="G23" s="5" cm="1">
-        <f t="array" ref="G23">SUMPRODUCT(ISNUMBER(G4:G22)*G4:G22)</f>
+      <c r="G26" s="5" cm="1">
+        <f t="array" ref="G26">SUMPRODUCT(ISNUMBER(G4:G25)*G4:G25)</f>
         <v>0</v>
       </c>
-      <c r="H23" s="5" cm="1">
-        <f t="array" ref="H23">SUMPRODUCT(ISNUMBER(H4:H22)*H4:H22)</f>
+      <c r="H26" s="5" cm="1">
+        <f t="array" ref="H26">SUMPRODUCT(ISNUMBER(H4:H25)*H4:H25)</f>
         <v>0</v>
       </c>
-      <c r="I23" s="4"/>
+      <c r="I26" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A23:C23"/>
+  <mergeCells count="5">
+    <mergeCell ref="A26:C26"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="A16:I16"/>
+    <mergeCell ref="A23:I23"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -7021,13 +7377,13 @@
     <mergeCell ref="B26:H26"/>
   </mergeCells>
   <conditionalFormatting sqref="H30:H74">
-    <cfRule type="cellIs" dxfId="32" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="38" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="31" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="37" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="36" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7466,13 +7822,13 @@
     <mergeCell ref="E21:E22"/>
   </mergeCells>
   <conditionalFormatting sqref="E23:E30">
-    <cfRule type="cellIs" dxfId="29" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="35" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="34" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="27" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="33" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7802,13 +8158,13 @@
     <mergeCell ref="B7:E7"/>
   </mergeCells>
   <conditionalFormatting sqref="E12:E19">
-    <cfRule type="cellIs" dxfId="26" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="32" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="31" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="30" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8347,13 +8703,13 @@
     <mergeCell ref="F4:I4"/>
   </mergeCells>
   <conditionalFormatting sqref="G23:G31">
-    <cfRule type="cellIs" dxfId="23" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="29" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="28" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="27" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8811,13 +9167,13 @@
     <mergeCell ref="F4:I4"/>
   </mergeCells>
   <conditionalFormatting sqref="F22:F29">
-    <cfRule type="cellIs" dxfId="20" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="26" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="19" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="25" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="24" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9572,13 +9928,13 @@
     <mergeCell ref="B24:I24"/>
   </mergeCells>
   <conditionalFormatting sqref="H29:H36">
-    <cfRule type="cellIs" dxfId="17" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="23" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="22" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="21" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10163,13 +10519,13 @@
     <mergeCell ref="F4:I4"/>
   </mergeCells>
   <conditionalFormatting sqref="G22:G32">
-    <cfRule type="cellIs" dxfId="14" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="20" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="18" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10669,13 +11025,13 @@
     <mergeCell ref="B6:F6"/>
   </mergeCells>
   <conditionalFormatting sqref="F11:F24">
-    <cfRule type="cellIs" dxfId="11" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="17" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11152,13 +11508,13 @@
     <mergeCell ref="F4:I4"/>
   </mergeCells>
   <conditionalFormatting sqref="F19:F27">
-    <cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11612,13 +11968,13 @@
     <mergeCell ref="F4:I4"/>
   </mergeCells>
   <conditionalFormatting sqref="F19:F26">
-    <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12462,13 +12818,13 @@
     <mergeCell ref="F4:I4"/>
   </mergeCells>
   <conditionalFormatting sqref="F20:F29">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12481,6 +12837,847 @@
   <hyperlinks>
     <hyperlink ref="E29" r:id="rId1" xr:uid="{5EEFAEC4-2013-432B-8EEE-0A7BCB87DC75}"/>
   </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE9FD148-76E2-4961-8D8E-DD3613A30109}">
+  <dimension ref="A1:I17"/>
+  <sheetFormatPr defaultColWidth="7.625" defaultRowHeight="23.25"/>
+  <cols>
+    <col min="1" max="1" width="19.25" style="8" customWidth="1"/>
+    <col min="2" max="2" width="15.75" style="8" customWidth="1"/>
+    <col min="3" max="3" width="49" style="8" customWidth="1"/>
+    <col min="4" max="4" width="37.25" style="8" customWidth="1"/>
+    <col min="5" max="5" width="17.125" style="8" customWidth="1"/>
+    <col min="6" max="7" width="7.625" style="8"/>
+    <col min="8" max="8" width="8.75" style="8" customWidth="1"/>
+    <col min="9" max="9" width="19.25" style="8" customWidth="1"/>
+    <col min="10" max="16384" width="7.625" style="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="31" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="15" t="s">
+        <v>1126</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="H2" s="17" t="s">
+        <v>224</v>
+      </c>
+      <c r="I2" s="17" t="s">
+        <v>933</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B3" s="33" t="s">
+        <v>1127</v>
+      </c>
+      <c r="C3" s="33"/>
+      <c r="D3" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="E3" s="14" t="s">
+        <v>154</v>
+      </c>
+      <c r="H3" s="17" t="s">
+        <v>228</v>
+      </c>
+      <c r="I3" s="17" t="s">
+        <v>936</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" s="33" t="s">
+        <v>231</v>
+      </c>
+      <c r="C4" s="33"/>
+      <c r="D4" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="E4" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="H4" s="17" t="s">
+        <v>232</v>
+      </c>
+      <c r="I4" s="17" t="s">
+        <v>938</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="46.5">
+      <c r="A5" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B5" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" s="33"/>
+      <c r="D5" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="H5" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="I5" s="17" t="s">
+        <v>935</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="46.5">
+      <c r="A6" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="B6" s="33" t="s">
+        <v>1128</v>
+      </c>
+      <c r="C6" s="33"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
+      <c r="H6" s="17" t="s">
+        <v>238</v>
+      </c>
+      <c r="I6" s="17" t="s">
+        <v>1129</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="46.5">
+      <c r="A7" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B7" s="33" t="s">
+        <v>1130</v>
+      </c>
+      <c r="C7" s="33"/>
+      <c r="D7" s="33"/>
+      <c r="E7" s="33"/>
+      <c r="H7" s="17" t="s">
+        <v>244</v>
+      </c>
+      <c r="I7" s="17" t="s">
+        <v>1131</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="B9" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="C9" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="D9" s="32" t="s">
+        <v>75</v>
+      </c>
+      <c r="E9" s="32" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" s="32"/>
+      <c r="B10" s="15" t="s">
+        <v>1126</v>
+      </c>
+      <c r="C10" s="32"/>
+      <c r="D10" s="32"/>
+      <c r="E10" s="32"/>
+    </row>
+    <row r="11" spans="1:9" ht="46.5">
+      <c r="A11" s="16" t="s">
+        <v>1132</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>933</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>1133</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="E11" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="46.5">
+      <c r="A12" s="16" t="s">
+        <v>1134</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>936</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>1135</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>1194</v>
+      </c>
+      <c r="E12" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="24.75" customHeight="1">
+      <c r="A13" s="16" t="s">
+        <v>1136</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>938</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>1137</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>1195</v>
+      </c>
+      <c r="E13" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" s="16" t="s">
+        <v>1138</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>935</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>1137</v>
+      </c>
+      <c r="D14" s="13" t="s">
+        <v>1195</v>
+      </c>
+      <c r="E14" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15" s="16" t="s">
+        <v>1139</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>1129</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>1137</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>1195</v>
+      </c>
+      <c r="E15" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="46.5">
+      <c r="A16" s="16" t="s">
+        <v>1140</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>908</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>1141</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>1196</v>
+      </c>
+      <c r="E16" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="46.5">
+      <c r="A17" s="16" t="s">
+        <v>1142</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>1131</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>1143</v>
+      </c>
+      <c r="D17" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="E17" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:E6"/>
+  </mergeCells>
+  <conditionalFormatting sqref="E11:E17">
+    <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
+      <formula>"Pass"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
+      <formula>"Fail"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
+      <formula>"Block"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" sqref="E11:E17" xr:uid="{832921AF-75EF-4347-9F7F-972662CC6DBE}">
+      <formula1>"Pass,Fail,No run,Block"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6AE9CF8C-F017-43DA-B70D-575F77D1CBC6}">
+  <dimension ref="A1:I30"/>
+  <sheetFormatPr defaultColWidth="7.625" defaultRowHeight="23.25"/>
+  <cols>
+    <col min="1" max="1" width="19.25" style="8" customWidth="1"/>
+    <col min="2" max="3" width="22.75" style="8" customWidth="1"/>
+    <col min="4" max="4" width="36.75" style="8" customWidth="1"/>
+    <col min="5" max="5" width="34.625" style="8" customWidth="1"/>
+    <col min="6" max="6" width="14.875" style="8" customWidth="1"/>
+    <col min="7" max="8" width="12.25" style="8" customWidth="1"/>
+    <col min="9" max="9" width="17.75" style="8" customWidth="1"/>
+    <col min="10" max="16384" width="7.625" style="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="24" thickBot="1">
+      <c r="A1" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+    </row>
+    <row r="2" spans="1:9" ht="24" thickBot="1">
+      <c r="A2" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" s="28" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" s="28"/>
+    </row>
+    <row r="3" spans="1:9" ht="24" thickBot="1">
+      <c r="A3" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="29" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="29"/>
+      <c r="E3" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="29" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" s="29"/>
+      <c r="H3" s="29"/>
+      <c r="I3" s="29"/>
+    </row>
+    <row r="4" spans="1:9" ht="24" thickBot="1">
+      <c r="A4" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="30" t="s">
+        <v>1144</v>
+      </c>
+      <c r="C4" s="30"/>
+      <c r="E4" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="30" t="s">
+        <v>1145</v>
+      </c>
+      <c r="G4" s="30"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="30"/>
+    </row>
+    <row r="5" spans="1:9" ht="24" thickBot="1">
+      <c r="A5" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="30" t="s">
+        <v>1146</v>
+      </c>
+      <c r="C5" s="30"/>
+      <c r="E5" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" s="30" t="s">
+        <v>1147</v>
+      </c>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+    </row>
+    <row r="6" spans="1:9" ht="24" thickBot="1">
+      <c r="A6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="30" t="s">
+        <v>1148</v>
+      </c>
+      <c r="C6" s="30"/>
+      <c r="E6" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="F6" s="30" t="s">
+        <v>1149</v>
+      </c>
+      <c r="G6" s="30"/>
+      <c r="H6" s="30"/>
+      <c r="I6" s="30"/>
+    </row>
+    <row r="7" spans="1:9" ht="24" thickBot="1">
+      <c r="A7" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="30" t="s">
+        <v>1150</v>
+      </c>
+      <c r="C7" s="30"/>
+      <c r="E7" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" s="30" t="s">
+        <v>1151</v>
+      </c>
+      <c r="G7" s="30"/>
+      <c r="H7" s="30"/>
+      <c r="I7" s="30"/>
+    </row>
+    <row r="8" spans="1:9" ht="24" thickBot="1">
+      <c r="E8" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="F8" s="30" t="s">
+        <v>1152</v>
+      </c>
+      <c r="G8" s="30"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="30"/>
+    </row>
+    <row r="9" spans="1:9" ht="24" thickBot="1">
+      <c r="E9" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="F9" s="30" t="s">
+        <v>1153</v>
+      </c>
+      <c r="G9" s="30"/>
+      <c r="H9" s="30"/>
+      <c r="I9" s="30"/>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" s="31" t="s">
+        <v>57</v>
+      </c>
+      <c r="B11" s="31"/>
+      <c r="C11" s="31"/>
+      <c r="D11" s="31"/>
+      <c r="E11" s="31"/>
+      <c r="F11" s="31"/>
+      <c r="G11" s="31"/>
+      <c r="H11" s="31"/>
+      <c r="I11" s="31"/>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B13" s="33" t="s">
+        <v>1154</v>
+      </c>
+      <c r="C13" s="33"/>
+      <c r="D13" s="33"/>
+      <c r="E13" s="21"/>
+      <c r="F13" s="21"/>
+      <c r="G13" s="21"/>
+      <c r="H13" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="I13" s="14" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="B14" s="33" t="s">
+        <v>62</v>
+      </c>
+      <c r="C14" s="33"/>
+      <c r="D14" s="33"/>
+      <c r="E14" s="21"/>
+      <c r="F14" s="21"/>
+      <c r="G14" s="21"/>
+      <c r="H14" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="I14" s="14" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="46.5">
+      <c r="A15" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B15" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="C15" s="33"/>
+      <c r="D15" s="33"/>
+      <c r="E15" s="21"/>
+      <c r="F15" s="21"/>
+      <c r="G15" s="21"/>
+      <c r="H15" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="I15" s="13" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="46.5">
+      <c r="A16" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="B16" s="33" t="s">
+        <v>1155</v>
+      </c>
+      <c r="C16" s="33"/>
+      <c r="D16" s="33"/>
+      <c r="E16" s="33"/>
+      <c r="F16" s="33"/>
+      <c r="G16" s="33"/>
+      <c r="H16" s="33"/>
+      <c r="I16" s="33"/>
+    </row>
+    <row r="17" spans="1:9" ht="46.5">
+      <c r="A17" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B17" s="33" t="s">
+        <v>1156</v>
+      </c>
+      <c r="C17" s="33"/>
+      <c r="D17" s="33"/>
+      <c r="E17" s="33"/>
+      <c r="F17" s="33"/>
+      <c r="G17" s="33"/>
+      <c r="H17" s="33"/>
+      <c r="I17" s="33"/>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="B19" s="32" t="s">
+        <v>73</v>
+      </c>
+      <c r="C19" s="32"/>
+      <c r="D19" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="E19" s="32" t="s">
+        <v>75</v>
+      </c>
+      <c r="F19" s="32" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="46.5">
+      <c r="A20" s="32"/>
+      <c r="B20" s="15" t="s">
+        <v>1157</v>
+      </c>
+      <c r="C20" s="15" t="s">
+        <v>1158</v>
+      </c>
+      <c r="D20" s="32"/>
+      <c r="E20" s="32"/>
+      <c r="F20" s="32"/>
+    </row>
+    <row r="21" spans="1:9" ht="46.5">
+      <c r="A21" s="16" t="s">
+        <v>1159</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>1160</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>1161</v>
+      </c>
+      <c r="D21" s="13" t="s">
+        <v>1162</v>
+      </c>
+      <c r="E21" s="13" t="s">
+        <v>1197</v>
+      </c>
+      <c r="F21" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="46.5">
+      <c r="A22" s="16" t="s">
+        <v>1163</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>1164</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>1165</v>
+      </c>
+      <c r="D22" s="13" t="s">
+        <v>1166</v>
+      </c>
+      <c r="E22" s="13" t="s">
+        <v>1200</v>
+      </c>
+      <c r="F22" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="46.5">
+      <c r="A23" s="16" t="s">
+        <v>1167</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>420</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>1168</v>
+      </c>
+      <c r="D23" s="13" t="s">
+        <v>1169</v>
+      </c>
+      <c r="E23" s="13" t="s">
+        <v>1198</v>
+      </c>
+      <c r="F23" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="46.5">
+      <c r="A24" s="16" t="s">
+        <v>1170</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>1171</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>1172</v>
+      </c>
+      <c r="D24" s="13" t="s">
+        <v>1173</v>
+      </c>
+      <c r="E24" s="13" t="s">
+        <v>1199</v>
+      </c>
+      <c r="F24" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="46.5">
+      <c r="A25" s="16" t="s">
+        <v>1174</v>
+      </c>
+      <c r="B25" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>1175</v>
+      </c>
+      <c r="D25" s="13" t="s">
+        <v>1176</v>
+      </c>
+      <c r="E25" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="F25" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9">
+      <c r="A26" s="16" t="s">
+        <v>1177</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>1178</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>1179</v>
+      </c>
+      <c r="D26" s="13" t="s">
+        <v>1180</v>
+      </c>
+      <c r="E26" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="F26" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="46.5">
+      <c r="A27" s="16" t="s">
+        <v>1181</v>
+      </c>
+      <c r="B27" s="13" t="s">
+        <v>505</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>1182</v>
+      </c>
+      <c r="D27" s="13" t="s">
+        <v>1183</v>
+      </c>
+      <c r="E27" s="13" t="s">
+        <v>201</v>
+      </c>
+      <c r="F27" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="46.5">
+      <c r="A28" s="16" t="s">
+        <v>1184</v>
+      </c>
+      <c r="B28" s="13" t="s">
+        <v>1185</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>1186</v>
+      </c>
+      <c r="D28" s="13" t="s">
+        <v>1187</v>
+      </c>
+      <c r="E28" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="F28" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="46.5">
+      <c r="A29" s="16" t="s">
+        <v>1188</v>
+      </c>
+      <c r="B29" s="13" t="s">
+        <v>1189</v>
+      </c>
+      <c r="C29" s="13" t="s">
+        <v>1172</v>
+      </c>
+      <c r="D29" s="13" t="s">
+        <v>1190</v>
+      </c>
+      <c r="E29" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="F29" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="46.5">
+      <c r="A30" s="16" t="s">
+        <v>1191</v>
+      </c>
+      <c r="B30" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="C30" s="13" t="s">
+        <v>1192</v>
+      </c>
+      <c r="D30" s="13" t="s">
+        <v>1193</v>
+      </c>
+      <c r="E30" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="F30" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="25">
+    <mergeCell ref="B16:I16"/>
+    <mergeCell ref="B17:I17"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="F8:I8"/>
+    <mergeCell ref="F9:I9"/>
+    <mergeCell ref="A11:I11"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="F5:I5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="F6:I6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="F7:I7"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="F3:I3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="F4:I4"/>
+  </mergeCells>
+  <conditionalFormatting sqref="F21:F30">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+      <formula>"Pass"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+      <formula>"Fail"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
+      <formula>"Block"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" sqref="F21:F30" xr:uid="{122556AA-8CA2-4B31-8461-856C2C782A24}">
+      <formula1>"Pass,Fail,No run,Block"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -13401,13 +14598,13 @@
     <mergeCell ref="G4:J4"/>
   </mergeCells>
   <conditionalFormatting sqref="J28:J42">
-    <cfRule type="cellIs" dxfId="53" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="59" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="52" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="58" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="51" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="57" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -14215,13 +15412,13 @@
     <mergeCell ref="H27:H28"/>
   </mergeCells>
   <conditionalFormatting sqref="H29:H38">
-    <cfRule type="cellIs" dxfId="50" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="56" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="49" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="55" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="48" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="54" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -14750,13 +15947,13 @@
     <mergeCell ref="B6:G6"/>
   </mergeCells>
   <conditionalFormatting sqref="G11:G23">
-    <cfRule type="cellIs" dxfId="47" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="53" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="46" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="52" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="45" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="51" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -15346,13 +16543,13 @@
     <mergeCell ref="H9:H10"/>
   </mergeCells>
   <conditionalFormatting sqref="H11:H23">
-    <cfRule type="cellIs" dxfId="44" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="50" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="43" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="49" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="42" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="48" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -16371,13 +17568,13 @@
     <mergeCell ref="I32:I33"/>
   </mergeCells>
   <conditionalFormatting sqref="I34:I45">
-    <cfRule type="cellIs" dxfId="41" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="47" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="46" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="39" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="45" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -16670,13 +17867,13 @@
     <mergeCell ref="F9:F10"/>
   </mergeCells>
   <conditionalFormatting sqref="F11:F15">
-    <cfRule type="cellIs" dxfId="38" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="44" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="43" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="36" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="42" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -17288,13 +18485,13 @@
     <mergeCell ref="G23:G24"/>
   </mergeCells>
   <conditionalFormatting sqref="G25:G32">
-    <cfRule type="cellIs" dxfId="35" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="41" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="34" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="40" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="33" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="39" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Unit Test in ReviewServiceImpl
</commit_message>
<xml_diff>
--- a/test/FIWDEE_UnitTest_Report.xlsx
+++ b/test/FIWDEE_UnitTest_Report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\ProjectPOS\FIWDEE-CP353002-69_1PrinciplesOfSoftwareDesign\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5E33E11-8F98-4122-95DC-35EE6951992B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4BFD972-D322-454C-BACE-7E99A85D5A2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9B0ECA1C-B255-4EEE-B7A8-035645CFC3D9}"/>
   </bookViews>
@@ -39,9 +39,11 @@
     <sheet name="UT22_CheckIn_Queue_EC" sheetId="26" r:id="rId24"/>
     <sheet name="UT23_QueueStatus_DT" sheetId="27" r:id="rId25"/>
     <sheet name="UT24_TherapistExec_DT" sheetId="28" r:id="rId26"/>
+    <sheet name="UT25_Review_Rating_BVA" sheetId="29" r:id="rId27"/>
+    <sheet name="UT26_Review_EC" sheetId="30" r:id="rId28"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId27"/>
+    <externalReference r:id="rId29"/>
   </externalReferences>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -89,7 +91,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3677" uniqueCount="1418">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3981" uniqueCount="1499">
   <si>
     <t>FIWDEE – Unit Test Design</t>
   </si>
@@ -4343,6 +4345,249 @@
   </si>
   <si>
     <t>DEF-010</t>
+  </si>
+  <si>
+    <t>Review</t>
+  </si>
+  <si>
+    <t>UT25 – ReviewServiceImpl.submitReview – คะแนน 3 ด้าน</t>
+  </si>
+  <si>
+    <t>UT26 – ReviewServiceImpl.submitReview – เงื่อนไขอื่น</t>
+  </si>
+  <si>
+    <t>DEF-011</t>
+  </si>
+  <si>
+    <t>ผู้ใช้คนใดก็รีวิว booking ของคนอื่นได้</t>
+  </si>
+  <si>
+    <t>service/impl/ReviewServiceImpl.submitReview และ ReviewController ไม่รับ/ไม่ตรวจผู้ใช้ปัจจุบัน • ผิด BR-SEC-01 • UT26-TC010</t>
+  </si>
+  <si>
+    <t>overallRating</t>
+  </si>
+  <si>
+    <t>therapistRating</t>
+  </si>
+  <si>
+    <t>cleanlinessRating</t>
+  </si>
+  <si>
+    <t>ReviewServiceImpl.submitReview – คะแนน 3 ด้าน</t>
+  </si>
+  <si>
+    <t>Review submitReview(bookingId, overallRating, therapistRating, cleanlinessRating, comment)</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>SRS 3.4 (ให้คะแนน 1–5 ดาว) • UC-18</t>
+  </si>
+  <si>
+    <t>UT25-TC001</t>
+  </si>
+  <si>
+    <t>บันทึกรีวิวสำเร็จ (nom)</t>
+  </si>
+  <si>
+    <t>UT25-TC002</t>
+  </si>
+  <si>
+    <t>ValidationException "Overall rating must be between 1 and 5" • ไม่บันทึก</t>
+  </si>
+  <si>
+    <t>UT25-TC003</t>
+  </si>
+  <si>
+    <t>บันทึกรีวิวสำเร็จ (saveAndFlush 1 ครั้ง)</t>
+  </si>
+  <si>
+    <t>UT25-TC004</t>
+  </si>
+  <si>
+    <t>UT25-TC005</t>
+  </si>
+  <si>
+    <t>UT25-TC006</t>
+  </si>
+  <si>
+    <t>UT25-TC007</t>
+  </si>
+  <si>
+    <t>UT25-TC008</t>
+  </si>
+  <si>
+    <t>ValidationException "Therapist rating must be between 1 and 5" • ไม่บันทึก</t>
+  </si>
+  <si>
+    <t>UT25-TC009</t>
+  </si>
+  <si>
+    <t>UT25-TC010</t>
+  </si>
+  <si>
+    <t>UT25-TC011</t>
+  </si>
+  <si>
+    <t>UT25-TC012</t>
+  </si>
+  <si>
+    <t>UT25-TC013</t>
+  </si>
+  <si>
+    <t>UT25-TC014</t>
+  </si>
+  <si>
+    <t>ValidationException "Cleanliness rating must be between 1 and 5" • ไม่บันทึก</t>
+  </si>
+  <si>
+    <t>UT25-TC015</t>
+  </si>
+  <si>
+    <t>UT25-TC016</t>
+  </si>
+  <si>
+    <t>UT25-TC017</t>
+  </si>
+  <si>
+    <t>UT25-TC018</t>
+  </si>
+  <si>
+    <t>UT25-TC019</t>
+  </si>
+  <si>
+    <t>booking COMPLETED ยังไม่มีรีวิว</t>
+  </si>
+  <si>
+    <t>comment มีช่องว่างหน้า/หลัง → trim</t>
+  </si>
+  <si>
+    <t>booking ยังไม่ COMPLETED</t>
+  </si>
+  <si>
+    <t>comment ว่างหรือช่องว่างล้วน → null</t>
+  </si>
+  <si>
+    <t>รีวิวซ้ำ</t>
+  </si>
+  <si>
+    <t>หมอนวดมีรีวิว 5, 4, 4 → average 4.33</t>
+  </si>
+  <si>
+    <t>คะแนน = null</t>
+  </si>
+  <si>
+    <t>booking ไม่มีหมอนวด → ไม่คำนวณ average และไม่ error</t>
+  </si>
+  <si>
+    <t>ผู้รีวิวไม่ใช่เจ้าของ booking</t>
+  </si>
+  <si>
+    <t>ReviewServiceImpl.submitReview – เงื่อนไขอื่น</t>
+  </si>
+  <si>
+    <t>submitReview(...) • refreshTherapistAverageRating • normalizeComment</t>
+  </si>
+  <si>
+    <t>UC-18 • SRS 3.4 • BR-SEC-01</t>
+  </si>
+  <si>
+    <t>bookingId / สถานะ</t>
+  </si>
+  <si>
+    <t>comment / อื่น ๆ</t>
+  </si>
+  <si>
+    <t>UT26-TC001</t>
+  </si>
+  <si>
+    <t>10 / COMPLETED</t>
+  </si>
+  <si>
+    <t>"นวดดีมาก"</t>
+  </si>
+  <si>
+    <t>(V1) บันทึกสำเร็จ, booking.review ถูกตั้งค่า</t>
+  </si>
+  <si>
+    <t>UT26-TC002</t>
+  </si>
+  <si>
+    <t>"  นวดดีมาก  "</t>
+  </si>
+  <si>
+    <t>(V2) comment = "นวดดีมาก"</t>
+  </si>
+  <si>
+    <t>UT26-TC003</t>
+  </si>
+  <si>
+    <t>(V3) comment = null</t>
+  </si>
+  <si>
+    <t>UT26-TC004</t>
+  </si>
+  <si>
+    <t>รีวิวหมอนวด T5 รวม 5, 4, 4</t>
+  </si>
+  <si>
+    <t>(V4) T5.averageRating = 4.33</t>
+  </si>
+  <si>
+    <t>UT26-TC005</t>
+  </si>
+  <si>
+    <t>30 / COMPLETED (therapist = null)</t>
+  </si>
+  <si>
+    <t>(V5) บันทึกสำเร็จ ไม่เกิด NullPointerException</t>
+  </si>
+  <si>
+    <t>UT26-TC006</t>
+  </si>
+  <si>
+    <t>UT26-TC007</t>
+  </si>
+  <si>
+    <t>10 / CONFIRMED</t>
+  </si>
+  <si>
+    <t>(I2) ValidationException "...only be submitted for a completed booking"</t>
+  </si>
+  <si>
+    <t>UT26-TC008</t>
+  </si>
+  <si>
+    <t>10 / COMPLETED มีรีวิวแล้ว</t>
+  </si>
+  <si>
+    <t>(I3) ConflictException</t>
+  </si>
+  <si>
+    <t>UT26-TC009</t>
+  </si>
+  <si>
+    <t>overallRating = null</t>
+  </si>
+  <si>
+    <t>(I4) ValidationException</t>
+  </si>
+  <si>
+    <t>บันทึกรีวิวสำเร็จ</t>
+  </si>
+  <si>
+    <t>บันทึกสำเร็จ</t>
+  </si>
+  <si>
+    <t>comment = "นวดดีมาก"</t>
+  </si>
+  <si>
+    <t>comment = null</t>
+  </si>
+  <si>
+    <t>T5.averageRating = 4.33</t>
   </si>
 </sst>
 </file>
@@ -4688,7 +4933,49 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="72">
+  <dxfs count="78">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -5669,7 +5956,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{659A469D-55E7-4F16-B797-78C1D60B492C}">
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="1" width="5.25" customWidth="1"/>
@@ -6557,41 +6844,119 @@
       <c r="I30" s="4"/>
     </row>
     <row r="31" spans="1:9" ht="21">
-      <c r="A31" s="24" t="s">
+      <c r="A31" s="26" t="s">
+        <v>1418</v>
+      </c>
+      <c r="B31" s="26"/>
+      <c r="C31" s="26"/>
+      <c r="D31" s="26"/>
+      <c r="E31" s="26"/>
+      <c r="F31" s="26"/>
+      <c r="G31" s="26"/>
+      <c r="H31" s="26"/>
+      <c r="I31" s="26"/>
+    </row>
+    <row r="32" spans="1:9" ht="21">
+      <c r="A32" s="3">
+        <v>25</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>1419</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="D32" s="3">
+        <f>COUNTA(UT25_Review_Rating_BVA!$A$12:$A$30)</f>
+        <v>18</v>
+      </c>
+      <c r="E32" s="3">
+        <f>COUNTIF(UT25_Review_Rating_BVA!$G$12:$G$30,"Pass")</f>
+        <v>18</v>
+      </c>
+      <c r="F32" s="3">
+        <f>COUNTIF(UT25_Review_Rating_BVA!$G$12:$G$30,"Fail")</f>
+        <v>0</v>
+      </c>
+      <c r="G32" s="3">
+        <f>COUNTIF(UT25_Review_Rating_BVA!$G$12:$G$30,"No run")</f>
+        <v>0</v>
+      </c>
+      <c r="H32" s="3">
+        <f>COUNTIF(UT25_Review_Rating_BVA!$G$12:$G$30,"Block")</f>
+        <v>0</v>
+      </c>
+      <c r="I32" s="4"/>
+    </row>
+    <row r="33" spans="1:9" ht="21">
+      <c r="A33" s="3">
+        <v>26</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>1420</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D33" s="3">
+        <f>COUNTA(UT26_Review_EC!$A$21:$A$30)</f>
+        <v>8</v>
+      </c>
+      <c r="E33" s="3">
+        <f>COUNTIF(UT26_Review_EC!$F$21:$F$30,"Pass")</f>
+        <v>8</v>
+      </c>
+      <c r="F33" s="3">
+        <f>COUNTIF(UT26_Review_EC!$F$21:$F$30,"Fail")</f>
+        <v>0</v>
+      </c>
+      <c r="G33" s="3">
+        <f>COUNTIF(UT26_Review_EC!$F$21:$F$30,"No run")</f>
+        <v>0</v>
+      </c>
+      <c r="H33" s="3">
+        <f>COUNTIF(UT26_Review_EC!$F$21:$F$30,"Block")</f>
+        <v>0</v>
+      </c>
+      <c r="I33" s="4"/>
+    </row>
+    <row r="34" spans="1:9" ht="21">
+      <c r="A34" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="B31" s="24"/>
-      <c r="C31" s="24"/>
-      <c r="D31" s="5" cm="1">
-        <f t="array" ref="D31">SUMPRODUCT(ISNUMBER(D4:D30)*D4:D30)</f>
-        <v>264</v>
-      </c>
-      <c r="E31" s="6" cm="1">
-        <f t="array" ref="E31">SUMPRODUCT(ISNUMBER(E4:E30)*E4:E30)</f>
-        <v>252</v>
-      </c>
-      <c r="F31" s="7" cm="1">
-        <f t="array" ref="F31">SUMPRODUCT(ISNUMBER(F4:F30)*F4:F30)</f>
+      <c r="B34" s="24"/>
+      <c r="C34" s="24"/>
+      <c r="D34" s="5" cm="1">
+        <f t="array" ref="D34">SUMPRODUCT(ISNUMBER(D4:D33)*D4:D33)</f>
+        <v>290</v>
+      </c>
+      <c r="E34" s="6" cm="1">
+        <f t="array" ref="E34">SUMPRODUCT(ISNUMBER(E4:E33)*E4:E33)</f>
+        <v>278</v>
+      </c>
+      <c r="F34" s="7" cm="1">
+        <f t="array" ref="F34">SUMPRODUCT(ISNUMBER(F4:F33)*F4:F33)</f>
         <v>12</v>
       </c>
-      <c r="G31" s="5" cm="1">
-        <f t="array" ref="G31">SUMPRODUCT(ISNUMBER(G4:G30)*G4:G30)</f>
+      <c r="G34" s="5" cm="1">
+        <f t="array" ref="G34">SUMPRODUCT(ISNUMBER(G4:G33)*G4:G33)</f>
         <v>0</v>
       </c>
-      <c r="H31" s="5" cm="1">
-        <f t="array" ref="H31">SUMPRODUCT(ISNUMBER(H4:H30)*H4:H30)</f>
+      <c r="H34" s="5" cm="1">
+        <f t="array" ref="H34">SUMPRODUCT(ISNUMBER(H4:H33)*H4:H33)</f>
         <v>0</v>
       </c>
-      <c r="I31" s="4"/>
+      <c r="I34" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A31:C31"/>
+  <mergeCells count="7">
+    <mergeCell ref="A34:C34"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="A16:I16"/>
     <mergeCell ref="A23:I23"/>
     <mergeCell ref="A26:I26"/>
+    <mergeCell ref="A31:I31"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -8265,13 +8630,13 @@
     <mergeCell ref="B26:H26"/>
   </mergeCells>
   <conditionalFormatting sqref="H30:H74">
-    <cfRule type="cellIs" dxfId="50" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="56" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="49" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="55" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="48" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="54" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8710,13 +9075,13 @@
     <mergeCell ref="E21:E22"/>
   </mergeCells>
   <conditionalFormatting sqref="E23:E30">
-    <cfRule type="cellIs" dxfId="47" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="53" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="46" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="52" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="45" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="51" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9046,13 +9411,13 @@
     <mergeCell ref="B7:E7"/>
   </mergeCells>
   <conditionalFormatting sqref="E12:E19">
-    <cfRule type="cellIs" dxfId="44" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="50" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="43" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="49" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="42" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="48" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9591,13 +9956,13 @@
     <mergeCell ref="F4:I4"/>
   </mergeCells>
   <conditionalFormatting sqref="G23:G31">
-    <cfRule type="cellIs" dxfId="41" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="47" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="46" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="39" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="45" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10055,13 +10420,13 @@
     <mergeCell ref="F4:I4"/>
   </mergeCells>
   <conditionalFormatting sqref="F22:F29">
-    <cfRule type="cellIs" dxfId="38" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="44" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="43" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="36" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="42" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10816,13 +11181,13 @@
     <mergeCell ref="B24:I24"/>
   </mergeCells>
   <conditionalFormatting sqref="H29:H36">
-    <cfRule type="cellIs" dxfId="35" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="41" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="34" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="40" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="33" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="39" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11407,13 +11772,13 @@
     <mergeCell ref="F4:I4"/>
   </mergeCells>
   <conditionalFormatting sqref="G22:G32">
-    <cfRule type="cellIs" dxfId="32" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="38" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="31" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="37" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="36" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11913,13 +12278,13 @@
     <mergeCell ref="B6:F6"/>
   </mergeCells>
   <conditionalFormatting sqref="F11:F24">
-    <cfRule type="cellIs" dxfId="29" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="35" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="34" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="27" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="33" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12396,13 +12761,13 @@
     <mergeCell ref="F4:I4"/>
   </mergeCells>
   <conditionalFormatting sqref="F19:F27">
-    <cfRule type="cellIs" dxfId="26" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="32" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="31" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="30" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12856,13 +13221,13 @@
     <mergeCell ref="F4:I4"/>
   </mergeCells>
   <conditionalFormatting sqref="F19:F26">
-    <cfRule type="cellIs" dxfId="23" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="29" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="28" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="27" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12878,7 +13243,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93C8330E-079C-4579-8133-7533964AD0F3}">
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr defaultColWidth="7.625" defaultRowHeight="23.25"/>
   <cols>
     <col min="1" max="1" width="5.25" style="8" customWidth="1"/>
@@ -13097,7 +13462,9 @@
         <v>67</v>
       </c>
       <c r="E7" s="13"/>
-      <c r="F7" s="14"/>
+      <c r="F7" s="14" t="s">
+        <v>156</v>
+      </c>
       <c r="G7" s="17" t="s">
         <v>216</v>
       </c>
@@ -13234,6 +13601,37 @@
       <c r="J11" s="13"/>
       <c r="K11" s="13" t="s">
         <v>1120</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="64.5" customHeight="1">
+      <c r="A12" s="17">
+        <v>11</v>
+      </c>
+      <c r="B12" s="17" t="s">
+        <v>1421</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>1422</v>
+      </c>
+      <c r="D12" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="E12" s="13"/>
+      <c r="F12" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="G12" s="17" t="s">
+        <v>216</v>
+      </c>
+      <c r="H12" s="17" t="s">
+        <v>441</v>
+      </c>
+      <c r="I12" s="17" t="s">
+        <v>441</v>
+      </c>
+      <c r="J12" s="13"/>
+      <c r="K12" s="13" t="s">
+        <v>1423</v>
       </c>
     </row>
   </sheetData>
@@ -13736,13 +14134,13 @@
     <mergeCell ref="F4:I4"/>
   </mergeCells>
   <conditionalFormatting sqref="F20:F29">
-    <cfRule type="cellIs" dxfId="20" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="26" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="19" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="25" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="24" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -14052,13 +14450,13 @@
     <mergeCell ref="B6:E6"/>
   </mergeCells>
   <conditionalFormatting sqref="E11:E17">
-    <cfRule type="cellIs" dxfId="17" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="23" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="22" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="21" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -14580,13 +14978,13 @@
     <mergeCell ref="F4:I4"/>
   </mergeCells>
   <conditionalFormatting sqref="F21:F30">
-    <cfRule type="cellIs" dxfId="14" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="20" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="18" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -14899,13 +15297,13 @@
     <mergeCell ref="B6:F6"/>
   </mergeCells>
   <conditionalFormatting sqref="F11:F16">
-    <cfRule type="cellIs" dxfId="11" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="17" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -15422,13 +15820,13 @@
     <mergeCell ref="F4:I4"/>
   </mergeCells>
   <conditionalFormatting sqref="F21:F30">
-    <cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -16440,13 +16838,13 @@
     <mergeCell ref="B22:E22"/>
   </mergeCells>
   <conditionalFormatting sqref="G28:G53">
-    <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -17076,6 +17474,1204 @@
     <mergeCell ref="B21:F21"/>
   </mergeCells>
   <conditionalFormatting sqref="H27:H34">
+    <cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
+      <formula>"Pass"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="7" priority="2" operator="equal">
+      <formula>"Fail"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="3" operator="equal">
+      <formula>"Block"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" sqref="H27:H34" xr:uid="{20B1E575-5034-4BD5-B1D2-38BFE4D9AB36}">
+      <formula1>"Pass,Fail,No run,Block"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F54AAF0-D70E-45F8-A138-60105A467C20}">
+  <dimension ref="A1:M29"/>
+  <sheetFormatPr defaultColWidth="7.625" defaultRowHeight="23.25"/>
+  <cols>
+    <col min="1" max="1" width="19.25" style="8" customWidth="1"/>
+    <col min="2" max="4" width="12.25" style="8" customWidth="1"/>
+    <col min="5" max="5" width="40.25" style="8" customWidth="1"/>
+    <col min="6" max="6" width="30.75" style="8" customWidth="1"/>
+    <col min="7" max="7" width="14.875" style="8" customWidth="1"/>
+    <col min="8" max="9" width="7.625" style="8"/>
+    <col min="10" max="10" width="8.75" style="8" customWidth="1"/>
+    <col min="11" max="13" width="13.125" style="8" customWidth="1"/>
+    <col min="14" max="16384" width="7.625" style="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" ht="46.5">
+      <c r="A1" s="31" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="15" t="s">
+        <v>1424</v>
+      </c>
+      <c r="L1" s="15" t="s">
+        <v>1425</v>
+      </c>
+      <c r="M1" s="15" t="s">
+        <v>1426</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="J2" s="17" t="s">
+        <v>224</v>
+      </c>
+      <c r="K2" s="17" t="s">
+        <v>308</v>
+      </c>
+      <c r="L2" s="17" t="s">
+        <v>308</v>
+      </c>
+      <c r="M2" s="17" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B3" s="33" t="s">
+        <v>1427</v>
+      </c>
+      <c r="C3" s="33"/>
+      <c r="D3" s="33"/>
+      <c r="E3" s="33"/>
+      <c r="F3" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="G3" s="14" t="s">
+        <v>154</v>
+      </c>
+      <c r="J3" s="17" t="s">
+        <v>228</v>
+      </c>
+      <c r="K3" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="L3" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="M3" s="17" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" s="33" t="s">
+        <v>231</v>
+      </c>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="33"/>
+      <c r="F4" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="G4" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="J4" s="17" t="s">
+        <v>232</v>
+      </c>
+      <c r="K4" s="17" t="s">
+        <v>714</v>
+      </c>
+      <c r="L4" s="17" t="s">
+        <v>714</v>
+      </c>
+      <c r="M4" s="17" t="s">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="46.5">
+      <c r="A5" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B5" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" s="33"/>
+      <c r="D5" s="33"/>
+      <c r="E5" s="33"/>
+      <c r="F5" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="G5" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="J5" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="K5" s="17" t="s">
+        <v>107</v>
+      </c>
+      <c r="L5" s="17" t="s">
+        <v>107</v>
+      </c>
+      <c r="M5" s="17" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="46.5">
+      <c r="A6" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="B6" s="33" t="s">
+        <v>1428</v>
+      </c>
+      <c r="C6" s="33"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
+      <c r="F6" s="33"/>
+      <c r="G6" s="33"/>
+      <c r="J6" s="17" t="s">
+        <v>238</v>
+      </c>
+      <c r="K6" s="17" t="s">
+        <v>1429</v>
+      </c>
+      <c r="L6" s="17" t="s">
+        <v>1429</v>
+      </c>
+      <c r="M6" s="17" t="s">
+        <v>1429</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" ht="46.5">
+      <c r="A7" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B7" s="33" t="s">
+        <v>1430</v>
+      </c>
+      <c r="C7" s="33"/>
+      <c r="D7" s="33"/>
+      <c r="E7" s="33"/>
+      <c r="F7" s="33"/>
+      <c r="G7" s="33"/>
+      <c r="J7" s="17" t="s">
+        <v>244</v>
+      </c>
+      <c r="K7" s="17" t="s">
+        <v>124</v>
+      </c>
+      <c r="L7" s="17" t="s">
+        <v>124</v>
+      </c>
+      <c r="M7" s="17" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="B9" s="32" t="s">
+        <v>73</v>
+      </c>
+      <c r="C9" s="32"/>
+      <c r="D9" s="32"/>
+      <c r="E9" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="F9" s="32" t="s">
+        <v>75</v>
+      </c>
+      <c r="G9" s="32" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" ht="46.5">
+      <c r="A10" s="32"/>
+      <c r="B10" s="15" t="s">
+        <v>1424</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>1425</v>
+      </c>
+      <c r="D10" s="15" t="s">
+        <v>1426</v>
+      </c>
+      <c r="E10" s="32"/>
+      <c r="F10" s="32"/>
+      <c r="G10" s="32"/>
+    </row>
+    <row r="11" spans="1:13">
+      <c r="A11" s="16" t="s">
+        <v>1431</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="E11" s="13" t="s">
+        <v>1432</v>
+      </c>
+      <c r="F11" s="13" t="s">
+        <v>1494</v>
+      </c>
+      <c r="G11" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" ht="46.5">
+      <c r="A12" s="16" t="s">
+        <v>1433</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>308</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>1434</v>
+      </c>
+      <c r="F12" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="G12" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13">
+      <c r="A13" s="16" t="s">
+        <v>1435</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="E13" s="13" t="s">
+        <v>1436</v>
+      </c>
+      <c r="F13" s="13" t="s">
+        <v>1494</v>
+      </c>
+      <c r="G13" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13">
+      <c r="A14" s="16" t="s">
+        <v>1437</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>714</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="D14" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="E14" s="13" t="s">
+        <v>1436</v>
+      </c>
+      <c r="F14" s="13" t="s">
+        <v>1494</v>
+      </c>
+      <c r="G14" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13">
+      <c r="A15" s="16" t="s">
+        <v>1438</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>1429</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>1436</v>
+      </c>
+      <c r="F15" s="13" t="s">
+        <v>1494</v>
+      </c>
+      <c r="G15" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13">
+      <c r="A16" s="16" t="s">
+        <v>1439</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="E16" s="13" t="s">
+        <v>1436</v>
+      </c>
+      <c r="F16" s="13" t="s">
+        <v>1494</v>
+      </c>
+      <c r="G16" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="46.5">
+      <c r="A17" s="16" t="s">
+        <v>1440</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="D17" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="E17" s="13" t="s">
+        <v>1434</v>
+      </c>
+      <c r="F17" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="G17" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="46.5">
+      <c r="A18" s="16" t="s">
+        <v>1441</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>308</v>
+      </c>
+      <c r="D18" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="E18" s="13" t="s">
+        <v>1442</v>
+      </c>
+      <c r="F18" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="G18" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" s="16" t="s">
+        <v>1443</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="D19" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="E19" s="13" t="s">
+        <v>1436</v>
+      </c>
+      <c r="F19" s="13" t="s">
+        <v>1494</v>
+      </c>
+      <c r="G19" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" s="16" t="s">
+        <v>1444</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>714</v>
+      </c>
+      <c r="D20" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>1436</v>
+      </c>
+      <c r="F20" s="13" t="s">
+        <v>1494</v>
+      </c>
+      <c r="G20" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" s="16" t="s">
+        <v>1445</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>1429</v>
+      </c>
+      <c r="D21" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="E21" s="13" t="s">
+        <v>1436</v>
+      </c>
+      <c r="F21" s="13" t="s">
+        <v>1494</v>
+      </c>
+      <c r="G21" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" s="16" t="s">
+        <v>1446</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="D22" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="E22" s="13" t="s">
+        <v>1436</v>
+      </c>
+      <c r="F22" s="13" t="s">
+        <v>1494</v>
+      </c>
+      <c r="G22" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="46.5">
+      <c r="A23" s="16" t="s">
+        <v>1447</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="D23" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="E23" s="13" t="s">
+        <v>1442</v>
+      </c>
+      <c r="F23" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="G23" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="46.5">
+      <c r="A24" s="16" t="s">
+        <v>1448</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="D24" s="13" t="s">
+        <v>308</v>
+      </c>
+      <c r="E24" s="13" t="s">
+        <v>1449</v>
+      </c>
+      <c r="F24" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="G24" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25" s="16" t="s">
+        <v>1450</v>
+      </c>
+      <c r="B25" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="D25" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="E25" s="13" t="s">
+        <v>1436</v>
+      </c>
+      <c r="F25" s="13" t="s">
+        <v>1494</v>
+      </c>
+      <c r="G25" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26" s="16" t="s">
+        <v>1451</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="D26" s="13" t="s">
+        <v>714</v>
+      </c>
+      <c r="E26" s="13" t="s">
+        <v>1436</v>
+      </c>
+      <c r="F26" s="13" t="s">
+        <v>1494</v>
+      </c>
+      <c r="G26" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="A27" s="16" t="s">
+        <v>1452</v>
+      </c>
+      <c r="B27" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="D27" s="13" t="s">
+        <v>1429</v>
+      </c>
+      <c r="E27" s="13" t="s">
+        <v>1436</v>
+      </c>
+      <c r="F27" s="13" t="s">
+        <v>1494</v>
+      </c>
+      <c r="G27" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="A28" s="16" t="s">
+        <v>1453</v>
+      </c>
+      <c r="B28" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="D28" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="E28" s="13" t="s">
+        <v>1436</v>
+      </c>
+      <c r="F28" s="13" t="s">
+        <v>1494</v>
+      </c>
+      <c r="G28" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="46.5">
+      <c r="A29" s="16" t="s">
+        <v>1454</v>
+      </c>
+      <c r="B29" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="C29" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="D29" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="E29" s="13" t="s">
+        <v>1449</v>
+      </c>
+      <c r="F29" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="G29" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="B7:G7"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="B6:G6"/>
+  </mergeCells>
+  <conditionalFormatting sqref="G11:G29">
+    <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
+      <formula>"Pass"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
+      <formula>"Fail"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
+      <formula>"Block"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" sqref="G11:G29" xr:uid="{FADC6F40-655C-429E-B827-530535B6F86D}">
+      <formula1>"Pass,Fail,No run,Block"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEC38A2E-1BE9-43B9-9B16-3CE4E06A3A66}">
+  <dimension ref="A1:I28"/>
+  <sheetFormatPr defaultColWidth="7.625" defaultRowHeight="23.25"/>
+  <cols>
+    <col min="1" max="1" width="19.25" style="8" customWidth="1"/>
+    <col min="2" max="3" width="21" style="8" customWidth="1"/>
+    <col min="4" max="4" width="40.25" style="8" customWidth="1"/>
+    <col min="5" max="5" width="33.25" style="8" customWidth="1"/>
+    <col min="6" max="6" width="14.875" style="8" customWidth="1"/>
+    <col min="7" max="8" width="12.25" style="8" customWidth="1"/>
+    <col min="9" max="9" width="15.875" style="8" customWidth="1"/>
+    <col min="10" max="16384" width="7.625" style="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="24" thickBot="1">
+      <c r="A1" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+    </row>
+    <row r="2" spans="1:9" ht="24" thickBot="1">
+      <c r="A2" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" s="28" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" s="28"/>
+    </row>
+    <row r="3" spans="1:9" ht="24" thickBot="1">
+      <c r="A3" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="29" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="29"/>
+      <c r="E3" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="29" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" s="29"/>
+      <c r="H3" s="29"/>
+      <c r="I3" s="29"/>
+    </row>
+    <row r="4" spans="1:9" ht="24" thickBot="1">
+      <c r="A4" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="30" t="s">
+        <v>1455</v>
+      </c>
+      <c r="C4" s="30"/>
+      <c r="E4" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="30" t="s">
+        <v>871</v>
+      </c>
+      <c r="G4" s="30"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="30"/>
+    </row>
+    <row r="5" spans="1:9" ht="24" thickBot="1">
+      <c r="A5" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="30" t="s">
+        <v>1456</v>
+      </c>
+      <c r="C5" s="30"/>
+      <c r="E5" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" s="30" t="s">
+        <v>1457</v>
+      </c>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+    </row>
+    <row r="6" spans="1:9" ht="24" thickBot="1">
+      <c r="A6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="30" t="s">
+        <v>1458</v>
+      </c>
+      <c r="C6" s="30"/>
+      <c r="E6" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="F6" s="30" t="s">
+        <v>1459</v>
+      </c>
+      <c r="G6" s="30"/>
+      <c r="H6" s="30"/>
+      <c r="I6" s="30"/>
+    </row>
+    <row r="7" spans="1:9" ht="24" thickBot="1">
+      <c r="A7" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="30" t="s">
+        <v>1460</v>
+      </c>
+      <c r="C7" s="30"/>
+      <c r="E7" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" s="30" t="s">
+        <v>1461</v>
+      </c>
+      <c r="G7" s="30"/>
+      <c r="H7" s="30"/>
+      <c r="I7" s="30"/>
+    </row>
+    <row r="8" spans="1:9" ht="24" thickBot="1">
+      <c r="A8" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" s="30" t="s">
+        <v>1462</v>
+      </c>
+      <c r="C8" s="30"/>
+      <c r="E8" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="F8" s="30" t="s">
+        <v>1463</v>
+      </c>
+      <c r="G8" s="30"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="30"/>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" s="31" t="s">
+        <v>57</v>
+      </c>
+      <c r="B10" s="31"/>
+      <c r="C10" s="31"/>
+      <c r="D10" s="31"/>
+      <c r="E10" s="31"/>
+      <c r="F10" s="31"/>
+      <c r="G10" s="31"/>
+      <c r="H10" s="31"/>
+      <c r="I10" s="31"/>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B12" s="33" t="s">
+        <v>1464</v>
+      </c>
+      <c r="C12" s="33"/>
+      <c r="D12" s="33"/>
+      <c r="E12" s="21"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="21"/>
+      <c r="H12" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="I12" s="14" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="B13" s="33" t="s">
+        <v>62</v>
+      </c>
+      <c r="C13" s="33"/>
+      <c r="D13" s="33"/>
+      <c r="E13" s="21"/>
+      <c r="F13" s="21"/>
+      <c r="G13" s="21"/>
+      <c r="H13" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="I13" s="14" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="46.5">
+      <c r="A14" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B14" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="C14" s="33"/>
+      <c r="D14" s="33"/>
+      <c r="E14" s="21"/>
+      <c r="F14" s="21"/>
+      <c r="G14" s="21"/>
+      <c r="H14" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="I14" s="13" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="46.5">
+      <c r="A15" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="B15" s="33" t="s">
+        <v>1465</v>
+      </c>
+      <c r="C15" s="33"/>
+      <c r="D15" s="33"/>
+      <c r="E15" s="33"/>
+      <c r="F15" s="33"/>
+      <c r="G15" s="33"/>
+      <c r="H15" s="33"/>
+      <c r="I15" s="33"/>
+    </row>
+    <row r="16" spans="1:9" ht="46.5">
+      <c r="A16" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B16" s="33" t="s">
+        <v>1466</v>
+      </c>
+      <c r="C16" s="33"/>
+      <c r="D16" s="33"/>
+      <c r="E16" s="33"/>
+      <c r="F16" s="33"/>
+      <c r="G16" s="33"/>
+      <c r="H16" s="33"/>
+      <c r="I16" s="33"/>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="B18" s="32" t="s">
+        <v>73</v>
+      </c>
+      <c r="C18" s="32"/>
+      <c r="D18" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="E18" s="32" t="s">
+        <v>75</v>
+      </c>
+      <c r="F18" s="32" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" s="32"/>
+      <c r="B19" s="15" t="s">
+        <v>1467</v>
+      </c>
+      <c r="C19" s="15" t="s">
+        <v>1468</v>
+      </c>
+      <c r="D19" s="32"/>
+      <c r="E19" s="32"/>
+      <c r="F19" s="32"/>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20" s="16" t="s">
+        <v>1469</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>1470</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>1471</v>
+      </c>
+      <c r="D20" s="13" t="s">
+        <v>1472</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>1495</v>
+      </c>
+      <c r="F20" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21" s="16" t="s">
+        <v>1473</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>1470</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>1474</v>
+      </c>
+      <c r="D21" s="13" t="s">
+        <v>1475</v>
+      </c>
+      <c r="E21" s="13" t="s">
+        <v>1496</v>
+      </c>
+      <c r="F21" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" s="16" t="s">
+        <v>1476</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>1470</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>1032</v>
+      </c>
+      <c r="D22" s="13" t="s">
+        <v>1477</v>
+      </c>
+      <c r="E22" s="13" t="s">
+        <v>1497</v>
+      </c>
+      <c r="F22" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="46.5">
+      <c r="A23" s="16" t="s">
+        <v>1478</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>1470</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>1479</v>
+      </c>
+      <c r="D23" s="13" t="s">
+        <v>1480</v>
+      </c>
+      <c r="E23" s="13" t="s">
+        <v>1498</v>
+      </c>
+      <c r="F23" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="46.5">
+      <c r="A24" s="16" t="s">
+        <v>1481</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>1482</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="D24" s="13" t="s">
+        <v>1483</v>
+      </c>
+      <c r="E24" s="13" t="s">
+        <v>1495</v>
+      </c>
+      <c r="F24" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
+      <c r="A25" s="16" t="s">
+        <v>1484</v>
+      </c>
+      <c r="B25" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="D25" s="13" t="s">
+        <v>780</v>
+      </c>
+      <c r="E25" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="F25" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="46.5">
+      <c r="A26" s="16" t="s">
+        <v>1485</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>1486</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="D26" s="13" t="s">
+        <v>1487</v>
+      </c>
+      <c r="E26" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="F26" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="46.5">
+      <c r="A27" s="16" t="s">
+        <v>1488</v>
+      </c>
+      <c r="B27" s="13" t="s">
+        <v>1489</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="D27" s="13" t="s">
+        <v>1490</v>
+      </c>
+      <c r="E27" s="13" t="s">
+        <v>201</v>
+      </c>
+      <c r="F27" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28" s="16" t="s">
+        <v>1491</v>
+      </c>
+      <c r="B28" s="13" t="s">
+        <v>1470</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>1492</v>
+      </c>
+      <c r="D28" s="13" t="s">
+        <v>1493</v>
+      </c>
+      <c r="E28" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="F28" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="25">
+    <mergeCell ref="B15:I15"/>
+    <mergeCell ref="B16:I16"/>
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="E18:E19"/>
+    <mergeCell ref="F18:F19"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="F8:I8"/>
+    <mergeCell ref="A10:I10"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="F5:I5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="F6:I6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="F7:I7"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="F3:I3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="F4:I4"/>
+  </mergeCells>
+  <conditionalFormatting sqref="F20:F28">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
@@ -17087,7 +18683,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="H27:H34" xr:uid="{20B1E575-5034-4BD5-B1D2-38BFE4D9AB36}">
+    <dataValidation type="list" allowBlank="1" sqref="F20:F28" xr:uid="{06F4C052-ED6E-47F6-BD02-3591D8C98550}">
       <formula1>"Pass,Fail,No run,Block"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -18012,13 +19608,13 @@
     <mergeCell ref="G4:J4"/>
   </mergeCells>
   <conditionalFormatting sqref="J28:J42">
-    <cfRule type="cellIs" dxfId="71" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="77" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="70" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="76" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="69" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="75" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -18826,13 +20422,13 @@
     <mergeCell ref="H27:H28"/>
   </mergeCells>
   <conditionalFormatting sqref="H29:H38">
-    <cfRule type="cellIs" dxfId="68" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="74" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="67" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="73" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="66" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="72" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -19361,13 +20957,13 @@
     <mergeCell ref="B6:G6"/>
   </mergeCells>
   <conditionalFormatting sqref="G11:G23">
-    <cfRule type="cellIs" dxfId="65" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="71" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="64" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="70" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="63" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="69" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -19957,13 +21553,13 @@
     <mergeCell ref="H9:H10"/>
   </mergeCells>
   <conditionalFormatting sqref="H11:H23">
-    <cfRule type="cellIs" dxfId="62" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="68" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="61" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="67" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="60" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="66" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -20982,13 +22578,13 @@
     <mergeCell ref="I32:I33"/>
   </mergeCells>
   <conditionalFormatting sqref="I34:I45">
-    <cfRule type="cellIs" dxfId="59" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="65" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="58" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="64" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="57" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="63" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -21281,13 +22877,13 @@
     <mergeCell ref="F9:F10"/>
   </mergeCells>
   <conditionalFormatting sqref="F11:F15">
-    <cfRule type="cellIs" dxfId="56" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="62" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="55" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="61" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="54" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="60" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -21899,13 +23495,13 @@
     <mergeCell ref="G23:G24"/>
   </mergeCells>
   <conditionalFormatting sqref="G25:G32">
-    <cfRule type="cellIs" dxfId="53" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="59" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="52" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="58" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="51" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="57" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Unit Test Admin resources
</commit_message>
<xml_diff>
--- a/test/FIWDEE_UnitTest_Report.xlsx
+++ b/test/FIWDEE_UnitTest_Report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\ProjectPOS\FIWDEE-CP353002-69_1PrinciplesOfSoftwareDesign\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38627A56-1F1B-4CC0-BFC1-A92AEB730A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFFDC2FB-1484-4930-88A0-00A0B7D2C7C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="10" xr2:uid="{9B0ECA1C-B255-4EEE-B7A8-035645CFC3D9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9B0ECA1C-B255-4EEE-B7A8-035645CFC3D9}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Summary" sheetId="1" r:id="rId1"/>
@@ -46,9 +46,13 @@
     <sheet name="UT29_UpdateProfile_DT" sheetId="33" r:id="rId31"/>
     <sheet name="UT30_UserSession_BVA" sheetId="34" r:id="rId32"/>
     <sheet name="UT31_JwtToken_EC" sheetId="35" r:id="rId33"/>
+    <sheet name="UT32_RoomService_EC" sheetId="36" r:id="rId34"/>
+    <sheet name="UT33_ServiceCatalog_EC" sheetId="37" r:id="rId35"/>
+    <sheet name="UT34_Schedule_Shift_BVA" sheetId="39" r:id="rId36"/>
+    <sheet name="UT35_ShopHours_BVA" sheetId="38" r:id="rId37"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId34"/>
+    <externalReference r:id="rId38"/>
   </externalReferences>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -96,7 +100,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4506" uniqueCount="1674">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4894" uniqueCount="1832">
   <si>
     <t>FIWDEE – Unit Test Design</t>
   </si>
@@ -5118,6 +5122,480 @@
   </si>
   <si>
     <t>false ไม่โยน Exception</t>
+  </si>
+  <si>
+    <t>Admin resources</t>
+  </si>
+  <si>
+    <t>UT32 – RoomServiceImpl</t>
+  </si>
+  <si>
+    <t>UT33 – ServiceCatalogServiceImpl</t>
+  </si>
+  <si>
+    <t>Weak Robust Equivalence Class Testing (ใช้ค่าขอบเป็นตัวแทนคลาส)</t>
+  </si>
+  <si>
+    <t>UT34 – TherapistServiceImpl.updateSchedule – กะทำงาน</t>
+  </si>
+  <si>
+    <t>UT35 – ShopServiceImpl.updateShop – เวลาเปิด–ปิด</t>
+  </si>
+  <si>
+    <t>เลขห้องใหม่ไม่ซ้ำ</t>
+  </si>
+  <si>
+    <t>เลขห้องซ้ำ (ต่างตัวพิมพ์)</t>
+  </si>
+  <si>
+    <t>แก้ไขห้องโดยใช้เลขเดิมของตัวเอง</t>
+  </si>
+  <si>
+    <t>แก้เป็นเลขของห้องอื่น</t>
+  </si>
+  <si>
+    <t>ลบ = ปิดใช้งาน</t>
+  </si>
+  <si>
+    <t>id ไม่มีอยู่</t>
+  </si>
+  <si>
+    <t>getRooms(activeOnly = true)</t>
+  </si>
+  <si>
+    <t>RoomServiceImpl</t>
+  </si>
+  <si>
+    <t>createRoom, updateRoom, deleteRoom, getRooms</t>
+  </si>
+  <si>
+    <t>UC-24 • BR-RES-01</t>
+  </si>
+  <si>
+    <t>UT32-TC001</t>
+  </si>
+  <si>
+    <t>createRoom</t>
+  </si>
+  <si>
+    <t>" R104 ", SINGLE, 1, 15</t>
+  </si>
+  <si>
+    <t>(V1) save: roomNumber "R104", AVAILABLE, isActive true</t>
+  </si>
+  <si>
+    <t>UT32-TC002</t>
+  </si>
+  <si>
+    <t>updateRoom(101)</t>
+  </si>
+  <si>
+    <t>"R101", VIP, 2, 20</t>
+  </si>
+  <si>
+    <t>(V2) สำเร็จ roomType VIP</t>
+  </si>
+  <si>
+    <t>UT32-TC003</t>
+  </si>
+  <si>
+    <t>deleteRoom(102)</t>
+  </si>
+  <si>
+    <t>(V3) isActive = false และ save (ไม่ลบจริง)</t>
+  </si>
+  <si>
+    <t>UT32-TC004</t>
+  </si>
+  <si>
+    <t>getRooms(true)</t>
+  </si>
+  <si>
+    <t>(V4) เรียก findByIsActiveTrue ไม่เรียก findAll</t>
+  </si>
+  <si>
+    <t>UT32-TC005</t>
+  </si>
+  <si>
+    <t>"r101"</t>
+  </si>
+  <si>
+    <t>(I1) ConflictException "Room number already exists"</t>
+  </si>
+  <si>
+    <t>UT32-TC006</t>
+  </si>
+  <si>
+    <t>"R102"</t>
+  </si>
+  <si>
+    <t>(I2) ConflictException</t>
+  </si>
+  <si>
+    <t>UT32-TC007</t>
+  </si>
+  <si>
+    <t>updateRoom(999) / deleteRoom(999)</t>
+  </si>
+  <si>
+    <t>(I3) NotFoundException</t>
+  </si>
+  <si>
+    <t>รหัสใหม่ + option อย่างน้อย 1 รายการ</t>
+  </si>
+  <si>
+    <t>durationOptions ว่างหรือ null</t>
+  </si>
+  <si>
+    <t>duration = 1 (ค่าบวกต่ำสุด)</t>
+  </si>
+  <si>
+    <t>duration ≤ 0</t>
+  </si>
+  <si>
+    <t>price = 0.00</t>
+  </si>
+  <si>
+    <t>price &lt; 0</t>
+  </si>
+  <si>
+    <t>update ด้วยรหัสเดิมของตัวเอง</t>
+  </si>
+  <si>
+    <t>รหัสซ้ำ (ต่างตัวพิมพ์)</t>
+  </si>
+  <si>
+    <t>getActiveService ของบริการที่ปิดอยู่</t>
+  </si>
+  <si>
+    <t>ServiceCatalogServiceImpl</t>
+  </si>
+  <si>
+    <t>Functional testing - Weak Robust Equivalence Class Testing (ใช้ค่าขอบเป็นตัวแทนคลาส)</t>
+  </si>
+  <si>
+    <t>createService, updateService, getActiveService, deleteService</t>
+  </si>
+  <si>
+    <t>UC-25 • SRS 6.3</t>
+  </si>
+  <si>
+    <t>serviceCode</t>
+  </si>
+  <si>
+    <t>durationOptions</t>
+  </si>
+  <si>
+    <t>UT33-TC001</t>
+  </si>
+  <si>
+    <t>createService</t>
+  </si>
+  <si>
+    <t>AROMA-01</t>
+  </si>
+  <si>
+    <t>[60/800]</t>
+  </si>
+  <si>
+    <t>(V1) save, isActive true, option 1 รายการ active</t>
+  </si>
+  <si>
+    <t>UT33-TC002</t>
+  </si>
+  <si>
+    <t>AROMA-02</t>
+  </si>
+  <si>
+    <t>[1/800]</t>
+  </si>
+  <si>
+    <t>(V2) สำเร็จ</t>
+  </si>
+  <si>
+    <t>UT33-TC003</t>
+  </si>
+  <si>
+    <t>AROMA-03</t>
+  </si>
+  <si>
+    <t>[60/0.00]</t>
+  </si>
+  <si>
+    <t>(V3) สำเร็จ</t>
+  </si>
+  <si>
+    <t>UT33-TC004</t>
+  </si>
+  <si>
+    <t>updateService(1)</t>
+  </si>
+  <si>
+    <t>thai-01</t>
+  </si>
+  <si>
+    <t>[60/600, 90/850]</t>
+  </si>
+  <si>
+    <t>(V4) สำเร็จ option ถูกแทนที่เป็น 2 รายการ</t>
+  </si>
+  <si>
+    <t>UT33-TC005</t>
+  </si>
+  <si>
+    <t>AROMA-04</t>
+  </si>
+  <si>
+    <t>[] และ null</t>
+  </si>
+  <si>
+    <t>(I1) ValidationException "At least one duration option is required"</t>
+  </si>
+  <si>
+    <t>UT33-TC006</t>
+  </si>
+  <si>
+    <t>AROMA-05</t>
+  </si>
+  <si>
+    <t>[0/800] และ [-1/800]</t>
+  </si>
+  <si>
+    <t>(I2) ValidationException</t>
+  </si>
+  <si>
+    <t>UT33-TC007</t>
+  </si>
+  <si>
+    <t>AROMA-06</t>
+  </si>
+  <si>
+    <t>[60/-0.01]</t>
+  </si>
+  <si>
+    <t>(I3) ValidationException</t>
+  </si>
+  <si>
+    <t>UT33-TC008</t>
+  </si>
+  <si>
+    <t>[60/600]</t>
+  </si>
+  <si>
+    <t>(I4) ConflictException "Service code already exists"</t>
+  </si>
+  <si>
+    <t>UT33-TC009</t>
+  </si>
+  <si>
+    <t>getActiveService(3)</t>
+  </si>
+  <si>
+    <t>บริการ 3 inactive</t>
+  </si>
+  <si>
+    <t>ความยาวกะ (นาที)</t>
+  </si>
+  <si>
+    <t>ช่องว่างระหว่างกะ (นาที)</t>
+  </si>
+  <si>
+    <t>TherapistServiceImpl.updateSchedule – กะทำงาน</t>
+  </si>
+  <si>
+    <t>480</t>
+  </si>
+  <si>
+    <t>60</t>
+  </si>
+  <si>
+    <t>updateSchedule(therapistId, request) → validateShifts: end &gt; start และกะต้องไม่ทับกัน</t>
+  </si>
+  <si>
+    <t>UC-27 • SRS 6.4 (Work Shifts)</t>
+  </si>
+  <si>
+    <t>dayOff</t>
+  </si>
+  <si>
+    <t>shifts</t>
+  </si>
+  <si>
+    <t>UT34-TC001</t>
+  </si>
+  <si>
+    <t>[10:00–18:00]</t>
+  </si>
+  <si>
+    <t>บันทึก 1 กะ ชื่อ "Shift", status ACTIVE (nom)</t>
+  </si>
+  <si>
+    <t>UT34-TC002</t>
+  </si>
+  <si>
+    <t>[10:00–10:00]</t>
+  </si>
+  <si>
+    <t>ValidationException "Shift end time must be after start time"</t>
+  </si>
+  <si>
+    <t>UT34-TC003</t>
+  </si>
+  <si>
+    <t>[10:00–10:01]</t>
+  </si>
+  <si>
+    <t>UT34-TC004</t>
+  </si>
+  <si>
+    <t>[10:00–10:02]</t>
+  </si>
+  <si>
+    <t>UT34-TC005</t>
+  </si>
+  <si>
+    <t>[10:00–14:00, 13:59–18:00]</t>
+  </si>
+  <si>
+    <t>ValidationException "Work shifts must not overlap"</t>
+  </si>
+  <si>
+    <t>UT34-TC006</t>
+  </si>
+  <si>
+    <t>[10:00–14:00, 14:00–18:00]</t>
+  </si>
+  <si>
+    <t>บันทึก 2 กะ</t>
+  </si>
+  <si>
+    <t>UT34-TC007</t>
+  </si>
+  <si>
+    <t>[10:00–14:00, 14:01–18:00]</t>
+  </si>
+  <si>
+    <t>UT34-TC008</t>
+  </si>
+  <si>
+    <t>[15:00–18:00, 10:00–14:00] (ไม่เรียงเวลา)</t>
+  </si>
+  <si>
+    <t>บันทึกสำเร็จ (โค้ดเรียงก่อนตรวจ)</t>
+  </si>
+  <si>
+    <t>UT34-TC009</t>
+  </si>
+  <si>
+    <t>ValidationException "Day-off schedules cannot contain work shifts"</t>
+  </si>
+  <si>
+    <t>UT34-TC010</t>
+  </si>
+  <si>
+    <t>[]</t>
+  </si>
+  <si>
+    <t>บันทึกวันหยุด ไม่มีกะ</t>
+  </si>
+  <si>
+    <t>closeTime − openTime (นาที)</t>
+  </si>
+  <si>
+    <t>ShopServiceImpl.updateShop – เวลาเปิด–ปิด</t>
+  </si>
+  <si>
+    <t>updateShop(request) : ถ้าไม่ปิด closeTime ต้องหลัง openTime, วันห้ามซ้ำ, ต้องมีอย่างน้อย 1 วัน</t>
+  </si>
+  <si>
+    <t>UC-23 / SRS 6 (เวลาทำการ) • BR-BKG-02</t>
+  </si>
+  <si>
+    <t>businessHours</t>
+  </si>
+  <si>
+    <t>closed</t>
+  </si>
+  <si>
+    <t>UT35-TC001</t>
+  </si>
+  <si>
+    <t>MONDAY 10:00–22:00</t>
+  </si>
+  <si>
+    <t>บันทึกสำเร็จ (nom)</t>
+  </si>
+  <si>
+    <t>UT35-TC002</t>
+  </si>
+  <si>
+    <t>MONDAY 10:00–09:59</t>
+  </si>
+  <si>
+    <t>ValidationException "Closing time must be after opening time"</t>
+  </si>
+  <si>
+    <t>UT35-TC003</t>
+  </si>
+  <si>
+    <t>MONDAY 10:00–10:00</t>
+  </si>
+  <si>
+    <t>UT35-TC004</t>
+  </si>
+  <si>
+    <t>MONDAY 10:00–10:01</t>
+  </si>
+  <si>
+    <t>UT35-TC005</t>
+  </si>
+  <si>
+    <t>SUNDAY 10:00–09:00</t>
+  </si>
+  <si>
+    <t>บันทึกสำเร็จ (วันปิดไม่ตรวจเวลา)</t>
+  </si>
+  <si>
+    <t>UT35-TC006</t>
+  </si>
+  <si>
+    <t>MONDAY 2 แถว</t>
+  </si>
+  <si>
+    <t>ValidationException "Duplicate business hours day: MONDAY"</t>
+  </si>
+  <si>
+    <t>UT35-TC007</t>
+  </si>
+  <si>
+    <t>[] (ว่าง)</t>
+  </si>
+  <si>
+    <t>ValidationException "Business hours for the week are required"</t>
+  </si>
+  <si>
+    <t>UT35-TC008</t>
+  </si>
+  <si>
+    <t>ไม่มีร้าน active</t>
+  </si>
+  <si>
+    <t>save: roomNumber "R104", AVAILABLE, isActive true</t>
+  </si>
+  <si>
+    <t>สำเร็จ roomType VIP</t>
+  </si>
+  <si>
+    <t>isActive = false และ save</t>
+  </si>
+  <si>
+    <t>เรียก findByIsActiveTrue ไม่เรียก findAl</t>
+  </si>
+  <si>
+    <t>save, isActive true, option 1 รายการ active</t>
+  </si>
+  <si>
+    <t>บันทึก 1 กะ ชื่อ "Shift", status ACTIVE</t>
   </si>
 </sst>
 </file>
@@ -5463,7 +5941,91 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="93">
+  <dxfs count="105">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -6591,7 +7153,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{659A469D-55E7-4F16-B797-78C1D60B492C}">
-  <dimension ref="A1:I40"/>
+  <dimension ref="A1:I45"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="1" width="5.25" customWidth="1"/>
@@ -7729,36 +8291,177 @@
       <c r="I39" s="4"/>
     </row>
     <row r="40" spans="1:9" ht="21">
-      <c r="A40" s="24" t="s">
+      <c r="A40" s="26" t="s">
+        <v>1674</v>
+      </c>
+      <c r="B40" s="26"/>
+      <c r="C40" s="26"/>
+      <c r="D40" s="26"/>
+      <c r="E40" s="26"/>
+      <c r="F40" s="26"/>
+      <c r="G40" s="26"/>
+      <c r="H40" s="26"/>
+      <c r="I40" s="26"/>
+    </row>
+    <row r="41" spans="1:9" ht="21">
+      <c r="A41" s="3">
+        <v>32</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>1675</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D41" s="3">
+        <f>COUNTA(UT32_RoomService_EC!$A$20:$A$26)</f>
+        <v>6</v>
+      </c>
+      <c r="E41" s="3">
+        <f>COUNTIF(UT32_RoomService_EC!$F$20:$F$26,"Pass")</f>
+        <v>6</v>
+      </c>
+      <c r="F41" s="3">
+        <f>COUNTIF(UT32_RoomService_EC!$F$20:$F$26,"Fail")</f>
+        <v>0</v>
+      </c>
+      <c r="G41" s="3">
+        <f>COUNTIF(UT32_RoomService_EC!$F$20:$F$26,"No run")</f>
+        <v>0</v>
+      </c>
+      <c r="H41" s="3">
+        <f>COUNTIF(UT32_RoomService_EC!$F$20:$F$26,"Block")</f>
+        <v>0</v>
+      </c>
+      <c r="I41" s="4"/>
+    </row>
+    <row r="42" spans="1:9" ht="42">
+      <c r="A42" s="3">
+        <v>33</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>1676</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>1677</v>
+      </c>
+      <c r="D42" s="3">
+        <f>COUNTA(UT33_ServiceCatalog_EC!$A$21:$A$29)</f>
+        <v>8</v>
+      </c>
+      <c r="E42" s="3">
+        <f>COUNTIF(UT33_ServiceCatalog_EC!$G$21:$G$29,"Pass")</f>
+        <v>8</v>
+      </c>
+      <c r="F42" s="3">
+        <f>COUNTIF(UT33_ServiceCatalog_EC!$G$21:$G$29,"Fail")</f>
+        <v>0</v>
+      </c>
+      <c r="G42" s="3">
+        <f>COUNTIF(UT33_ServiceCatalog_EC!$G$21:$G$29,"No run")</f>
+        <v>0</v>
+      </c>
+      <c r="H42" s="3">
+        <f>COUNTIF(UT33_ServiceCatalog_EC!$G$21:$G$29,"Block")</f>
+        <v>0</v>
+      </c>
+      <c r="I42" s="4"/>
+    </row>
+    <row r="43" spans="1:9" ht="21">
+      <c r="A43" s="3">
+        <v>34</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>1678</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>451</v>
+      </c>
+      <c r="D43" s="3">
+        <f>COUNTA(UT34_Schedule_Shift_BVA!$A$12:$A$21)</f>
+        <v>9</v>
+      </c>
+      <c r="E43" s="3">
+        <f>COUNTIF(UT34_Schedule_Shift_BVA!$F$12:$F$21,"Pass")</f>
+        <v>9</v>
+      </c>
+      <c r="F43" s="3">
+        <f>COUNTIF(UT34_Schedule_Shift_BVA!$F$12:$F$21,"Fail")</f>
+        <v>0</v>
+      </c>
+      <c r="G43" s="3">
+        <f>COUNTIF(UT34_Schedule_Shift_BVA!$F$12:$F$21,"No run")</f>
+        <v>0</v>
+      </c>
+      <c r="H43" s="3">
+        <f>COUNTIF(UT34_Schedule_Shift_BVA!$F$12:$F$21,"Block")</f>
+        <v>0</v>
+      </c>
+      <c r="I43" s="4"/>
+    </row>
+    <row r="44" spans="1:9" ht="21">
+      <c r="A44" s="3">
+        <v>35</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>1679</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>451</v>
+      </c>
+      <c r="D44" s="3">
+        <f>COUNTA(UT35_ShopHours_BVA!$A$12:$A$19)</f>
+        <v>7</v>
+      </c>
+      <c r="E44" s="3">
+        <f>COUNTIF(UT35_ShopHours_BVA!$F$12:$F$19,"Pass")</f>
+        <v>7</v>
+      </c>
+      <c r="F44" s="3">
+        <f>COUNTIF(UT35_ShopHours_BVA!$F$12:$F$19,"Fail")</f>
+        <v>0</v>
+      </c>
+      <c r="G44" s="3">
+        <f>COUNTIF(UT35_ShopHours_BVA!$F$12:$F$19,"No run")</f>
+        <v>0</v>
+      </c>
+      <c r="H44" s="3">
+        <f>COUNTIF(UT35_ShopHours_BVA!$F$12:$F$19,"Block")</f>
+        <v>0</v>
+      </c>
+      <c r="I44" s="4"/>
+    </row>
+    <row r="45" spans="1:9" ht="21">
+      <c r="A45" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="B40" s="24"/>
-      <c r="C40" s="24"/>
-      <c r="D40" s="5" cm="1">
-        <f t="array" ref="D40">SUMPRODUCT(ISNUMBER(D4:D39)*D4:D39)</f>
-        <v>320</v>
-      </c>
-      <c r="E40" s="6" cm="1">
-        <f t="array" ref="E40">SUMPRODUCT(ISNUMBER(E4:E39)*E4:E39)</f>
-        <v>308</v>
-      </c>
-      <c r="F40" s="7" cm="1">
-        <f t="array" ref="F40">SUMPRODUCT(ISNUMBER(F4:F39)*F4:F39)</f>
+      <c r="B45" s="24"/>
+      <c r="C45" s="24"/>
+      <c r="D45" s="5" cm="1">
+        <f t="array" ref="D45">SUMPRODUCT(ISNUMBER(D4:D44)*D4:D44)</f>
+        <v>350</v>
+      </c>
+      <c r="E45" s="6" cm="1">
+        <f t="array" ref="E45">SUMPRODUCT(ISNUMBER(E4:E44)*E4:E44)</f>
+        <v>338</v>
+      </c>
+      <c r="F45" s="7" cm="1">
+        <f t="array" ref="F45">SUMPRODUCT(ISNUMBER(F4:F44)*F4:F44)</f>
         <v>12</v>
       </c>
-      <c r="G40" s="5" cm="1">
-        <f t="array" ref="G40">SUMPRODUCT(ISNUMBER(G4:G39)*G4:G39)</f>
+      <c r="G45" s="5" cm="1">
+        <f t="array" ref="G45">SUMPRODUCT(ISNUMBER(G4:G44)*G4:G44)</f>
         <v>0</v>
       </c>
-      <c r="H40" s="5" cm="1">
-        <f t="array" ref="H40">SUMPRODUCT(ISNUMBER(H4:H39)*H4:H39)</f>
+      <c r="H45" s="5" cm="1">
+        <f t="array" ref="H45">SUMPRODUCT(ISNUMBER(H4:H44)*H4:H44)</f>
         <v>0</v>
       </c>
-      <c r="I40" s="4"/>
+      <c r="I45" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A40:C40"/>
+  <mergeCells count="9">
+    <mergeCell ref="A45:C45"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="A16:I16"/>
@@ -7766,6 +8469,7 @@
     <mergeCell ref="A26:I26"/>
     <mergeCell ref="A31:I31"/>
     <mergeCell ref="A34:I34"/>
+    <mergeCell ref="A40:I40"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -9439,13 +10143,13 @@
     <mergeCell ref="B26:H26"/>
   </mergeCells>
   <conditionalFormatting sqref="H30:H74">
-    <cfRule type="cellIs" dxfId="71" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="83" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="70" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="82" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="69" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="81" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9884,13 +10588,13 @@
     <mergeCell ref="E21:E22"/>
   </mergeCells>
   <conditionalFormatting sqref="E23:E30">
-    <cfRule type="cellIs" dxfId="68" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="80" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="67" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="79" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="66" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="78" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10220,13 +10924,13 @@
     <mergeCell ref="B7:E7"/>
   </mergeCells>
   <conditionalFormatting sqref="E12:E19">
-    <cfRule type="cellIs" dxfId="65" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="77" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="64" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="76" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="63" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="75" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10765,13 +11469,13 @@
     <mergeCell ref="F4:I4"/>
   </mergeCells>
   <conditionalFormatting sqref="G23:G31">
-    <cfRule type="cellIs" dxfId="62" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="74" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="61" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="73" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="60" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="72" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11229,13 +11933,13 @@
     <mergeCell ref="F4:I4"/>
   </mergeCells>
   <conditionalFormatting sqref="F22:F29">
-    <cfRule type="cellIs" dxfId="59" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="71" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="58" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="70" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="57" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="69" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11990,13 +12694,13 @@
     <mergeCell ref="B24:I24"/>
   </mergeCells>
   <conditionalFormatting sqref="H29:H36">
-    <cfRule type="cellIs" dxfId="56" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="68" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="55" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="67" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="54" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="66" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12581,13 +13285,13 @@
     <mergeCell ref="F4:I4"/>
   </mergeCells>
   <conditionalFormatting sqref="G22:G32">
-    <cfRule type="cellIs" dxfId="53" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="65" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="52" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="64" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="51" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="63" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13087,13 +13791,13 @@
     <mergeCell ref="B6:F6"/>
   </mergeCells>
   <conditionalFormatting sqref="F11:F24">
-    <cfRule type="cellIs" dxfId="50" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="62" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="49" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="61" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="48" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="60" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13570,13 +14274,13 @@
     <mergeCell ref="F4:I4"/>
   </mergeCells>
   <conditionalFormatting sqref="F19:F27">
-    <cfRule type="cellIs" dxfId="47" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="59" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="46" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="58" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="45" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="57" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -14030,13 +14734,13 @@
     <mergeCell ref="F4:I4"/>
   </mergeCells>
   <conditionalFormatting sqref="F19:F26">
-    <cfRule type="cellIs" dxfId="44" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="56" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="43" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="55" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="42" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="54" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -14943,13 +15647,13 @@
     <mergeCell ref="F4:I4"/>
   </mergeCells>
   <conditionalFormatting sqref="F20:F29">
-    <cfRule type="cellIs" dxfId="41" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="53" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="52" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="39" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="51" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -15259,13 +15963,13 @@
     <mergeCell ref="B6:E6"/>
   </mergeCells>
   <conditionalFormatting sqref="E11:E17">
-    <cfRule type="cellIs" dxfId="38" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="50" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="49" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="36" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="48" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -15787,13 +16491,13 @@
     <mergeCell ref="F4:I4"/>
   </mergeCells>
   <conditionalFormatting sqref="F21:F30">
-    <cfRule type="cellIs" dxfId="35" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="47" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="34" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="46" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="33" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="45" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -16106,13 +16810,13 @@
     <mergeCell ref="B6:F6"/>
   </mergeCells>
   <conditionalFormatting sqref="F11:F16">
-    <cfRule type="cellIs" dxfId="32" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="44" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="31" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="43" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="42" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -16629,13 +17333,13 @@
     <mergeCell ref="F4:I4"/>
   </mergeCells>
   <conditionalFormatting sqref="F21:F30">
-    <cfRule type="cellIs" dxfId="29" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="41" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="40" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="27" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="39" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -17647,13 +18351,13 @@
     <mergeCell ref="B22:E22"/>
   </mergeCells>
   <conditionalFormatting sqref="G28:G53">
-    <cfRule type="cellIs" dxfId="26" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="38" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="37" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="36" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -18283,13 +18987,13 @@
     <mergeCell ref="B21:F21"/>
   </mergeCells>
   <conditionalFormatting sqref="H27:H34">
-    <cfRule type="cellIs" dxfId="23" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="35" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="34" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="33" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -18977,13 +19681,13 @@
     <mergeCell ref="B6:G6"/>
   </mergeCells>
   <conditionalFormatting sqref="G11:G29">
-    <cfRule type="cellIs" dxfId="20" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="32" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="19" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="31" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="30" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -19481,13 +20185,13 @@
     <mergeCell ref="F4:I4"/>
   </mergeCells>
   <conditionalFormatting sqref="F20:F28">
-    <cfRule type="cellIs" dxfId="17" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="29" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="28" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="27" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -19966,13 +20670,13 @@
     <mergeCell ref="B16:H16"/>
   </mergeCells>
   <conditionalFormatting sqref="H21:H27">
-    <cfRule type="cellIs" dxfId="14" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="26" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="25" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="24" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -20902,13 +21606,13 @@
     <mergeCell ref="G4:J4"/>
   </mergeCells>
   <conditionalFormatting sqref="J28:J42">
-    <cfRule type="cellIs" dxfId="92" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="104" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="91" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="103" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="90" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="102" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -21297,13 +22001,13 @@
     <mergeCell ref="F4:I4"/>
   </mergeCells>
   <conditionalFormatting sqref="G18:G22">
-    <cfRule type="cellIs" dxfId="11" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="23" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="22" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="21" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -21983,13 +22687,13 @@
     <mergeCell ref="B22:H22"/>
   </mergeCells>
   <conditionalFormatting sqref="H27:H34">
-    <cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="20" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="18" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -22341,13 +23045,13 @@
     <mergeCell ref="B6:F6"/>
   </mergeCells>
   <conditionalFormatting sqref="F11:F18">
-    <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="17" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -22768,6 +23472,1728 @@
     <mergeCell ref="F4:I4"/>
   </mergeCells>
   <conditionalFormatting sqref="F20:F26">
+    <cfRule type="cellIs" dxfId="14" priority="1" operator="equal">
+      <formula>"Pass"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="13" priority="2" operator="equal">
+      <formula>"Fail"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="12" priority="3" operator="equal">
+      <formula>"Block"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" sqref="F20:F26" xr:uid="{9AA52BE7-8579-4E4A-AC94-AE3F037312CB}">
+      <formula1>"Pass,Fail,No run,Block"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FFC814A-D9A7-4110-82AF-A5280D96BAD0}">
+  <dimension ref="A1:I25"/>
+  <sheetFormatPr defaultColWidth="7.625" defaultRowHeight="23.25"/>
+  <cols>
+    <col min="1" max="1" width="19.25" style="8" customWidth="1"/>
+    <col min="2" max="3" width="17.5" style="8" customWidth="1"/>
+    <col min="4" max="4" width="40.25" style="8" customWidth="1"/>
+    <col min="5" max="5" width="31.25" style="8" customWidth="1"/>
+    <col min="6" max="6" width="14.875" style="8" customWidth="1"/>
+    <col min="7" max="8" width="12.25" style="8" customWidth="1"/>
+    <col min="9" max="9" width="16.125" style="8" customWidth="1"/>
+    <col min="10" max="16384" width="7.625" style="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="24" thickBot="1">
+      <c r="A1" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+    </row>
+    <row r="2" spans="1:9" ht="24" thickBot="1">
+      <c r="A2" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" s="28" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" s="28"/>
+    </row>
+    <row r="3" spans="1:9" ht="24" thickBot="1">
+      <c r="A3" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="29" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="29"/>
+      <c r="E3" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="29" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" s="29"/>
+      <c r="H3" s="29"/>
+      <c r="I3" s="29"/>
+    </row>
+    <row r="4" spans="1:9" ht="24" thickBot="1">
+      <c r="A4" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="30" t="s">
+        <v>1680</v>
+      </c>
+      <c r="C4" s="30"/>
+      <c r="E4" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="30" t="s">
+        <v>1681</v>
+      </c>
+      <c r="G4" s="30"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="30"/>
+    </row>
+    <row r="5" spans="1:9" ht="24" thickBot="1">
+      <c r="A5" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="30" t="s">
+        <v>1682</v>
+      </c>
+      <c r="C5" s="30"/>
+      <c r="E5" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" s="30" t="s">
+        <v>1683</v>
+      </c>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+    </row>
+    <row r="6" spans="1:9" ht="24" thickBot="1">
+      <c r="A6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="30" t="s">
+        <v>1684</v>
+      </c>
+      <c r="C6" s="30"/>
+      <c r="E6" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="F6" s="30" t="s">
+        <v>1685</v>
+      </c>
+      <c r="G6" s="30"/>
+      <c r="H6" s="30"/>
+      <c r="I6" s="30"/>
+    </row>
+    <row r="7" spans="1:9" ht="24" thickBot="1">
+      <c r="A7" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="30" t="s">
+        <v>1686</v>
+      </c>
+      <c r="C7" s="30"/>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" s="31" t="s">
+        <v>57</v>
+      </c>
+      <c r="B9" s="31"/>
+      <c r="C9" s="31"/>
+      <c r="D9" s="31"/>
+      <c r="E9" s="31"/>
+      <c r="F9" s="31"/>
+      <c r="G9" s="31"/>
+      <c r="H9" s="31"/>
+      <c r="I9" s="31"/>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B11" s="33" t="s">
+        <v>1687</v>
+      </c>
+      <c r="C11" s="33"/>
+      <c r="D11" s="33"/>
+      <c r="E11" s="21"/>
+      <c r="F11" s="21"/>
+      <c r="G11" s="21"/>
+      <c r="H11" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="I11" s="14" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="B12" s="33" t="s">
+        <v>62</v>
+      </c>
+      <c r="C12" s="33"/>
+      <c r="D12" s="33"/>
+      <c r="E12" s="21"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="21"/>
+      <c r="H12" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="I12" s="14" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="46.5">
+      <c r="A13" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B13" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="C13" s="33"/>
+      <c r="D13" s="33"/>
+      <c r="E13" s="21"/>
+      <c r="F13" s="21"/>
+      <c r="G13" s="21"/>
+      <c r="H13" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="I13" s="13" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="46.5">
+      <c r="A14" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="B14" s="33" t="s">
+        <v>1688</v>
+      </c>
+      <c r="C14" s="33"/>
+      <c r="D14" s="33"/>
+      <c r="E14" s="33"/>
+      <c r="F14" s="33"/>
+      <c r="G14" s="33"/>
+      <c r="H14" s="33"/>
+      <c r="I14" s="33"/>
+    </row>
+    <row r="15" spans="1:9" ht="46.5">
+      <c r="A15" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B15" s="33" t="s">
+        <v>1689</v>
+      </c>
+      <c r="C15" s="33"/>
+      <c r="D15" s="33"/>
+      <c r="E15" s="33"/>
+      <c r="F15" s="33"/>
+      <c r="G15" s="33"/>
+      <c r="H15" s="33"/>
+      <c r="I15" s="33"/>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="B17" s="32" t="s">
+        <v>73</v>
+      </c>
+      <c r="C17" s="32"/>
+      <c r="D17" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="E17" s="32" t="s">
+        <v>75</v>
+      </c>
+      <c r="F17" s="32" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" s="32"/>
+      <c r="B18" s="15" t="s">
+        <v>805</v>
+      </c>
+      <c r="C18" s="15" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D18" s="32"/>
+      <c r="E18" s="32"/>
+      <c r="F18" s="32"/>
+    </row>
+    <row r="19" spans="1:6" ht="46.5">
+      <c r="A19" s="16" t="s">
+        <v>1690</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>1691</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>1692</v>
+      </c>
+      <c r="D19" s="13" t="s">
+        <v>1693</v>
+      </c>
+      <c r="E19" s="13" t="s">
+        <v>1826</v>
+      </c>
+      <c r="F19" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="46.5">
+      <c r="A20" s="16" t="s">
+        <v>1694</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>1695</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>1696</v>
+      </c>
+      <c r="D20" s="13" t="s">
+        <v>1697</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>1827</v>
+      </c>
+      <c r="F20" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21" s="16" t="s">
+        <v>1698</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>1699</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="D21" s="13" t="s">
+        <v>1700</v>
+      </c>
+      <c r="E21" s="13" t="s">
+        <v>1828</v>
+      </c>
+      <c r="F21" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="46.5">
+      <c r="A22" s="16" t="s">
+        <v>1701</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>1702</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="D22" s="13" t="s">
+        <v>1703</v>
+      </c>
+      <c r="E22" s="13" t="s">
+        <v>1829</v>
+      </c>
+      <c r="F22" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="46.5">
+      <c r="A23" s="16" t="s">
+        <v>1704</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>1691</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>1705</v>
+      </c>
+      <c r="D23" s="13" t="s">
+        <v>1706</v>
+      </c>
+      <c r="E23" s="13" t="s">
+        <v>201</v>
+      </c>
+      <c r="F23" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="46.5">
+      <c r="A24" s="16" t="s">
+        <v>1707</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>1695</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>1708</v>
+      </c>
+      <c r="D24" s="13" t="s">
+        <v>1709</v>
+      </c>
+      <c r="E24" s="13" t="s">
+        <v>201</v>
+      </c>
+      <c r="F24" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="69.75">
+      <c r="A25" s="16" t="s">
+        <v>1710</v>
+      </c>
+      <c r="B25" s="13" t="s">
+        <v>1711</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="D25" s="13" t="s">
+        <v>1712</v>
+      </c>
+      <c r="E25" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="F25" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="22">
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="D17:D18"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B14:I14"/>
+    <mergeCell ref="B15:I15"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="F5:I5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="F6:I6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="A9:I9"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="F3:I3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="F4:I4"/>
+  </mergeCells>
+  <conditionalFormatting sqref="F19:F25">
+    <cfRule type="cellIs" dxfId="11" priority="1" operator="equal">
+      <formula>"Pass"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="10" priority="2" operator="equal">
+      <formula>"Fail"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="9" priority="3" operator="equal">
+      <formula>"Block"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" sqref="F19:F25" xr:uid="{FDAF44D4-F146-4074-9EFE-1FC8114DE863}">
+      <formula1>"Pass,Fail,No run,Block"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45B130A7-1DE5-43F5-BD16-6323B63E7DA0}">
+  <dimension ref="A1:I28"/>
+  <sheetFormatPr defaultColWidth="7.625" defaultRowHeight="23.25"/>
+  <cols>
+    <col min="1" max="1" width="19.25" style="8" customWidth="1"/>
+    <col min="2" max="4" width="15.75" style="8" customWidth="1"/>
+    <col min="5" max="5" width="36.75" style="8" customWidth="1"/>
+    <col min="6" max="6" width="30.5" style="8" customWidth="1"/>
+    <col min="7" max="7" width="14.875" style="8" customWidth="1"/>
+    <col min="8" max="8" width="12.25" style="8" customWidth="1"/>
+    <col min="9" max="9" width="15.5" style="8" customWidth="1"/>
+    <col min="10" max="16384" width="7.625" style="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="24" thickBot="1">
+      <c r="A1" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+    </row>
+    <row r="2" spans="1:9" ht="24" thickBot="1">
+      <c r="A2" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" s="28" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" s="28"/>
+    </row>
+    <row r="3" spans="1:9" ht="24" thickBot="1">
+      <c r="A3" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="29" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="29"/>
+      <c r="E3" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="29" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" s="29"/>
+      <c r="H3" s="29"/>
+      <c r="I3" s="29"/>
+    </row>
+    <row r="4" spans="1:9" ht="24" thickBot="1">
+      <c r="A4" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="30" t="s">
+        <v>1713</v>
+      </c>
+      <c r="C4" s="30"/>
+      <c r="E4" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="30" t="s">
+        <v>1714</v>
+      </c>
+      <c r="G4" s="30"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="30"/>
+    </row>
+    <row r="5" spans="1:9" ht="24" thickBot="1">
+      <c r="A5" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="30" t="s">
+        <v>1715</v>
+      </c>
+      <c r="C5" s="30"/>
+      <c r="E5" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" s="30" t="s">
+        <v>1716</v>
+      </c>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+    </row>
+    <row r="6" spans="1:9" ht="24" thickBot="1">
+      <c r="A6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="30" t="s">
+        <v>1717</v>
+      </c>
+      <c r="C6" s="30"/>
+      <c r="E6" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="F6" s="30" t="s">
+        <v>1718</v>
+      </c>
+      <c r="G6" s="30"/>
+      <c r="H6" s="30"/>
+      <c r="I6" s="30"/>
+    </row>
+    <row r="7" spans="1:9" ht="24" thickBot="1">
+      <c r="A7" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="30" t="s">
+        <v>1719</v>
+      </c>
+      <c r="C7" s="30"/>
+      <c r="E7" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" s="30" t="s">
+        <v>1720</v>
+      </c>
+      <c r="G7" s="30"/>
+      <c r="H7" s="30"/>
+      <c r="I7" s="30"/>
+    </row>
+    <row r="8" spans="1:9" ht="24" thickBot="1">
+      <c r="E8" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="F8" s="30" t="s">
+        <v>1721</v>
+      </c>
+      <c r="G8" s="30"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="30"/>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" s="31" t="s">
+        <v>57</v>
+      </c>
+      <c r="B10" s="31"/>
+      <c r="C10" s="31"/>
+      <c r="D10" s="31"/>
+      <c r="E10" s="31"/>
+      <c r="F10" s="31"/>
+      <c r="G10" s="31"/>
+      <c r="H10" s="31"/>
+      <c r="I10" s="31"/>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B12" s="33" t="s">
+        <v>1722</v>
+      </c>
+      <c r="C12" s="33"/>
+      <c r="D12" s="33"/>
+      <c r="E12" s="33"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="21"/>
+      <c r="H12" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="I12" s="14" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="B13" s="33" t="s">
+        <v>1723</v>
+      </c>
+      <c r="C13" s="33"/>
+      <c r="D13" s="33"/>
+      <c r="E13" s="33"/>
+      <c r="F13" s="21"/>
+      <c r="G13" s="21"/>
+      <c r="H13" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="I13" s="14" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="46.5">
+      <c r="A14" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B14" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="C14" s="33"/>
+      <c r="D14" s="33"/>
+      <c r="E14" s="33"/>
+      <c r="F14" s="21"/>
+      <c r="G14" s="21"/>
+      <c r="H14" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="I14" s="13" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="46.5">
+      <c r="A15" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="B15" s="33" t="s">
+        <v>1724</v>
+      </c>
+      <c r="C15" s="33"/>
+      <c r="D15" s="33"/>
+      <c r="E15" s="33"/>
+      <c r="F15" s="33"/>
+      <c r="G15" s="33"/>
+      <c r="H15" s="33"/>
+      <c r="I15" s="33"/>
+    </row>
+    <row r="16" spans="1:9" ht="46.5">
+      <c r="A16" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B16" s="33" t="s">
+        <v>1725</v>
+      </c>
+      <c r="C16" s="33"/>
+      <c r="D16" s="33"/>
+      <c r="E16" s="33"/>
+      <c r="F16" s="33"/>
+      <c r="G16" s="33"/>
+      <c r="H16" s="33"/>
+      <c r="I16" s="33"/>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="B18" s="32" t="s">
+        <v>73</v>
+      </c>
+      <c r="C18" s="32"/>
+      <c r="D18" s="32"/>
+      <c r="E18" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="F18" s="32" t="s">
+        <v>75</v>
+      </c>
+      <c r="G18" s="32" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="46.5">
+      <c r="A19" s="32"/>
+      <c r="B19" s="15" t="s">
+        <v>805</v>
+      </c>
+      <c r="C19" s="15" t="s">
+        <v>1726</v>
+      </c>
+      <c r="D19" s="15" t="s">
+        <v>1727</v>
+      </c>
+      <c r="E19" s="32"/>
+      <c r="F19" s="32"/>
+      <c r="G19" s="32"/>
+    </row>
+    <row r="20" spans="1:7" ht="69.75">
+      <c r="A20" s="16" t="s">
+        <v>1728</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>1729</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>1730</v>
+      </c>
+      <c r="D20" s="13" t="s">
+        <v>1731</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>1732</v>
+      </c>
+      <c r="F20" s="13" t="s">
+        <v>1830</v>
+      </c>
+      <c r="G20" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" s="16" t="s">
+        <v>1733</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>1729</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>1734</v>
+      </c>
+      <c r="D21" s="13" t="s">
+        <v>1735</v>
+      </c>
+      <c r="E21" s="13" t="s">
+        <v>1736</v>
+      </c>
+      <c r="F21" s="13" t="s">
+        <v>1218</v>
+      </c>
+      <c r="G21" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" s="16" t="s">
+        <v>1737</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>1729</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>1738</v>
+      </c>
+      <c r="D22" s="13" t="s">
+        <v>1739</v>
+      </c>
+      <c r="E22" s="13" t="s">
+        <v>1740</v>
+      </c>
+      <c r="F22" s="13" t="s">
+        <v>1218</v>
+      </c>
+      <c r="G22" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="46.5">
+      <c r="A23" s="16" t="s">
+        <v>1741</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>1742</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>1743</v>
+      </c>
+      <c r="D23" s="13" t="s">
+        <v>1744</v>
+      </c>
+      <c r="E23" s="13" t="s">
+        <v>1745</v>
+      </c>
+      <c r="F23" s="13" t="s">
+        <v>1218</v>
+      </c>
+      <c r="G23" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="46.5">
+      <c r="A24" s="16" t="s">
+        <v>1746</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>1729</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>1747</v>
+      </c>
+      <c r="D24" s="13" t="s">
+        <v>1748</v>
+      </c>
+      <c r="E24" s="13" t="s">
+        <v>1749</v>
+      </c>
+      <c r="F24" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="G24" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="46.5">
+      <c r="A25" s="16" t="s">
+        <v>1750</v>
+      </c>
+      <c r="B25" s="13" t="s">
+        <v>1729</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>1751</v>
+      </c>
+      <c r="D25" s="13" t="s">
+        <v>1752</v>
+      </c>
+      <c r="E25" s="13" t="s">
+        <v>1753</v>
+      </c>
+      <c r="F25" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="G25" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26" s="16" t="s">
+        <v>1754</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>1729</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>1755</v>
+      </c>
+      <c r="D26" s="13" t="s">
+        <v>1756</v>
+      </c>
+      <c r="E26" s="13" t="s">
+        <v>1757</v>
+      </c>
+      <c r="F26" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="G26" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="46.5">
+      <c r="A27" s="16" t="s">
+        <v>1758</v>
+      </c>
+      <c r="B27" s="13" t="s">
+        <v>1729</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>1743</v>
+      </c>
+      <c r="D27" s="13" t="s">
+        <v>1759</v>
+      </c>
+      <c r="E27" s="13" t="s">
+        <v>1760</v>
+      </c>
+      <c r="F27" s="13" t="s">
+        <v>201</v>
+      </c>
+      <c r="G27" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="46.5">
+      <c r="A28" s="16" t="s">
+        <v>1761</v>
+      </c>
+      <c r="B28" s="13" t="s">
+        <v>1762</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>1763</v>
+      </c>
+      <c r="D28" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="E28" s="13" t="s">
+        <v>1188</v>
+      </c>
+      <c r="F28" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="G28" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="24">
+    <mergeCell ref="B16:I16"/>
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="E18:E19"/>
+    <mergeCell ref="F18:F19"/>
+    <mergeCell ref="G18:G19"/>
+    <mergeCell ref="F8:I8"/>
+    <mergeCell ref="A10:I10"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="B13:E13"/>
+    <mergeCell ref="B14:E14"/>
+    <mergeCell ref="B15:I15"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="F5:I5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="F6:I6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="F7:I7"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="F3:I3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="F4:I4"/>
+  </mergeCells>
+  <conditionalFormatting sqref="G20:G28">
+    <cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
+      <formula>"Pass"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="7" priority="2" operator="equal">
+      <formula>"Fail"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="3" operator="equal">
+      <formula>"Block"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" sqref="G20:G28" xr:uid="{FB6F7310-52BB-4FF8-9EB0-839B9888E94E}">
+      <formula1>"Pass,Fail,No run,Block"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BF7A10B-9A29-47EB-8CB6-AC092355D5D8}">
+  <dimension ref="A1:K20"/>
+  <sheetFormatPr defaultColWidth="7.625" defaultRowHeight="23.25"/>
+  <cols>
+    <col min="1" max="1" width="19.25" style="8" customWidth="1"/>
+    <col min="2" max="3" width="12.25" style="8" customWidth="1"/>
+    <col min="4" max="4" width="40.25" style="8" customWidth="1"/>
+    <col min="5" max="5" width="32" style="8" customWidth="1"/>
+    <col min="6" max="6" width="14.875" style="8" customWidth="1"/>
+    <col min="7" max="8" width="7.625" style="8"/>
+    <col min="9" max="9" width="8.75" style="8" customWidth="1"/>
+    <col min="10" max="11" width="17.5" style="8" customWidth="1"/>
+    <col min="12" max="16384" width="7.625" style="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="46.5">
+      <c r="A1" s="31" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="15" t="s">
+        <v>1764</v>
+      </c>
+      <c r="K1" s="15" t="s">
+        <v>1765</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="I2" s="17" t="s">
+        <v>302</v>
+      </c>
+      <c r="J2" s="17" t="s">
+        <v>308</v>
+      </c>
+      <c r="K2" s="17" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B3" s="33" t="s">
+        <v>1766</v>
+      </c>
+      <c r="C3" s="33"/>
+      <c r="D3" s="33"/>
+      <c r="E3" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="F3" s="14" t="s">
+        <v>154</v>
+      </c>
+      <c r="I3" s="17" t="s">
+        <v>306</v>
+      </c>
+      <c r="J3" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="K3" s="17" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" s="33" t="s">
+        <v>309</v>
+      </c>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="F4" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="I4" s="17" t="s">
+        <v>310</v>
+      </c>
+      <c r="J4" s="17" t="s">
+        <v>714</v>
+      </c>
+      <c r="K4" s="17" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="46.5">
+      <c r="A5" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B5" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" s="33"/>
+      <c r="D5" s="33"/>
+      <c r="E5" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="F5" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="I5" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="J5" s="17" t="s">
+        <v>1767</v>
+      </c>
+      <c r="K5" s="17" t="s">
+        <v>1768</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="46.5">
+      <c r="A6" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="B6" s="33" t="s">
+        <v>1769</v>
+      </c>
+      <c r="C6" s="33"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
+      <c r="F6" s="33"/>
+    </row>
+    <row r="7" spans="1:11" ht="46.5">
+      <c r="A7" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B7" s="33" t="s">
+        <v>1770</v>
+      </c>
+      <c r="C7" s="33"/>
+      <c r="D7" s="33"/>
+      <c r="E7" s="33"/>
+      <c r="F7" s="33"/>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="B9" s="32" t="s">
+        <v>73</v>
+      </c>
+      <c r="C9" s="32"/>
+      <c r="D9" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="E9" s="32" t="s">
+        <v>75</v>
+      </c>
+      <c r="F9" s="32" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
+      <c r="A10" s="32"/>
+      <c r="B10" s="15" t="s">
+        <v>1771</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>1772</v>
+      </c>
+      <c r="D10" s="32"/>
+      <c r="E10" s="32"/>
+      <c r="F10" s="32"/>
+    </row>
+    <row r="11" spans="1:11" ht="46.5">
+      <c r="A11" s="16" t="s">
+        <v>1773</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>947</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>1774</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>1775</v>
+      </c>
+      <c r="E11" s="13" t="s">
+        <v>1831</v>
+      </c>
+      <c r="F11" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="46.5">
+      <c r="A12" s="16" t="s">
+        <v>1776</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>947</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>1777</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>1778</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="F12" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="46.5">
+      <c r="A13" s="16" t="s">
+        <v>1779</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>947</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>1780</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>1495</v>
+      </c>
+      <c r="E13" s="13" t="s">
+        <v>1495</v>
+      </c>
+      <c r="F13" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="46.5">
+      <c r="A14" s="16" t="s">
+        <v>1781</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>947</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>1782</v>
+      </c>
+      <c r="D14" s="13" t="s">
+        <v>1495</v>
+      </c>
+      <c r="E14" s="13" t="s">
+        <v>1495</v>
+      </c>
+      <c r="F14" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="93">
+      <c r="A15" s="16" t="s">
+        <v>1783</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>947</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>1784</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>1785</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="F15" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="93">
+      <c r="A16" s="16" t="s">
+        <v>1786</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>947</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>1787</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>1788</v>
+      </c>
+      <c r="E16" s="13" t="s">
+        <v>1788</v>
+      </c>
+      <c r="F16" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="93">
+      <c r="A17" s="16" t="s">
+        <v>1789</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>947</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>1790</v>
+      </c>
+      <c r="D17" s="13" t="s">
+        <v>1788</v>
+      </c>
+      <c r="E17" s="13" t="s">
+        <v>1788</v>
+      </c>
+      <c r="F17" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="116.25">
+      <c r="A18" s="16" t="s">
+        <v>1791</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>947</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>1792</v>
+      </c>
+      <c r="D18" s="13" t="s">
+        <v>1793</v>
+      </c>
+      <c r="E18" s="13" t="s">
+        <v>1495</v>
+      </c>
+      <c r="F18" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="46.5">
+      <c r="A19" s="16" t="s">
+        <v>1794</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>950</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>1774</v>
+      </c>
+      <c r="D19" s="13" t="s">
+        <v>1795</v>
+      </c>
+      <c r="E19" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="F19" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20" s="16" t="s">
+        <v>1796</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>950</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>1797</v>
+      </c>
+      <c r="D20" s="13" t="s">
+        <v>1798</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>1798</v>
+      </c>
+      <c r="F20" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B6:F6"/>
+  </mergeCells>
+  <conditionalFormatting sqref="F11:F20">
+    <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
+      <formula>"Pass"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
+      <formula>"Fail"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
+      <formula>"Block"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" sqref="F11:F20" xr:uid="{82F4A8E7-F2E1-4FF0-A3A5-771829438754}">
+      <formula1>"Pass,Fail,No run,Block"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27F16D95-552F-4C97-BDF6-E24F68B177A9}">
+  <dimension ref="A1:J18"/>
+  <sheetFormatPr defaultColWidth="7.625" defaultRowHeight="23.25"/>
+  <cols>
+    <col min="1" max="1" width="19.25" style="8" customWidth="1"/>
+    <col min="2" max="3" width="21" style="8" customWidth="1"/>
+    <col min="4" max="4" width="38.5" style="8" customWidth="1"/>
+    <col min="5" max="5" width="31.75" style="8" customWidth="1"/>
+    <col min="6" max="6" width="14.875" style="8" customWidth="1"/>
+    <col min="7" max="8" width="7.625" style="8"/>
+    <col min="9" max="9" width="8.75" style="8" customWidth="1"/>
+    <col min="10" max="10" width="19.25" style="8" customWidth="1"/>
+    <col min="11" max="16384" width="7.625" style="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="46.5">
+      <c r="A1" s="31" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="15" t="s">
+        <v>1799</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="I2" s="17" t="s">
+        <v>302</v>
+      </c>
+      <c r="J2" s="17" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B3" s="33" t="s">
+        <v>1800</v>
+      </c>
+      <c r="C3" s="33"/>
+      <c r="D3" s="33"/>
+      <c r="E3" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="F3" s="14" t="s">
+        <v>154</v>
+      </c>
+      <c r="I3" s="17" t="s">
+        <v>306</v>
+      </c>
+      <c r="J3" s="17" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" s="33" t="s">
+        <v>309</v>
+      </c>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="F4" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="I4" s="17" t="s">
+        <v>310</v>
+      </c>
+      <c r="J4" s="17" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="46.5">
+      <c r="A5" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B5" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" s="33"/>
+      <c r="D5" s="33"/>
+      <c r="E5" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="F5" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="I5" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="J5" s="17" t="s">
+        <v>732</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="46.5">
+      <c r="A6" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="B6" s="33" t="s">
+        <v>1801</v>
+      </c>
+      <c r="C6" s="33"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
+      <c r="F6" s="33"/>
+    </row>
+    <row r="7" spans="1:10" ht="46.5">
+      <c r="A7" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B7" s="33" t="s">
+        <v>1802</v>
+      </c>
+      <c r="C7" s="33"/>
+      <c r="D7" s="33"/>
+      <c r="E7" s="33"/>
+      <c r="F7" s="33"/>
+    </row>
+    <row r="9" spans="1:10">
+      <c r="A9" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="B9" s="32" t="s">
+        <v>73</v>
+      </c>
+      <c r="C9" s="32"/>
+      <c r="D9" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="E9" s="32" t="s">
+        <v>75</v>
+      </c>
+      <c r="F9" s="32" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10">
+      <c r="A10" s="32"/>
+      <c r="B10" s="15" t="s">
+        <v>1803</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>1804</v>
+      </c>
+      <c r="D10" s="32"/>
+      <c r="E10" s="32"/>
+      <c r="F10" s="32"/>
+    </row>
+    <row r="11" spans="1:10" ht="46.5">
+      <c r="A11" s="16" t="s">
+        <v>1805</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>1806</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>947</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>1807</v>
+      </c>
+      <c r="E11" s="13" t="s">
+        <v>1495</v>
+      </c>
+      <c r="F11" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="46.5">
+      <c r="A12" s="16" t="s">
+        <v>1808</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>1809</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>947</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>1810</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="F12" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="46.5">
+      <c r="A13" s="16" t="s">
+        <v>1811</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>1812</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>947</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="E13" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="F13" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="46.5">
+      <c r="A14" s="16" t="s">
+        <v>1813</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>1814</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>947</v>
+      </c>
+      <c r="D14" s="13" t="s">
+        <v>1495</v>
+      </c>
+      <c r="E14" s="13" t="s">
+        <v>1495</v>
+      </c>
+      <c r="F14" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10">
+      <c r="A15" s="16" t="s">
+        <v>1815</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>1816</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>950</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>1817</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>1495</v>
+      </c>
+      <c r="F15" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="46.5">
+      <c r="A16" s="16" t="s">
+        <v>1818</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>1819</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>947</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>1820</v>
+      </c>
+      <c r="E16" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="F16" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="46.5">
+      <c r="A17" s="16" t="s">
+        <v>1821</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>1822</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="D17" s="13" t="s">
+        <v>1823</v>
+      </c>
+      <c r="E17" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="F17" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" s="16" t="s">
+        <v>1824</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>1825</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="D18" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="E18" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="F18" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B6:F6"/>
+  </mergeCells>
+  <conditionalFormatting sqref="F11:F18">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
@@ -22779,7 +25205,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F20:F26" xr:uid="{9AA52BE7-8579-4E4A-AC94-AE3F037312CB}">
+    <dataValidation type="list" allowBlank="1" sqref="F11:F18" xr:uid="{6C6C1C92-A46B-4DF9-AB61-F88208529E4D}">
       <formula1>"Pass,Fail,No run,Block"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -23582,13 +26008,13 @@
     <mergeCell ref="H27:H28"/>
   </mergeCells>
   <conditionalFormatting sqref="H29:H38">
-    <cfRule type="cellIs" dxfId="89" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="101" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="88" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="100" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="87" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="99" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -24117,13 +26543,13 @@
     <mergeCell ref="B6:G6"/>
   </mergeCells>
   <conditionalFormatting sqref="G11:G23">
-    <cfRule type="cellIs" dxfId="86" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="98" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="85" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="97" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="84" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="96" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -24713,13 +27139,13 @@
     <mergeCell ref="H9:H10"/>
   </mergeCells>
   <conditionalFormatting sqref="H11:H23">
-    <cfRule type="cellIs" dxfId="83" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="95" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="82" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="94" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="81" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="93" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -25738,13 +28164,13 @@
     <mergeCell ref="I32:I33"/>
   </mergeCells>
   <conditionalFormatting sqref="I34:I45">
-    <cfRule type="cellIs" dxfId="80" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="92" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="79" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="91" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="78" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="90" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -26037,13 +28463,13 @@
     <mergeCell ref="F9:F10"/>
   </mergeCells>
   <conditionalFormatting sqref="F11:F15">
-    <cfRule type="cellIs" dxfId="77" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="89" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="76" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="88" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="75" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="87" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -26655,13 +29081,13 @@
     <mergeCell ref="G23:G24"/>
   </mergeCells>
   <conditionalFormatting sqref="G25:G32">
-    <cfRule type="cellIs" dxfId="74" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="86" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="73" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="85" priority="2" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="72" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="84" priority="3" operator="equal">
       <formula>"Block"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>